<commit_message>
Flag prices that come from a reseller, not biobalance.tn
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/initial-catalog/produits.xlsx
+++ b/data/initial-catalog/produits.xlsx
@@ -2142,10 +2142,14 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="N27" t="inlineStr"/>
+          <t>prix à confirmer (tarif revendeur)</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>Prix relevé chez un revendeur, absent de biobalance.tn : à confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2402,10 +2406,14 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="N31" t="inlineStr"/>
+          <t>prix à confirmer (tarif revendeur)</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>Prix relevé chez un revendeur, absent de biobalance.tn : à confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">

</xml_diff>

<commit_message>
Catalog reduced to the 39 listed products, without prices; copy of the removed data
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/initial-catalog/produits.xlsx
+++ b/data/initial-catalog/produits.xlsx
@@ -8,7 +8,6 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Produits" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hors liste (site seulement)" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -414,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N40"/>
+  <dimension ref="A1:M40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -425,12 +424,11 @@
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
     <col width="70" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="26" customWidth="1" min="11" max="11"/>
-    <col width="36" customWidth="1" min="12" max="12"/>
-    <col width="26" customWidth="1" min="13" max="13"/>
-    <col width="50" customWidth="1" min="14" max="14"/>
+    <col width="26" customWidth="1" min="9" max="9"/>
+    <col width="36" customWidth="1" min="10" max="10"/>
+    <col width="50" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -476,30 +474,25 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>Prix de vente conseillé (TND)</t>
+          <t>Image</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>Source du prix</t>
+          <t>Source de l’image</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>Image</t>
+          <t>Source des données</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>Source de l’image</t>
+          <t>Statut</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
-        <is>
-          <t>Statut</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
         <is>
           <t>Remarques</t>
         </is>
@@ -538,30 +531,27 @@
           <t>MAGIC TOUCH – PRIMER • FOUNDATION • CONCEALER + VITAMINE C 30 ml TESTÉ DERMATOLOGIQUEMENT Magic Touch est une formule 3-en-1 (base de maquillage, fond de teint et anti-cernes) qui unifie immédiatement le teint, couvre les rougeurs, les taches sombres, les cernes, les ridules et les imperfections de la peau. La texture invisible et légère laisse la peau lisse, douce et uniforme, avec un fini mat et velouté. Avantages : • Couvre toutes les imperfections (cernes, décolorations, ridules, pores, etc.) • En quelques secondes, la peau paraît parfaite et lisse • S’harmonise facilement avec toutes les carnations • Texture invisible, légère comme si elle n’existait pas • Fini mat et velouté pour un teint impeccable • Formule légère avec haute couvrance • Boost de radiance grâce à la vitamine C • Non comédogène – n’obstrue pas les pores Conseil d’utilisation : Après votre routine de soin, appliquer le produit avec les doigts ou une éponge sur le visage et le cou jusqu’à atteindre le niveau de couvrance souhaité.</t>
         </is>
       </c>
-      <c r="I2" t="n">
-        <v>56</v>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>images/8697711601118.jpg</t>
+        </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>biobalance.tn</t>
+          <t>https://biobalance.tn/maquillage/46-customizable-mug.html</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>images/8697711601118.jpg</t>
+          <t>https://biobalance.tn/maquillage/46-customizable-mug.html</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>https://biobalance.tn/maquillage/46-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr"/>
+          <t>complet</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -600,30 +590,27 @@
           <t>HUILE D’ARGAN BIOLOGIQUE – BEURRE DE KARITÉ – PROVITAMINE B5 330 ml TESTÉ DERMATOLOGIQUEMENT Soin réparateur hydratant et protecteur pour cheveux secs, abîmés ou fragilisés Après le shampoing, cet après-shampoing riche et onctueux à base d’huile d’argan biologique nourrit profondément les cheveux, répare les dommages, renforce la cuticule à chaque utilisation et aide à restaurer douceur, élasticité et brillance. Il protège également les cheveux contre la chaleur du coiffage et les agressions environnementales tout en facilitant le démêlage pour une chevelure plus lisse, soyeuse et disciplinée. Avantages : • Hydrate, nourrit et adoucit les cheveux • Répare les cheveux abîmés et les pointes fourchues • Renforce la structure capillaire pour plus de résistance • Protège contre les dommages liés à la chaleur du coiffage • Réduit les frisottis et facilite le démêlage • Laisse les cheveux plus doux, brillants et lisses Conseil d’utilisation : Après le shampoing, appliquer une quantité suffisante d’après-shampoing sur cheveux mouillés, masser doucement puis laisser poser 1 à 2 minutes, puis rincer abondamment. Pour de meilleurs résultats, utiliser régulièrement avec un shampoing Biobalance adapté.</t>
         </is>
       </c>
-      <c r="I3" t="n">
-        <v>42.5</v>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>images/8697711700224.jpg</t>
+        </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>biobalance.tn</t>
+          <t>https://biobalance.tn/soins-capillaires/51-customizable-mug.html</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>images/8697711700224.jpg</t>
+          <t>https://biobalance.tn/soins-capillaires/51-customizable-mug.html</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>https://biobalance.tn/soins-capillaires/51-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr"/>
+          <t>complet</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -658,30 +645,27 @@
           <t>La niacinamide multifonctionnelle (vitamine B3) apporte des solutions efficaces aux problématiques des peaux grasses et sujettes au vieillissement, en agissant simultanément sur l’hydratation, le sébum et les imperfections. Avantages : • Hydrate la peau sans provoquer d’acné • Régule la sécrétion de sébum • Cible les imperfections et les points noirs • Affine le grain de peau et l’apparence des pores Conseil d’utilisation : Appliquer deux fois par jour, matin et soir, sur le visage et le cou.</t>
         </is>
       </c>
-      <c r="I4" t="n">
-        <v>49</v>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>images/8697711602016.jpg</t>
+        </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>biobalance.tn</t>
+          <t>https://biobalance.tn/supercreams-/31-customizable-mug.html</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>images/8697711602016.jpg</t>
+          <t>https://biobalance.tn/supercreams-/31-customizable-mug.html</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>https://biobalance.tn/supercreams-/31-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr"/>
+          <t>complet</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -720,30 +704,27 @@
           <t>Cette crème hydratante combine collagène hydrolysé et acide hyaluronique multi-moléculaire pour offrir une hydratation profonde, repulper la peau, améliorer l’élasticité et atténuer l’apparence des rides et des ridules. Sa texture riche mais rapidement absorbée aide à donner un aspect plus lisse, ferme et revitalisé à la peau. Avantages : • Soutient la production de collagène pour une peau plus ferme • Hydrate intensément en profondeur • Repulpe la peau et réduit les rides et ridules • Améliore l’élasticité et l’apparence générale • Texture riche, veloutée et rapidement absorbée Conseil d’utilisation : Appliquer deux fois par jour, matin et soir, sur le visage et le cou, sur une peau propre.</t>
         </is>
       </c>
-      <c r="I5" t="n">
-        <v>49</v>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>images/8697711602030.jpg</t>
+        </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>biobalance.tn</t>
+          <t>https://biobalance.tn/supercreams-/33-customizable-mug.html</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>images/8697711602030.jpg</t>
+          <t>https://biobalance.tn/supercreams-/33-customizable-mug.html</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>https://biobalance.tn/supercreams-/33-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr"/>
+          <t>complet</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -778,34 +759,27 @@
           <t>Cette crème contour des yeux associe collagène hydrolysé, acide hyaluronique multi-moléculaire et vitamine C pour hydrater intensément, améliorer l’élasticité de la peau et lisser l’apparence des rides et ridules. Elle aide également à illuminer et raffermir le contour des yeux. Avantages : • Améliore la fermeté et l’élasticité de la peau • Hydrate intensément le contour des yeux • Aide à réduire l’apparence des rides et ridules • Illumine et unifie le regard • Texture légère, rapidement absorbée Conseil d’utilisation : Appliquer deux fois par jour, matin et soir, sur le contour des yeux en tapotant délicatement.</t>
         </is>
       </c>
-      <c r="I6" t="n">
-        <v>52</v>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>images/8697711602061.jpg</t>
+        </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>biobalance.tn</t>
+          <t>https://biobalance.tn/supercreams-/32-customizable-mug.html</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>images/8697711602061.jpg</t>
+          <t>https://biobalance.tn/supercreams-/32-customizable-mug.html</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>https://biobalance.tn/supercreams-/32-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>Prix mis à jour depuis le site (49 → 52 TND)</t>
-        </is>
-      </c>
+          <t>complet</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -844,30 +818,27 @@
           <t>Le Dry &amp; Smooth Roll-On de Biobalance protège efficacement contre les odeurs pendant 48h, tout en aidant à réduire l’apparence des poils sous les aisselles. Sa formule douce, sans alcool, convient à tous les types de peau.</t>
         </is>
       </c>
-      <c r="I7" t="n">
-        <v>29</v>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>images/8697711622427.jpg</t>
+        </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>biobalance.tn</t>
+          <t>https://biobalance.tn/soins-personnels/66-customizable-mug.html</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>images/8697711622427.jpg</t>
+          <t>https://biobalance.tn/soins-personnels/66-customizable-mug.html</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>https://biobalance.tn/soins-personnels/66-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr"/>
+          <t>complet</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -910,30 +881,27 @@
           <t>Le Dry &amp; Sport Roll-On pour homme assure une protection efficace contre les odeurs jusqu’à 48h, tout en aidant à éclaircir et uniformiser la peau des aisselles. Sa formule naturelle, sans alcool et sans sels d’aluminium agressifs, respecte la peau sensible et permet de maintenir une sensation de fraîcheur et de confort tout au long de la journée.Adapté aux hommes actifs, il combine efficacité déodorante et soin de la peau.</t>
         </is>
       </c>
-      <c r="I8" t="n">
-        <v>29</v>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>images/8697711622434.jpg</t>
+        </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>biobalance.tn</t>
+          <t>https://biobalance.tn/soins-personnels/68-customizable-mug.html</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>images/8697711622434.jpg</t>
+          <t>https://biobalance.tn/soins-personnels/68-customizable-mug.html</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>https://biobalance.tn/soins-personnels/68-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="N8" t="inlineStr"/>
+          <t>complet</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -976,32 +944,29 @@
           <t>Déodorant roll-on naturel qui offre une protection efficace jusqu’à 48 heures contre les odeurs et l’humidité, tout en respectant le processus naturel de transpiration. Sa formule est enrichie en Alpha-Arbutine, Niacinamide (Vitamine B3) et Vitamine C, des actifs reconnus pour aider à éclaircir et uniformiser la peau des aisselles, en réduisant progressivement les taches foncées. Sans alcool ni sels d’aluminium, il convient aux peaux sensibles et laisse une sensation de fraîcheur et de confort durable.</t>
         </is>
       </c>
-      <c r="I9" t="n">
-        <v>29</v>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>images/8697711622410.jpg</t>
+        </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>biobalance.tn</t>
+          <t>https://biobalance.tn/soins-personnels/67-customizable-mug.html</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>images/8697711622410.jpg</t>
+          <t>https://biobalance.tn/soins-personnels/67-customizable-mug.html</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>https://biobalance.tn/soins-personnels/67-customizable-mug.html</t>
+          <t>complet</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>Prix, photo et description repris du code 8697711740411 (même produit, ancien code probable)</t>
+          <t>Données et photo reprises du code 8697711740411 (même produit, ancien code probable)</t>
         </is>
       </c>
     </row>
@@ -1046,30 +1011,27 @@
           <t>Déodorant roll-on naturel qui offre une protection efficace jusqu’à 48 heures contre les odeurs et l’humidité, tout en respectant le processus naturel de transpiration. Sa formule est enrichie en Alpha-Arbutine, Niacinamide (Vitamine B3) et Vitamine C, des actifs reconnus pour aider à éclaircir et uniformiser la peau des aisselles, en réduisant progressivement les taches foncées. Sans alcool ni sels d’aluminium, il convient aux peaux sensibles et laisse une sensation de fraîcheur et de confort durable.</t>
         </is>
       </c>
-      <c r="I10" t="n">
-        <v>29</v>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>images/8697711740411.jpg</t>
+        </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>biobalance.tn</t>
+          <t>https://biobalance.tn/soins-personnels/67-customizable-mug.html</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>images/8697711740411.jpg</t>
+          <t>https://biobalance.tn/soins-personnels/67-customizable-mug.html</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>https://biobalance.tn/soins-personnels/67-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="N10" t="inlineStr"/>
+          <t>complet</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1112,30 +1074,27 @@
           <t>Un soin quotidien contre les problèmes de peau grasse Effet « Soft Peeling » La formule sans savon et sans huile nettoie en douceur et en profondeur les pores en éliminant saletés, impuretés et maquillage. La mousse légère se rince facilement, sans laisser de résidus pouvant obstruer les pores. Gluconate de Zinc et AHA naturels (Myrtille, canne à sucre, érable à sucre, citron et extrait d’orange) réduisent la production excessive de sébum, la taille des pores, la brillance et les points noirs. Glycérine, Allantoïne, Bétaïne naturelle et Vitamine E Améliorent la barrière naturelle de la peau, préviennent la perte d’hydratation et aident à maintenir une peau bien hydratée. Mode d’emploi Utiliser quotidiennement. Masser délicatement sur le visage et le cou humides, deux fois par jour. Rincer abondamment à l’eau tiède puis sécher en tamponnant avec une serviette douce.</t>
         </is>
       </c>
-      <c r="I11" t="n">
-        <v>38</v>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>images/8697711701009.jpg</t>
+        </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>biobalance.tn</t>
+          <t>https://biobalance.tn/nettoyants-visage/28-customizable-mug.html</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>images/8697711701009.jpg</t>
+          <t>https://biobalance.tn/nettoyants-visage/28-customizable-mug.html</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>https://biobalance.tn/nettoyants-visage/28-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="N11" t="inlineStr"/>
+          <t>complet</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1178,30 +1137,27 @@
           <t>Un soin apaisant qui respecte les peaux sensibles. Effet « Soft Peeling » La formule sans savon et sans huile nettoie la peau en douceur et élimine saletés, impuretés et maquillage.La mousse légère se rince facilement, sans laisser de résidus pouvant obstruer les pores. Avantages : Améliore la fonction naturelle de la barrière cutanée et réduit les rougeurs, les picotements et la sensibilité. INGRÉDIENTS : Bisabolol Complexe d’Acides AminésRenforce la résistance et la tolérance de la peau face aux agressions extérieures irritantes responsables de rougeurs, tiraillements et sensations de picotement.Glycérine, Aloe Vera, Allantoïne, Panthénol et Vitamine E Améliorent la barrière naturelle de la peau, préviennent la perte d’hydratation et aident à maintenir une peau bien hydratée. Mode d’emploi : Utiliser quotidiennement. Masser délicatement sur le visage et le cou humides, deux fois par jour. Rincer abondamment à l’eau tiède puis sécher en tamponnant avec une serviette douce.</t>
         </is>
       </c>
-      <c r="I12" t="n">
-        <v>38</v>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>images/8697711701016.jpg</t>
+        </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>biobalance.tn</t>
+          <t>https://biobalance.tn/nettoyants-visage/23-customizable-mug.html</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>images/8697711701016.jpg</t>
+          <t>https://biobalance.tn/nettoyants-visage/23-customizable-mug.html</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>https://biobalance.tn/nettoyants-visage/23-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="N12" t="inlineStr"/>
+          <t>complet</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1244,30 +1200,27 @@
           <t>Eau micellaire biphasée démaquillante hydratante 500 ml Démaquillant micellaire biphasé spécialement formulé pour les peaux sèches, normales et sensibles. Sa formule à deux phases élimine efficacement le maquillage waterproof, les impuretés et l’excès de sébum, tout en renforçant la barrière cutanée, apportant une hydratation profonde et en calmant les sensations d’inconfort. Enrichie en céramide, vitamine C, camomille et squalane, elle nourrit et apaise la peau sans laisser de résidu gras ni collant. Avantages : • Élimine facilement le maquillage, même waterproof • Renforce la barrière cutanée pour protéger contre la perte d’hydratation • Hydrate profondément et nourrit la peau • Apaise la sensibilité et réduit les rougeurs • Laisse la peau douce, propre et confortable sans sensation grasse ou collante Conseil d’utilisation : Agiter avant utilisation pour mélanger les deux phases. Appliquer sur le visage, les yeux et les lèvres à l’aide d’un coton, sans frotter. Aucun rinçage nécessaire.</t>
         </is>
       </c>
-      <c r="I13" t="n">
-        <v>38</v>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>images/8697711621833.jpg</t>
+        </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>biobalance.tn</t>
+          <t>https://biobalance.tn/nettoyants-visage/34-customizable-mug.html</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>images/8697711621833.jpg</t>
+          <t>https://biobalance.tn/nettoyants-visage/34-customizable-mug.html</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>https://biobalance.tn/nettoyants-visage/34-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="N13" t="inlineStr"/>
+          <t>complet</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1310,30 +1263,27 @@
           <t>Eau micellaire démaquillante hydratante 500 ml Démaquillant micellaire hydratant spécialement formulé pour nettoyer en profondeur tout en apportant une hydratation intense, même aux peaux sèches et sensibles. Grâce à un complexe d’acide hyaluronique, d’acides aminés, de Pentavitin et d’extrait de Centella Asiatica, cette eau micellaire élimine efficacement le maquillage, les impuretés et l’excès de sébum, tout en nourrissant, repulpant et sublimant l’éclat naturel de la peau. Avantages : • Nettoie en profondeur – élimine maquillage, impuretés et excès de sébum • Hydratation intense – l’acide hyaluronique et le Pentavitin boostent l’hydratation • Renforce la barrière cutanée – grâce au complexe d’acides aminés et à la Centella Asiatica • Repulpe et illumine la peau pour une apparence plus lisse et radieuse • Douce pour les yeux – ne pique pas et ne trouble pas la vision Conseil d’utilisation : Appliquer sur le visage, les yeux et les lèvres à l’aide d’un coton. Inutile de rincer.</t>
         </is>
       </c>
-      <c r="I14" t="n">
-        <v>38</v>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>images/8697711621819.jpg</t>
+        </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>biobalance.tn</t>
+          <t>https://biobalance.tn/nettoyants-visage/27-customizable-mug.html</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>images/8697711621819.jpg</t>
+          <t>https://biobalance.tn/nettoyants-visage/27-customizable-mug.html</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>https://biobalance.tn/nettoyants-visage/27-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="N14" t="inlineStr"/>
+          <t>complet</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1376,30 +1326,27 @@
           <t>Eau micellaire démaquillante clarifiante 500 ml Démaquillant micellaire spécialement formulé pour les peaux grasses et mixtes. Sa formule enrichie en niacinamide, extrait de thé vert et extrait de concombre aide à réguler la production de sébum, nettoyer les pores en profondeur et prévenir l’apparition d’acné et de points noirs, tout en éliminant le maquillage, l’excès d’huile et les impuretés sans dessécher la peau. Avantages : • Aide à contrôler l’excès de sébum et la brillance • Nettoie efficacement le maquillage et les impuretés • Aide à réduire l’apparence des pores dilatés • Rafraîchit, apaise et hydrate grâce aux extraits naturels • Préserve l’équilibre naturel de la peau sans dessécher Conseil d’utilisation : Appliquer sur le visage, les yeux et les lèvres à l’aide d’un coton, sans frotter. Aucun rinçage nécessaire.</t>
         </is>
       </c>
-      <c r="I15" t="n">
-        <v>38</v>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>images/8697711621826.jpg</t>
+        </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>biobalance.tn</t>
+          <t>https://biobalance.tn/nettoyants-visage/35-customizable-mug.html</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>images/8697711621826.jpg</t>
+          <t>https://biobalance.tn/nettoyants-visage/35-customizable-mug.html</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>https://biobalance.tn/nettoyants-visage/35-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="N15" t="inlineStr"/>
+          <t>complet</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1438,28 +1385,27 @@
           <t>Sérum pour cils et sourcils aux peptides (Biotinoyl Tripeptide-1), à la biotine et à l’acide hyaluronique. Appliquer une fine ligne à la base des cils ou sur les sourcils, de préférence le soir, pendant au moins 30 jours.</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>images/8697711722011.jpg</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>https://www.barcodelookup.com/8697711722011</t>
+        </is>
+      </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>images/8697711722011.jpg</t>
+          <t>https://www.barcodelookup.com/8697711722011</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>https://www.barcodelookup.com/8697711722011</t>
-        </is>
-      </c>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>à compléter : prix</t>
-        </is>
-      </c>
-      <c r="N16" t="inlineStr">
-        <is>
-          <t>Prix à fixer par BioBalance : absent du site et de la liste</t>
-        </is>
-      </c>
+          <t>complet</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1502,28 +1448,27 @@
           <t>Baume nettoyant visage 3 en 1 à la vitamine C pure, pour peau terne. Sa texture sorbet se transforme en huile soyeuse au contact de la peau : il démaquille, nettoie et illumine. Spatule fournie.</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>images/8697711601514.jpg</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>https://www.barcodelookup.com/8697711601514</t>
+        </is>
+      </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>images/8697711601514.jpg</t>
+          <t>https://www.barcodelookup.com/8697711601514</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>https://www.barcodelookup.com/8697711601514</t>
-        </is>
-      </c>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>à compléter : prix</t>
-        </is>
-      </c>
-      <c r="N17" t="inlineStr">
-        <is>
-          <t>Prix à fixer par BioBalance : absent du site et de la liste</t>
-        </is>
-      </c>
+          <t>complet</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1566,28 +1511,27 @@
           <t>Baume nettoyant visage 3 en 1 à l’acide hyaluronique, pour peau normale à sèche. Sa texture sorbet se transforme en huile soyeuse au contact de la peau : il démaquille, nettoie et hydrate. Spatule fournie.</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>images/8697711601538.jpg</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>https://www.barcodelookup.com/8697711601538</t>
+        </is>
+      </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>images/8697711601538.jpg</t>
+          <t>https://www.barcodelookup.com/8697711601538</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>https://www.barcodelookup.com/8697711601538</t>
-        </is>
-      </c>
-      <c r="M18" t="inlineStr">
-        <is>
-          <t>à compléter : prix</t>
-        </is>
-      </c>
-      <c r="N18" t="inlineStr">
-        <is>
-          <t>Prix à fixer par BioBalance : absent du site et de la liste</t>
-        </is>
-      </c>
+          <t>complet</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1630,28 +1574,27 @@
           <t>Baume nettoyant visage 3 en 1 au squalane et au bisabolol, pour peau sensible ou à rougeurs. Sa texture sorbet se transforme en huile soyeuse au contact de la peau : il démaquille, nettoie et apaise. Spatule fournie.</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>images/8697711601521.jpg</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>https://www.barcodelookup.com/8697711601521</t>
+        </is>
+      </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>images/8697711601521.jpg</t>
+          <t>https://www.barcodelookup.com/8697711601521</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>https://www.barcodelookup.com/8697711601521</t>
-        </is>
-      </c>
-      <c r="M19" t="inlineStr">
-        <is>
-          <t>à compléter : prix</t>
-        </is>
-      </c>
-      <c r="N19" t="inlineStr">
-        <is>
-          <t>Prix à fixer par BioBalance : absent du site et de la liste</t>
-        </is>
-      </c>
+          <t>complet</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1694,28 +1637,27 @@
           <t>Baume nettoyant visage 3 en 1 à l’acide oléanolique, pour peau grasse ou mixte : il contrôle l’excès de sébum et minimise les pores. Sa texture sorbet se transforme en huile soyeuse au contact de la peau. Spatule fournie.</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>images/8697711601545.jpg</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>https://www.barcodelookup.com/8697711601545</t>
+        </is>
+      </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>images/8697711601545.jpg</t>
+          <t>https://www.barcodelookup.com/8697711601545</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>https://www.barcodelookup.com/8697711601545</t>
-        </is>
-      </c>
-      <c r="M20" t="inlineStr">
-        <is>
-          <t>à compléter : prix</t>
-        </is>
-      </c>
-      <c r="N20" t="inlineStr">
-        <is>
-          <t>Prix à fixer par BioBalance : absent du site et de la liste</t>
-        </is>
-      </c>
+          <t>complet</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1754,30 +1696,27 @@
           <t>30 ml Testé dermatologiquement Exfoliation chimique ciblée contre les points noirs et blancs Ce sérum concentré contient 2 % d’acide salicylique, un acide bêta-hydroxy (BHA) reconnu pour ses propriétés lipolytiques (dissolution du sébum), kératolytiques (exfoliation des cellules mortes) et comédolytiques (désincrustation des pores). Grâce à sa capacité à pénétrer profondément dans les pores, il aide à éliminer les cellules mortes et l’excès de sébum, favorisant ainsi une peau plus nette et plus claire, notamment en ciblant les points noirs et points blancs. Avantages : • Élimine les cellules mortes et le sébum à l’intérieur des pores • Réduit visiblement les points noirs et les points blancs • Régule la production excessive de sébum • Améliore la texture et l’apparence globale de la peau • Aide à prévenir l’apparition de nouvelles imperfections Conseil d’utilisation : Utiliser une petite quantité sur une peau propre après le nettoyage, en évitant le contour des yeux. Appliquer matin et soir. Laisser le sérum être absorbé avant d’appliquer votre crème hydratante. Pour optimiser les résultats et protéger la peau, appliquer toujours une protection solaire pendant la journée lorsque vous utilisez ce produit et pendant une semaine après la fin de son utilisation.</t>
         </is>
       </c>
-      <c r="I21" t="n">
-        <v>74</v>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>images/8697711600845.jpg</t>
+        </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>biobalance.tn</t>
+          <t>https://biobalance.tn/serum/40-customizable-mug.html</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>images/8697711600845.jpg</t>
+          <t>https://biobalance.tn/serum/40-customizable-mug.html</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>https://biobalance.tn/serum/40-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="N21" t="inlineStr"/>
+          <t>complet</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1816,30 +1755,27 @@
           <t>AHA 10% + BHA 2% + RED ALGAE 30 ml TESTÉ DERMATOLOGIQUEMENT Peeling visage illuminateur &amp; unifiant le teint Le sérum Deep Peeling exfolie à la fois la surface de la peau et l’intérieur des pores grâce à une combinaison de 10 % d’AHAs (acides alpha-hydroxy : glycolique, lactique, mandélique) et 2 % de BHA (acide salicylique) dans une seule formule. Les AHAs agissent en éliminant les cellules mortes à la surface, tandis que le BHA pénètre profondément pour déboucher les pores et aider à prévenir les points noirs et boutons. Les algues rouges hydratent la peau et aident à accroître sa tolérance au traitement acide, pour un teint plus lisse, net et éclatant. Avantages : • Exfolie les couches externes de la peau pour un teint plus lumineux (AHAs) • Nettoie en profondeur l’intérieur des pores (BHA) • Aide à prévenir la formation de points noirs et de boutons • Redonne de l’éclat et unifie le teint • Hydrate et renforce la résistance de la peau au peeling Conseil d’utilisation : Utiliser uniquement le soir sur une peau propre et sèche, en évitant le contour des yeux. Laisser agir 10 minutes, puis rincer abondamment à l’eau. À appliquer deux fois par semaine, en laissant au moins 3 jours de pause entre chaque usage. Pour des résultats durables, utilisez régulièrement.</t>
         </is>
       </c>
-      <c r="I22" t="n">
-        <v>74</v>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>images/8697711602122.jpg</t>
+        </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>biobalance.tn</t>
+          <t>https://biobalance.tn/serum/42-customizable-mug.html</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>images/8697711602122.jpg</t>
+          <t>https://biobalance.tn/serum/42-customizable-mug.html</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>https://biobalance.tn/serum/42-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="M22" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="N22" t="inlineStr"/>
+          <t>complet</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1878,30 +1814,27 @@
           <t>EXTRAITS D’ALOE VERA BIO &amp; PROVITAMINE B5 330 ml TESTÉ DERMATOLOGIQUEMENT Hydratation intense &amp; soin réparateur pour cheveux secs, cassants et abîmés Ce shampoing à l’aloe vera biologique est spécialement formulé pour hydrater profondément les cheveux et le cuir chevelu, nourrir en douceur, réduire la casse, renforcer la fibre capillaire et apaiser les sensations de sécheresse. Enrichi en provitamine B5, protéines végétales et minéraux bio- fermentés, il aide à restaurer la douceur, la brillance et la résistance des cheveux fragilisés tout en nettoyant sans agresser. Avantages : • Hydrate profondément le cuir chevelu et les cheveux secs • Aide à prévenir la sécheresse, la casse et la fragilité des cheveux • Renforce la fibre capillaire de la racine aux pointes • Scelle l’humidité pour une douceur durable et une brillance naturelle • Aide à réduire les pellicules et apaise le cuir chevelu Conseil d’utilisation : Appliquer sur cheveux mouillés, masser doucement du cuir chevelu jusqu’aux pointes, puis rincer abondamment. Pour de meilleurs résultats, utiliser ensuite avec l’après-shampoing à l’huile d’argan biologique.</t>
         </is>
       </c>
-      <c r="I23" t="n">
-        <v>39.5</v>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>images/8697711700187.jpg</t>
+        </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>biobalance.tn</t>
+          <t>https://biobalance.tn/soins-capillaires/50-customizable-mug.html</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>images/8697711700187.jpg</t>
+          <t>https://biobalance.tn/soins-capillaires/50-customizable-mug.html</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>https://biobalance.tn/soins-capillaires/50-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="M23" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="N23" t="inlineStr"/>
+          <t>complet</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1940,30 +1873,27 @@
           <t>300EXTRAITS D’AGRUMES BIO &amp; COMPLEXE NATUREL MULTI-ACTIF 330 ml TESTÉ DERMATOLOGIQUEMENT Shampoing purifiant pour cuir chevelu gras et cheveux propres plus longtemps Ce shampoing aux extraits d’agrumes biologiques est spécialement formulé pour réguler l’excès de sébum, purifier le cuir chevelu et les cheveux, éliminer les pellicules et apaiser les démangeaisons du cuir chevelu. Grâce à un complexe d’ingrédients naturels, il aide aussi à renforcer les racines, hydrater la fibre capillaire, améliorer l’élasticité, tout en redonnant aux cheveux leur éclat et leur fraîcheur naturelle. Avantages : • Régule l’excès de sébum pour garder les cheveux propres plus longtemps • Purifie le cuir chevelu et les cheveux • Élimine les pellicules et les impuretés • Apaise les démangeaisons du cuir chevelu • Renforce les racines et améliore la résistance des cheveux • Améliore l’éclat, la brillance et la texture générale des cheveux Conseil d’utilisation : Appliquer sur cheveux mouillés, masser doucement jusqu’aux pointes puis rincer abondamment. Pour de meilleurs résultats, utiliser ensuite avec un après-shampoing à l’huile d’argan biologique.</t>
         </is>
       </c>
-      <c r="I24" t="n">
-        <v>39.5</v>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>images/8697711700170.jpg</t>
+        </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>biobalance.tn</t>
+          <t>https://biobalance.tn/soins-capillaires/49-customizable-mug.html</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>images/8697711700170.jpg</t>
+          <t>https://biobalance.tn/soins-capillaires/49-customizable-mug.html</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>https://biobalance.tn/soins-capillaires/49-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="M24" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="N24" t="inlineStr"/>
+          <t>complet</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2002,30 +1932,27 @@
           <t>EXTRAIT DE LAVANDE BIO, NIACINAMIDE &amp; MINÉRAUX BIO-FERMENTÉS 330 ml TESTÉ DERMATOLOGIQUEMENT Shampoing fortifiant pour cheveux longs, forts et en bonne santé Ce shampoing à la lavande biologique est spécialement formulé pour soutenir une croissance capillaire plus longue, plus forte et plus saine. Il nourrit les cheveux de la racine jusqu’aux pointes, aide à réparer les dommages, améliore la brillance et la flexibilité des fibres capillaires, et réduit les pellicules pour une chevelure éclatante de vitalité et de santé. Avantages : • Favorise une croissance capillaire plus longue et plus forte • Nourrit et renforce les cheveux de la racine aux pointes • Répare les dommages et illumine les cheveux ternes • Améliore la souplesse, la force et la brillance des cheveux • Aide à éliminer les pellicules et purifie le cuir chevelu Conseil d’utilisation : Appliquer sur cheveux mouillés, masser doucement jusqu’aux pointes et rincer abondamment. Pour de meilleurs résultats, utiliser ensuite avec le conditioner à l’huile d’argan biologique Bio Balance.</t>
         </is>
       </c>
-      <c r="I25" t="n">
-        <v>39.5</v>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>images/8697711700156.jpg</t>
+        </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>biobalance.tn</t>
+          <t>https://biobalance.tn/soins-capillaires/48-customizable-mug.html</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>images/8697711700156.jpg</t>
+          <t>https://biobalance.tn/soins-capillaires/48-customizable-mug.html</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>https://biobalance.tn/soins-capillaires/48-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="M25" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="N25" t="inlineStr"/>
+          <t>complet</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2064,30 +1991,27 @@
           <t>EXTRAIT DE GRENADE BIO &amp; KÉRATINE VÉGÉTALE 330 ml TESTÉ DERMATOLOGIQUEMENT Soin protecteur pour cheveux colorés, abîmés &amp; fragilisés Ce shampoing à la grenade bio est spécialement formulé pour protéger, réparer et renforcer les cheveux fragilisés, abîmés ou colorés. Sa formule riche en antioxydants aide à préserver la couleur, sceller la brillance et détoxifier le cuir chevelu, tout en renforçant la fibre capillaire contre les agressions du soleil, de la chaleur, des produits chimiques et du coiffage quotidien. Avantages : • Protège et prolonge l’éclat de la couleur des cheveux • Renforce les cheveux fragilisés et abîmés • Répare la fibre capillaire et améliore la résistance • Aide à éliminer les pellicules et purifie le cuir chevelu • Laisse les cheveux plus lisses, brillants et faciles à coiffer Conseil d’utilisation : Appliquer sur cheveux mouillés, masser doucement jusqu’aux pointes et rincer abondamment. Pour de meilleurs résultats, utiliser ensuite avec le conditioner à l’huile d’argan biologique Bio Balance.</t>
         </is>
       </c>
-      <c r="I26" t="n">
-        <v>39.5</v>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>images/8697711700163.jpg</t>
+        </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>biobalance.tn</t>
+          <t>https://biobalance.tn/soins-capillaires/47-customizable-mug.html</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>images/8697711700163.jpg</t>
+          <t>https://biobalance.tn/soins-capillaires/47-customizable-mug.html</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>https://biobalance.tn/soins-capillaires/47-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="M26" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="N26" t="inlineStr"/>
+          <t>complet</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2122,34 +2046,27 @@
           <t>Ce sérum à 4,5 % de collagène marin et à 0,5 % de vitamine C agit pour uniformiser le teint et la texture de la peau, augmenter l'élasticité pour une peau plus ferme, laisse le teint doux, lisse et éclatant.</t>
         </is>
       </c>
-      <c r="I27" t="n">
-        <v>63.7</v>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>images/8697711600838.jpg</t>
+        </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>MaPara Tunisie (tarif revendeur de démonstration)</t>
+          <t>https://www.maparatunisie.tn/produit/biobalance-serum-collagene-marin-vitamine-c-30ml/</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>images/8697711600838.jpg</t>
+          <t>https://www.maparatunisie.tn/produit/biobalance-serum-collagene-marin-vitamine-c-30ml/</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>https://www.maparatunisie.tn/produit/biobalance-serum-collagene-marin-vitamine-c-30ml/</t>
-        </is>
-      </c>
-      <c r="M27" t="inlineStr">
-        <is>
-          <t>prix à confirmer (tarif revendeur)</t>
-        </is>
-      </c>
-      <c r="N27" t="inlineStr">
-        <is>
-          <t>Prix relevé chez un revendeur, absent de biobalance.tn : à confirmer</t>
-        </is>
-      </c>
+          <t>complet</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2192,30 +2109,27 @@
           <t>Sérum super-éclat anti-taches 30 ml Testé dermatologiquement Sérum avancé conçu pour réduire visiblement l’hyperpigmentation et unifier le teint. Ce traitement ciblé à base de Lumiskin® 4 %, une molécule performante, agit en régulant la production de mélanine pour aider à atténuer les taches brunes, les marques d’acné et les zones de pigmentation irrégulière, tout en restaurer l’éclat naturel et la clarté de la peau. Avantages : • Réduit la quantité de mélanine jusqu’à –70 % • Diminue visiblement l’apparence des taches brunes et empêche leur réapparition • Éclaircit et unifie le teint • Améliore l’éclat et la luminosité de la peau • Convient à tous les types de peau, même sensibles Conseil d’utilisation : Appliquer directement sur une peau propre, matin et soir. Laisser le sérum être absorbé avant d’appliquer votre crème hydratante ou soin quotidien. Il est recommandé d’utiliser une protection solaire haute (SPF 50+) pendant la journée pour optimiser les résultats et aider à prévenir la formation de nouvelles tâches pigmentaires.</t>
         </is>
       </c>
-      <c r="I28" t="n">
-        <v>74</v>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>images/8697711600814.jpg</t>
+        </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>biobalance.tn</t>
+          <t>https://biobalance.tn/serum/36-customizable-mug.html</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>images/8697711600814.jpg</t>
+          <t>https://biobalance.tn/serum/36-customizable-mug.html</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>https://biobalance.tn/serum/36-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="M28" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="N28" t="inlineStr"/>
+          <t>complet</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2258,30 +2172,27 @@
           <t>30 ml Testé dermatologiquement Ce sérum avancé est formulé avec un complexe d’acide hyaluronique multimoléculaire à 1 %, combinant des acides hyaluroniques de faible, moyen et haut poids moléculaire pour une hydratation multi-niveaux qui pénètre toutes les couches de la peau. Cette approche renforce l’hydratation, repulpe la peau et aide à améliorer son apparence générale en ciblant la sécheresse, les ridules et la perte d’élasticité. Avantages : • Hydrate intensément à plusieurs niveaux — de la surface aux couches profondes de la peau • Aide à réduire visiblement l’apparence des ridules et des rides • Améliore la texture, l’élasticité et la fermeté de la peau • Laisse la peau plus souple, rebondie et rafraîchie • Convient à tous les types de peau, y compris sensibles Conseil d’utilisation : Appliquer directement sur le visage propre, matin et soir. Laisser le sérum être absorbé avant d’appliquer votre crème hydratante ou soin quotidien.</t>
         </is>
       </c>
-      <c r="I29" t="n">
-        <v>74</v>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>images/8697711600777.jpg</t>
+        </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>biobalance.tn</t>
+          <t>https://biobalance.tn/serum/38-customizable-mug.html</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>images/8697711600777.jpg</t>
+          <t>https://biobalance.tn/serum/38-customizable-mug.html</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>https://biobalance.tn/serum/38-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="M29" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="N29" t="inlineStr"/>
+          <t>complet</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2324,30 +2235,27 @@
           <t>30 ml Testé dermatologiquement Anti-taches, Anti-rides &amp; Éclaircissant Ce sérum révolutionnaire combine 15 % de niacinamide (vitamine B3) et 5 % d’acide glycolique dans une seule formule pour offrir une solution complète aux problèmes de vieillissement cutané, d’excès de sébum et d’imperfections. Avantages : • Réduit l’apparence des taches brunes et de l’hyperpigmentation • Diminue l’apparence des rides et des ridules • Régule la sécrétion de sébum pour une peau plus équilibrée • Cible les imperfections, les points noirs et les éruptions • Effet exfoliant doux : affine la texture de la peau et resserre l’apparence des pores • Aide à révéler une peau plus claire, lisse et lumineuse Conseil d’utilisation : Utiliser une seule fois par jour, le soir seulement, sur une peau propre. Ne pas rincer. Laisser le sérum être absorbé par la peau avant d’appliquer votre crème hydratante. Si vous avez la peau sensible, utilisez-le 2 à 3 fois par semaine.</t>
         </is>
       </c>
-      <c r="I30" t="n">
-        <v>74</v>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>images/8697711600876.jpg</t>
+        </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>biobalance.tn</t>
+          <t>https://biobalance.tn/serum/39-customizable-mug.html</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>images/8697711600876.jpg</t>
+          <t>https://biobalance.tn/serum/39-customizable-mug.html</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>https://biobalance.tn/serum/39-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="M30" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="N30" t="inlineStr"/>
+          <t>complet</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2386,34 +2294,27 @@
           <t>Répare, renouvelle, protège et détoxifie la peau en stimulant le processus de récupération nocturne de la peau.</t>
         </is>
       </c>
-      <c r="I31" t="n">
-        <v>65.8</v>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>images/8697711602115.jpg</t>
+        </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>MaPara Tunisie (tarif revendeur de démonstration)</t>
+          <t>https://www.maparatunisie.tn/produit/biobalance-super-serum-advanced-night-recovery-30ml/</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>images/8697711602115.jpg</t>
+          <t>https://www.maparatunisie.tn/produit/biobalance-super-serum-advanced-night-recovery-30ml/</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>https://www.maparatunisie.tn/produit/biobalance-super-serum-advanced-night-recovery-30ml/</t>
-        </is>
-      </c>
-      <c r="M31" t="inlineStr">
-        <is>
-          <t>prix à confirmer (tarif revendeur)</t>
-        </is>
-      </c>
-      <c r="N31" t="inlineStr">
-        <is>
-          <t>Prix relevé chez un revendeur, absent de biobalance.tn : à confirmer</t>
-        </is>
-      </c>
+          <t>complet</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2456,28 +2357,27 @@
           <t>Super sérum contour des yeux au phyto-rétinol (bakuchiol), aux céramides et à l’acide hyaluronique, anti-rides et réparateur intense. Appliquer une petite quantité sur peau propre et sèche, autour des yeux, par mouvements circulaires.</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr"/>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>images/8697711602139.jpg</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>https://www.barcodelookup.com/8697711602139</t>
+        </is>
+      </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>images/8697711602139.jpg</t>
+          <t>https://www.barcodelookup.com/8697711602139</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>https://www.barcodelookup.com/8697711602139</t>
-        </is>
-      </c>
-      <c r="M32" t="inlineStr">
-        <is>
-          <t>à compléter : prix</t>
-        </is>
-      </c>
-      <c r="N32" t="inlineStr">
-        <is>
-          <t>Prix à fixer par BioBalance : absent du site et de la liste</t>
-        </is>
-      </c>
+          <t>complet</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2520,30 +2420,27 @@
           <t>30 ml Testé dermatologiquement Sérum concentré à base de 10 % d’acide L-ascorbique (vitamine C pure) formulé sans eau pour une stabilité maximale et une efficacité renforcée. Cette forme stabilisée de vitamine C est un antioxydant puissant qui aide à protéger la peau contre les radicaux libres, stimuler la synthèse du collagène et améliorer l’éclat du teint, tout en contribuant à réduire l’apparence des taches pigmentaires, des rides et des ridules. Avantages : • Protège la peau des dommages causés par les radicaux libres grâce à son action antioxydante • Stimule la synthèse du collagène pour une peau visiblement plus ferme et rebondie • Améliore la clarté du teint et réduit l’apparence des rides • Aide à atténuer les taches brunes et les irrégularités du teint • Formule sans eau, stable et adaptée à tous les types de peau Conseil d’utilisation : Appliquer directement sur le visage propre, matin et soir. Laisser le sérum être absorbé avant d’appliquer votre soin hydratant. Pour de meilleurs résultats, utiliser une protection solaire le matin.</t>
         </is>
       </c>
-      <c r="I33" t="n">
-        <v>74</v>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>images/8697711600760.jpg</t>
+        </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>biobalance.tn</t>
+          <t>https://biobalance.tn/serum/37-customizable-mug.html</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>images/8697711600760.jpg</t>
+          <t>https://biobalance.tn/serum/37-customizable-mug.html</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>https://biobalance.tn/serum/37-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="M33" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="N33" t="inlineStr"/>
+          <t>complet</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2586,30 +2483,27 @@
           <t>30 ml Testé dermatologiquement Ce sérum avancé associe 0,3 % de rétinol pur et 2 % de vitamine E pour améliorer visiblement la qualité de la peau. Sa formule aide à lisser la surface cutanée, favoriser le renouvellement de la peau et améliorer l’uniformité du teint, tout en apportant nutrition et protection grâce à la vitamine E. Cette combinaison agit efficacement sur les signes de l’âge, la texture irrégulière et le manque d’éclat. Avantages : • Aide à réduire visiblement l’apparence des rides et ridules • Améliore la texture et la fermeté de la peau • Favorise un teint plus uniforme et lumineux • Aide à soutenir le renouvellement cutané • Contribue à nourrir et protéger la peau grâce à la vitamine E • Convient à la plupart des types de peau Conseil d’utilisation : Appliquer le soir sur une peau propre et sèche. Laisser le sérum être absorbé avant d’appliquer votre crème hydratante. Utiliser une protection solaire durant la journée. Commencer par 2 à 3 applications par semaine, puis augmenter progressivement selon la tolérance de la peau.</t>
         </is>
       </c>
-      <c r="I34" t="n">
-        <v>74</v>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>images/8697711600852.jpg</t>
+        </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>biobalance.tn</t>
+          <t>https://biobalance.tn/serum/64-customizable-mug.html</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>images/8697711600852.jpg</t>
+          <t>https://biobalance.tn/serum/64-customizable-mug.html</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>https://biobalance.tn/serum/64-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="M34" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="N34" t="inlineStr"/>
+          <t>complet</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2652,30 +2546,27 @@
           <t>30 ml Testé dermatologiquement Anti-cernes, Anti-poches &amp; Fermeté du contour de l’œil Ce sérum yeux léger est formulé avec 5 % de caféine, EGCG dérivé du thé vert et acide hyaluronique pour revitaliser et éclaircir le contour délicat des yeux. Il aide à réduire l’apparence des cernes, atténuer les poches, hydrater intensément et améliorer l’élasticité de la peau autour du regard. Avantages : • Éclaircit visiblement le contour des yeux • Hydrate intensément et repulpe la peau • Contribue à raffermir la zone fragile du regard • Réduit l’apparence des poches et signes de fatigue • Améliore l’élasticité et l’apparence générale de la peau autour des yeux Conseil d’utilisation : Appliquer matin et soir sur le contour des yeux propre et sec en mouvements circulaires doux. Laisser le sérum être absorbé avant d’appliquer votre soin hydratant.</t>
         </is>
       </c>
-      <c r="I35" t="n">
-        <v>74</v>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>images/8697711600890.jpg</t>
+        </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>biobalance.tn</t>
+          <t>https://biobalance.tn/serum/41-customizable-mug.html</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>images/8697711600890.jpg</t>
+          <t>https://biobalance.tn/serum/41-customizable-mug.html</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>https://biobalance.tn/serum/41-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="M35" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="N35" t="inlineStr"/>
+          <t>complet</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2710,30 +2601,27 @@
           <t>Enrichie en vitamine C stabilisée (3-O-Ethyl Ascorbic Acid) et en acide férulique, cette gel-crème illumine le teint, unifie la peau et aide à lutter contre les signes visibles du vieillissement, tout en protégeant la peau des agressions extérieures. Avantages : • Illumine et ravive l’éclat du teint • Aide à atténuer l’apparence des taches pigmentaires • Unifie le teint et améliore la luminosité • Protège la peau grâce à une action antioxydante • Texture légère, rapidement absorbée Conseil d’utilisation : Appliquer deux fois par jour, matin et soir, sur le visage et le cou, sur une peau propre.</t>
         </is>
       </c>
-      <c r="I36" t="n">
-        <v>49</v>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>images/8697711602023.jpg</t>
+        </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>biobalance.tn</t>
+          <t>https://biobalance.tn/supercreams-/29-customizable-mug.html</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>images/8697711602023.jpg</t>
+          <t>https://biobalance.tn/supercreams-/29-customizable-mug.html</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>https://biobalance.tn/supercreams-/29-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="M36" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="N36" t="inlineStr"/>
+          <t>complet</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2768,30 +2656,27 @@
           <t>Testé dermatologiquement Cette crème hydratante avancée est formulée avec Céramide NP et Vitamine F, une combinaison essentielle qui aide à renforcer la barrière naturelle d’hydratation de la peau et à prévenir la perte d’eau. Sa texture légère pénètre rapidement pour offrir une hydratation profonde, apaiser la peau et améliorer son équilibre naturel. Avantages : • Hydrate intensément et durablement la peau • Renforce la barrière cutanée et limite la déshydratation • Apaise et améliore l’élasticité de la peau • Laisse la peau douce, lisse et équilibrée • Idéale pour les peaux sèches, très sèches et sensibles Conseil d’utilisation : Appliquer sur le visage propre, matin et soir. Masser doucement jusqu’à absorption complète avant d’appliquer votre routine quotidienne..</t>
         </is>
       </c>
-      <c r="I37" t="n">
-        <v>49</v>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>images/8697711602054.jpg</t>
+        </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>biobalance.tn</t>
+          <t>https://biobalance.tn/supercreams-/65-customizable-mug.html</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>images/8697711602054.jpg</t>
+          <t>https://biobalance.tn/supercreams-/65-customizable-mug.html</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>https://biobalance.tn/supercreams-/65-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="M37" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="N37" t="inlineStr"/>
+          <t>complet</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2826,30 +2711,27 @@
           <t>Le Phyto-Retinol (Bakuchiol) associé à la L-Carnosine agit de manière multifonctionnelle pour cibler les signes visibles du vieillissement cutané, améliorer la fermeté de la peau et renforcer sa structure. Avantages : • Raffermit la peau et améliore l’élasticité • Réduit l’apparence des rides et ridules • Stimule la production de collagène • Protège contre le vieillissement induit par la lumière bleue • Aide à uniformiser le teint et à atténuer les taches pigmentaires Conseil d’utilisation : Appliquer deux fois par jour, matin et soir, sur le visage et le cou.</t>
         </is>
       </c>
-      <c r="I38" t="n">
-        <v>49</v>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>images/8697711602047.jpg</t>
+        </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>biobalance.tn</t>
+          <t>https://biobalance.tn/super-lift/30-customizable-mug.html</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>images/8697711602047.jpg</t>
+          <t>https://biobalance.tn/super-lift/30-customizable-mug.html</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>https://biobalance.tn/super-lift/30-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="M38" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="N38" t="inlineStr"/>
+          <t>complet</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2888,30 +2770,27 @@
           <t>ETHYL ASCORBIC ACID – EXTRAit DE RACINE DE RÉGLISSE – ACIDE HYALURONIQUE 96 % d’origine naturelle 250 ml TESTÉ DERMATOLOGIQUEMENT Éclaircissant parfait – Anti-taches – Anti-rides Les lotions toniques éliminent visiblement les dernières traces de maquillage, laissant la peau exceptionnellement propre, fraîche et adoucie. Avantages : • Lisse, adoucit et revitalise instantanément la peau • llumine et restaure l’éclat pour un teint radieux • Hydrate et équilibre la peau Conseil d’utilisation : Appliquer à l’aide d’un coton après avoir nettoyé la peau. Essuyer avec des mouvements du centre du visage vers l’extérieur jusqu’à ce que le coton soit propre.</t>
         </is>
       </c>
-      <c r="I39" t="n">
-        <v>39</v>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>images/8697711602313.jpg</t>
+        </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>biobalance.tn</t>
+          <t>https://biobalance.tn/nettoyants-visage/43-customizable-mug.html</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>images/8697711602313.jpg</t>
+          <t>https://biobalance.tn/nettoyants-visage/43-customizable-mug.html</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>https://biobalance.tn/nettoyants-visage/43-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="M39" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="N39" t="inlineStr"/>
+          <t>complet</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2954,371 +2833,27 @@
           <t>LACTIC ACID 7% – AHA + BHA + PHA – TEA TREE OIL 88 % d’origine naturelle 250 ml TESTÉ DERMATOLOGIQUEMENT Anti-acné, Anti-points noirs – Uniformise le teint – Minimise les pores Ce tonique à action multiple est formulé pour cibler les imperfections, les points noirs, les pores dilatés et le teint irrégulier en une seule étape. Enrichi en acide lactique (7 %), un AHA doux mais efficace, et combiné à un complexe d’exfoliation AHA + BHA + PHA, il aide à éliminer les cellules mortes, nettoyer les pores en profondeur et stimuler le renouvellement cellulaire. L’huile d’arbre à thé purifiante contribue à réduire l’excès de sébum et à calmer les zones sujettes aux imperfections, laissant la peau propre, rafraîchie et lisse. Avantages : • Élimine les dernières traces de maquillage et l’excès de sébum • Exfolie en douceur la peau pour un teint plus net • Aide à prévenir les points noirs et boutons • Minimise visiblement l’apparence des pores dilatés • Laisse la peau rafraîchie, plus lisse et équilibrée Conseil d’utilisation : Appliquer le soir à l’aide d’un coton après avoir nettoyé la peau. Essuyer délicatement le visage du centre vers l’extérieur jusqu’à ce que le coton soit propre. Ne pas rincer.</t>
         </is>
       </c>
-      <c r="I40" t="n">
-        <v>39</v>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>images/8697711602337.jpg</t>
+        </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>biobalance.tn</t>
+          <t>https://biobalance.tn/nettoyants-visage/44-customizable-mug.html</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>images/8697711602337.jpg</t>
+          <t>https://biobalance.tn/nettoyants-visage/44-customizable-mug.html</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>https://biobalance.tn/nettoyants-visage/44-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="M40" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="N40" t="inlineStr"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Référence</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Nom</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Prix (TND)</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Page</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Remarque</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>BB-WEB-52</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Repulpeur de lèvres - N°03 Lipojen - Hot Chocolate</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>44.5</v>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>https://biobalance.tn/maquillage/52-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Sur le site, pas dans votre liste, sans code-barres</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>BB-WEB-54</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Repulpeur Lèvres Rose Venus N°04</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>44.5</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>https://biobalance.tn/maquillage/54-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Sur le site, pas dans votre liste, sans code-barres</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>BB-WEB-55</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Repulpeur Lèvres Rosy Petal N°05</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>44.5</v>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>https://biobalance.tn/maquillage/55-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Sur le site, pas dans votre liste, sans code-barres</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>BB-WEB-56</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Repulpeur Lèvres High Society N°07</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>44.5</v>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>https://biobalance.tn/maquillage/56-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Sur le site, pas dans votre liste, sans code-barres</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>BB-WEB-57</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Repulpeur Lèvres Hot Red N°10</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>44.5</v>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>https://biobalance.tn/maquillage/57-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Sur le site, pas dans votre liste, sans code-barres</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>BB-WEB-58</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Repulpeur Lèvres Flamingo Love N°31</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>44.5</v>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>https://biobalance.tn/maquillage/58-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Sur le site, pas dans votre liste, sans code-barres</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>BB-WEB-59</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Repulpeur Lévres Coral Dream N°32</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>44.5</v>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>https://biobalance.tn/maquillage/59-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Sur le site, pas dans votre liste, sans code-barres</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>BB-WEB-60</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Repulpeur Lèvres Fuchia Vibes N°34</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>44.5</v>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>https://biobalance.tn/maquillage/60-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Sur le site, pas dans votre liste, sans code-barres</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>BB-WEB-61</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Repulpeur Lèvres Candy Crush N°35</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>44.5</v>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>https://biobalance.tn/maquillage/61-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Sur le site, pas dans votre liste, sans code-barres</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>BB-WEB-62</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Repulpeur Lèvres Cinnamon Roll N°37</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
-        <v>44.5</v>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>https://biobalance.tn/maquillage/62-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>Sur le site, pas dans votre liste, sans code-barres</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>BB-WEB-63</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>ACNEVIT ANTI-ACNE CLEANSING GEL</t>
-        </is>
-      </c>
-      <c r="C12" t="n">
-        <v>41</v>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>https://biobalance.tn/nettoyants-visage/63-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Sur le site, pas dans votre liste, sans code-barres</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>BB-WEB-53</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>ACNEVIT ANTI-ACNE SERUM</t>
-        </is>
-      </c>
-      <c r="C13" t="n">
-        <v>67</v>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>https://biobalance.tn/serum/53-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>Sur le site, pas dans votre liste, sans code-barres</t>
-        </is>
-      </c>
+          <t>complet</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Clean and complete product data: official ingredients, usage, sizes, claims; applied to production
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/initial-catalog/produits.xlsx
+++ b/data/initial-catalog/produits.xlsx
@@ -413,22 +413,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M40"/>
+  <dimension ref="A1:O40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="44" customWidth="1" min="3" max="3"/>
-    <col width="48" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
     <col width="70" customWidth="1" min="8" max="8"/>
-    <col width="26" customWidth="1" min="9" max="9"/>
-    <col width="36" customWidth="1" min="10" max="10"/>
-    <col width="50" customWidth="1" min="11" max="11"/>
-    <col width="22" customWidth="1" min="12" max="12"/>
-    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="60" customWidth="1" min="9" max="9"/>
+    <col width="60" customWidth="1" min="10" max="10"/>
+    <col width="40" customWidth="1" min="11" max="11"/>
+    <col width="26" customWidth="1" min="12" max="12"/>
+    <col width="36" customWidth="1" min="13" max="13"/>
+    <col width="60" customWidth="1" min="14" max="14"/>
+    <col width="24" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -449,7 +451,7 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Nom affiché</t>
+          <t>Nom</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
@@ -474,27 +476,37 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
+          <t>Conseils d’utilisation</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Ingrédients</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Précautions</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
           <t>Image</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Source de l’image</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>Source des données</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>Statut</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>Remarques</t>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Sources</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>Champs manquants</t>
         </is>
       </c>
     </row>
@@ -516,42 +528,65 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>MAGIC TOUCH</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr"/>
+          <t>Magic Touch</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Magic Touch</t>
+        </is>
+      </c>
       <c r="F2" t="inlineStr">
         <is>
           <t>Maquillage</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>30 ml</t>
+        </is>
+      </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>MAGIC TOUCH – PRIMER • FOUNDATION • CONCEALER + VITAMINE C 30 ml TESTÉ DERMATOLOGIQUEMENT Magic Touch est une formule 3-en-1 (base de maquillage, fond de teint et anti-cernes) qui unifie immédiatement le teint, couvre les rougeurs, les taches sombres, les cernes, les ridules et les imperfections de la peau. La texture invisible et légère laisse la peau lisse, douce et uniforme, avec un fini mat et velouté. Avantages : • Couvre toutes les imperfections (cernes, décolorations, ridules, pores, etc.) • En quelques secondes, la peau paraît parfaite et lisse • S’harmonise facilement avec toutes les carnations • Texture invisible, légère comme si elle n’existait pas • Fini mat et velouté pour un teint impeccable • Formule légère avec haute couvrance • Boost de radiance grâce à la vitamine C • Non comédogène – n’obstrue pas les pores Conseil d’utilisation : Après votre routine de soin, appliquer le produit avec les doigts ou une éponge sur le visage et le cou jusqu’à atteindre le niveau de couvrance souhaité.</t>
+          <t>Magic touch – primer • foundation • concealer + vitamine C. Magic Touch est une formule 3-en-1 (base de maquillage, fond de teint et anti-cernes) qui unifie immédiatement le teint, couvre les rougeurs, les taches sombres, les cernes, les ridules et les imperfections de la peau. La texture invisible et légère laisse la peau lisse, douce et uniforme, avec un fini mat et velouté.
+Avantages :
+• Couvre toutes les imperfections (cernes, décolorations, ridules, pores, etc.)
+• En quelques secondes, la peau paraît parfaite et lisse
+• S’harmonise facilement avec toutes les carnations
+• Texture invisible, légère comme si elle n’existait pas
+• Fini mat et velouté pour un teint impeccable
+• Formule légère avec haute couvrance
+• Boost de radiance grâce à la vitamine C
+• Non comédogène – n’obstrue pas les pores</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
+          <t>Après votre routine de soin, appliquer le produit avec les doigts ou une éponge sur le visage et le cou jusqu’à atteindre le niveau de couvrance souhaité.</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>DIMETHICONE, DIMETHICONE CROSSPOLYMER, HYDROGENATED POLYISOBUTENE, HYDROGENATED POLYDECENE, ISONONYL ISONONANOATE, ISOPROPYL MYRISTATE, DICAPRYLYL CARBONATE, ASCORBYL TETRAISOPALMITATE, ISOPROPYL TITANIUM TRIISOSTEARATE, STEARALKONIUM HECTORITE, PROPYLENE CARBONATE, POLYHYDROXYSTEARIC ACID, TOCOPHEROL, CI 77891</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr">
+        <is>
           <t>images/8697711601118.jpg</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>https://biobalance.tn/maquillage/46-customizable-mug.html</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>https://biobalance.tn/maquillage/46-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>https://biobalance.tn/maquillage/46-customizable-mug.html | https://www.barcodelookup.com/8697711601118</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -571,10 +606,14 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>ORGANIC ARGAN OIL CONDITIONER</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr"/>
+          <t>Organic Argan Oil Conditioner</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Organic</t>
+        </is>
+      </c>
       <c r="F3" t="inlineStr">
         <is>
           <t>Soins capillaires</t>
@@ -587,30 +626,44 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>HUILE D’ARGAN BIOLOGIQUE – BEURRE DE KARITÉ – PROVITAMINE B5 330 ml TESTÉ DERMATOLOGIQUEMENT Soin réparateur hydratant et protecteur pour cheveux secs, abîmés ou fragilisés Après le shampoing, cet après-shampoing riche et onctueux à base d’huile d’argan biologique nourrit profondément les cheveux, répare les dommages, renforce la cuticule à chaque utilisation et aide à restaurer douceur, élasticité et brillance. Il protège également les cheveux contre la chaleur du coiffage et les agressions environnementales tout en facilitant le démêlage pour une chevelure plus lisse, soyeuse et disciplinée. Avantages : • Hydrate, nourrit et adoucit les cheveux • Répare les cheveux abîmés et les pointes fourchues • Renforce la structure capillaire pour plus de résistance • Protège contre les dommages liés à la chaleur du coiffage • Réduit les frisottis et facilite le démêlage • Laisse les cheveux plus doux, brillants et lisses Conseil d’utilisation : Après le shampoing, appliquer une quantité suffisante d’après-shampoing sur cheveux mouillés, masser doucement puis laisser poser 1 à 2 minutes, puis rincer abondamment. Pour de meilleurs résultats, utiliser régulièrement avec un shampoing Biobalance adapté.</t>
+          <t>Huile d’argan biologique – beurre de karité – provitamine B5. Soin réparateur hydratant et protecteur pour cheveux secs, abîmés ou fragilisés Après le shampoing, cet après-shampoing riche et onctueux à base d’huile d’argan biologique nourrit profondément les cheveux, répare les dommages, renforce la cuticule à chaque utilisation et aide à restaurer douceur, élasticité et brillance. Il protège également les cheveux contre la chaleur du coiffage et les agressions environnementales tout en facilitant le démêlage pour une chevelure plus lisse, soyeuse et disciplinée.
+Avantages :
+• Hydrate, nourrit et adoucit les cheveux
+• Répare les cheveux abîmés et les pointes fourchues
+• Renforce la structure capillaire pour plus de résistance
+• Protège contre les dommages liés à la chaleur du coiffage
+• Réduit les frisottis et facilite le démêlage
+• Laisse les cheveux plus doux, brillants et lisses
+Formule : respectueux des animaux, sans colorant, testé dermatologiquement, sans gluten, sans huile minérale, sans pétrolatum, sans silicone.</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
+          <t>Après le shampoing, appliquer une quantité suffisante d’après-shampoing sur cheveux mouillés, masser doucement puis laisser poser 1 à 2 minutes, puis rincer abondamment. Pour de meilleurs résultats, utiliser régulièrement avec un shampoing Biobalance adapté.</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Aqua, Cetearyl Alcohol, Behentrimonium Chloride, Coco-Glucoside, Glyceryl Oleate, Betaine, Behenamidopropyl Dimethylamine, Argania Spinosa Kernel Oil, Cetearyl Glucoside, Hydrolyzed Corn Protein, Hydrolyzed Wheat Protein, Butyrospermum Parkii Butter, Hydrogenated Palm Glycerides Citrate, Tocopherol, Panthenol, Hexylene Glycol, Saccharum Officinarum Extract, Citrus Limon Fruit Extract, Pyrus Malus Fruit Extract, Camellia Sinensis Leaf Extract, Hexapeptide-11, Hydrolyzed Soy Protein, Saccharomyces/Zinc Ferment, Saccharomyces/Copper Ferment, Saccharomyces/Magnesium Ferment, Saccharomyces/Iron Ferment, Saccharomyces/Silicon Ferment, Leuconostoc/Radish Root Ferment Filtrate, Glycerin, Allantoin, Centella Asiatica Extract, Hydroxypropyl Guar Hydroxypropyltrimonium Chloride, Hydroxyethylcellulose, Tetrasodium Glutamate Diacetate, Sorbitan Caprylate, Propanediol, Isopropyl Alcohol, Parfum, Citric Acid, Benzoic Acid</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr">
+        <is>
           <t>images/8697711700224.jpg</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>https://biobalance.tn/soins-capillaires/51-customizable-mug.html</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>https://biobalance.tn/soins-capillaires/51-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>https://biobalance.tn/soins-capillaires/51-customizable-mug.html | https://www.barcodelookup.com/8697711700224</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -633,39 +686,59 @@
           <t>Super Pure Gel Cream Moisturizer</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Super Cream</t>
+        </is>
+      </c>
       <c r="F4" t="inlineStr">
         <is>
           <t>Crèmes visage</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>50 ml</t>
+        </is>
+      </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>La niacinamide multifonctionnelle (vitamine B3) apporte des solutions efficaces aux problématiques des peaux grasses et sujettes au vieillissement, en agissant simultanément sur l’hydratation, le sébum et les imperfections. Avantages : • Hydrate la peau sans provoquer d’acné • Régule la sécrétion de sébum • Cible les imperfections et les points noirs • Affine le grain de peau et l’apparence des pores Conseil d’utilisation : Appliquer deux fois par jour, matin et soir, sur le visage et le cou.</t>
+          <t>La niacinamide multifonctionnelle (vitamine B3) apporte des solutions efficaces aux problématiques des peaux grasses et sujettes au vieillissement, en agissant simultanément sur l’hydratation, le sébum et les imperfections.
+Avantages :
+• Hydrate la peau sans provoquer d’acné
+• Régule la sécrétion de sébum
+• Cible les imperfections et les points noirs
+• Affine le grain de peau et l’apparence des pores
+Formule : respectueux des animaux, sans colorant, testé dermatologiquement, sans gluten, sans huile minérale, sans parfum, sans pétrolatum, sans silicone, vegan, d’origine naturelle.</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
+          <t>Appliquer deux fois par jour, matin et soir, sur le visage et le cou.</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Aqua, Glycerin, Coco-Caprylate/Caprate, Glyceryl Stearate, Butylene Glycol, Niacinamide, Cetearyl Alcohol, Salicylic Acid, Polyglyceryl-6 Palmitate/Succinate, Zinc PCA, Acacia Senegal Gum, Xanthan Gum, Tocopherol, Propanediol, Tetrasodium Glutamate Diacetate, Sorbitan Caprylate, Benzoic Acid. ALCOHOL FREE</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr">
+        <is>
           <t>images/8697711602016.jpg</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>https://biobalance.tn/supercreams-/31-customizable-mug.html</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>https://biobalance.tn/supercreams-/31-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>https://biobalance.tn/supercreams-/31-customizable-mug.html | https://www.barcodelookup.com/8697711602016</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -688,7 +761,11 @@
           <t>Super Plump Cream Moisturizer</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Super Cream</t>
+        </is>
+      </c>
       <c r="F5" t="inlineStr">
         <is>
           <t>Crèmes visage</t>
@@ -701,30 +778,43 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Cette crème hydratante combine collagène hydrolysé et acide hyaluronique multi-moléculaire pour offrir une hydratation profonde, repulper la peau, améliorer l’élasticité et atténuer l’apparence des rides et des ridules. Sa texture riche mais rapidement absorbée aide à donner un aspect plus lisse, ferme et revitalisé à la peau. Avantages : • Soutient la production de collagène pour une peau plus ferme • Hydrate intensément en profondeur • Repulpe la peau et réduit les rides et ridules • Améliore l’élasticité et l’apparence générale • Texture riche, veloutée et rapidement absorbée Conseil d’utilisation : Appliquer deux fois par jour, matin et soir, sur le visage et le cou, sur une peau propre.</t>
+          <t>Cette crème hydratante combine collagène hydrolysé et acide hyaluronique multi-moléculaire pour offrir une hydratation profonde, repulper la peau, améliorer l’élasticité et atténuer l’apparence des rides et des ridules. Sa texture riche mais rapidement absorbée aide à donner un aspect plus lisse, ferme et revitalisé à la peau.
+Avantages :
+• Soutient la production de collagène pour une peau plus ferme
+• Hydrate intensément en profondeur
+• Repulpe la peau et réduit les rides et ridules
+• Améliore l’élasticité et l’apparence générale
+• Texture riche, veloutée et rapidement absorbée
+Formule : respectueux des animaux, sans colorant, testé dermatologiquement, sans gluten, sans huile minérale, sans parfum, sans pétrolatum, sans silicone.</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
+          <t>Appliquer deux fois par jour, matin et soir, sur le visage et le cou, sur une peau propre.</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Aqua, Glycerin, Caprylic/Capric Triglyceride, Coco-Caprylate/Caprate, Butylene Glycol, Glyceryl Stearate, Cetearyl Alcohol, Hydrolyzed Collagen, Polyglyceryl-6 Palmitate/Succinate, Sodium Hyaluronate, Tocopherol, Xanthan Gum, Tetrasodium Glutamate Diacetate, Sorbitan Caprylate, Propanediol, Benzoic Acid. ALCOHOL FREE</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr">
+        <is>
           <t>images/8697711602030.jpg</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>https://biobalance.tn/supercreams-/33-customizable-mug.html</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>https://biobalance.tn/supercreams-/33-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>https://biobalance.tn/supercreams-/33-customizable-mug.html | https://www.barcodelookup.com/8697711602030</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -747,39 +837,60 @@
           <t>Super Eye Intensive Moisturizing Eye Contour Cream</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Super Cream</t>
+        </is>
+      </c>
       <c r="F6" t="inlineStr">
         <is>
           <t>Crèmes visage</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>20 ml</t>
+        </is>
+      </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Cette crème contour des yeux associe collagène hydrolysé, acide hyaluronique multi-moléculaire et vitamine C pour hydrater intensément, améliorer l’élasticité de la peau et lisser l’apparence des rides et ridules. Elle aide également à illuminer et raffermir le contour des yeux. Avantages : • Améliore la fermeté et l’élasticité de la peau • Hydrate intensément le contour des yeux • Aide à réduire l’apparence des rides et ridules • Illumine et unifie le regard • Texture légère, rapidement absorbée Conseil d’utilisation : Appliquer deux fois par jour, matin et soir, sur le contour des yeux en tapotant délicatement.</t>
+          <t>Cette crème contour des yeux associe collagène hydrolysé, acide hyaluronique multi-moléculaire et vitamine C pour hydrater intensément, améliorer l’élasticité de la peau et lisser l’apparence des rides et ridules. Elle aide également à illuminer et raffermir le contour des yeux.
+Avantages :
+• Améliore la fermeté et l’élasticité de la peau
+• Hydrate intensément le contour des yeux
+• Aide à réduire l’apparence des rides et ridules
+• Illumine et unifie le regard
+• Texture légère, rapidement absorbée
+Formule : respectueux des animaux, sans colorant, testé dermatologiquement, sans gluten, sans huile minérale, sans parfum, sans pétrolatum, sans silicone.</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
+          <t>Appliquer deux fois par jour, matin et soir, sur le contour des yeux en tapotant délicatement.</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Aqua, Glycerin, Coco-Caprylate/Caprate, Butylene Glycol, Glyceryl Stearate, Cetearyl Alcohol, Hydrolyzed Collagen, Polyglyceryl-6 Palmitate/Succinate, Sodium Hyaluronate, 3-O-Ethyl Ascorbic Acid, Tocopherol, Propanediol, Xanthan Gum, Tetrasodium Glutamate Diacetate, Sorbitan Caprylate, Benzoic Acid. ALCOHOL FREE</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr">
+        <is>
           <t>images/8697711602061.jpg</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="M6" t="inlineStr">
         <is>
           <t>https://biobalance.tn/supercreams-/32-customizable-mug.html</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>https://biobalance.tn/supercreams-/32-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>https://biobalance.tn/supercreams-/32-customizable-mug.html | https://www.barcodelookup.com/8697711602061</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -799,10 +910,14 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Déodorant naturel roll-on 50 ml</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr"/>
+          <t>Déodorant Naturel Roll-On Anti-Repousse</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Dry &amp; Smooth</t>
+        </is>
+      </c>
       <c r="F7" t="inlineStr">
         <is>
           <t>Soins personnels</t>
@@ -815,30 +930,37 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Le Dry &amp; Smooth Roll-On de Biobalance protège efficacement contre les odeurs pendant 48h, tout en aidant à réduire l’apparence des poils sous les aisselles. Sa formule douce, sans alcool, convient à tous les types de peau.</t>
+          <t>Le Dry &amp; Smooth Roll-On de Biobalance protège efficacement contre les odeurs pendant 48h, tout en aidant à réduire l’apparence des poils sous les aisselles. Sa formule douce, sans alcool, convient à tous les types de peau.
+Formule : respectueux des animaux, sans colorant, testé dermatologiquement, sans gluten, sans huile minérale, sans pétrolatum, sans silicone, vegan, d’origine naturelle.</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
+          <t>Agiter avant emploi pour activer la formule. Appliquer sur des aisselles propres et sèches.</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Aqua, Butylene Glycol, Pentylene Glycol, Glycerin, Propanediol, Potassium Alum, Triethyl Citrate, Cetearyl Alcohol, Dicaprylyl Carbonate, Polyglyceryl-6 Stearate, Caprylic/Capric Triglyceride, Tribehenin, Tocopherol, Polyglyceryl-6 Behenate, Tetrasodium Glutamate Diacetate, Sorbitan Laurate, Nylon-12, Palmatine, Hydroxyethylcellulose, Parfum, Hydroxyacetophenone. ALCOHOL FREE ALUMINUM CHLOROHYDRATE FREE</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr">
+        <is>
           <t>images/8697711622427.jpg</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="M7" t="inlineStr">
         <is>
           <t>https://biobalance.tn/soins-personnels/66-customizable-mug.html</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="N7" t="inlineStr">
         <is>
           <t>https://biobalance.tn/soins-personnels/66-customizable-mug.html</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -858,7 +980,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>DRY &amp; SPORT POUR HOMME ROLL-ON NATUREL 50 ML</t>
+          <t>Dry &amp; Sport pour Homme Roll-On Naturel</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -878,30 +1000,37 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Le Dry &amp; Sport Roll-On pour homme assure une protection efficace contre les odeurs jusqu’à 48h, tout en aidant à éclaircir et uniformiser la peau des aisselles. Sa formule naturelle, sans alcool et sans sels d’aluminium agressifs, respecte la peau sensible et permet de maintenir une sensation de fraîcheur et de confort tout au long de la journée.Adapté aux hommes actifs, il combine efficacité déodorante et soin de la peau.</t>
+          <t>Le Dry &amp; Sport Roll-On pour homme assure une protection efficace contre les odeurs jusqu’à 48h, tout en aidant à éclaircir et uniformiser la peau des aisselles. Sa formule naturelle, sans alcool et sans sels d’aluminium agressifs, respecte la peau sensible et permet de maintenir une sensation de fraîcheur et de confort tout au long de la journée. Adapté aux hommes actifs, il combine efficacité déodorante et soin de la peau.
+Formule : respectueux des animaux, sans colorant, testé dermatologiquement, sans gluten, sans huile minérale, sans pétrolatum, sans silicone, vegan, d’origine naturelle.</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
+          <t>Agiter avant emploi pour activer la formule. Appliquer sur des aisselles propres et sèches.</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Aqua, Butylene Glycol, Pentylene Glycol, Glycerin, Propanediol, Potassium Alum, Triethyl Citrate, Magnesium PCA, Camellia Sinensis Leaf Extract, Menthol, Tetrasodium Glutamate Diacetate, Hydroxyethylcellulose, Parfum, Hydroxyacetophenone. ALCOHOL FREE ALUMINUM CHLOROHYDRATE FREE</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr">
+        <is>
           <t>images/8697711622434.jpg</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="M8" t="inlineStr">
         <is>
           <t>https://biobalance.tn/soins-personnels/68-customizable-mug.html</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="N8" t="inlineStr">
         <is>
           <t>https://biobalance.tn/soins-personnels/68-customizable-mug.html</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -921,7 +1050,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>DRY &amp; WHITE – Roll-On Naturel Éclaircissant 50 ml</t>
+          <t>Dry &amp; White Whitening Natural Roll-On Deodorant</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -941,34 +1070,37 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Déodorant roll-on naturel qui offre une protection efficace jusqu’à 48 heures contre les odeurs et l’humidité, tout en respectant le processus naturel de transpiration. Sa formule est enrichie en Alpha-Arbutine, Niacinamide (Vitamine B3) et Vitamine C, des actifs reconnus pour aider à éclaircir et uniformiser la peau des aisselles, en réduisant progressivement les taches foncées. Sans alcool ni sels d’aluminium, il convient aux peaux sensibles et laisse une sensation de fraîcheur et de confort durable.</t>
+          <t>Déodorant roll-on naturel éclaircissant : protection 48 h contre les mauvaises odeurs et aide à éclaircir la peau délicate des aisselles.
+Formule : respectueux des animaux, sans colorant, testé dermatologiquement, sans gluten, sans huile minérale, sans pétrolatum, sans silicone, vegan, d’origine naturelle.</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
+          <t>Agiter avant emploi pour activer la formule. Appliquer sur des aisselles propres et sèches.</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Aqua, Butylene Glycol, Pentylene Glycol, Glycerin, Propanediol, Potassium Alum, Triethyl Citrate, Alpha-Arbutin, Niacinamide, 3-O-Ethyl Ascorbic Acid, Tetrasodium Glutamate Diacetate, Hydroxyethylcellulose, Parfum, Hydroxyacetophenone. ALCOHOL FREE ALUMINUM CHLOROHYDRATE FREE</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr">
+        <is>
           <t>images/8697711622410.jpg</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="M9" t="inlineStr">
         <is>
           <t>https://biobalance.tn/soins-personnels/67-customizable-mug.html</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>https://biobalance.tn/soins-personnels/67-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>Données et photo reprises du code 8697711740411 (même produit, ancien code probable)</t>
-        </is>
-      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>https://biobalance.tn/soins-personnels/67-customizable-mug.html | https://www.barcodelookup.com/8697711622410</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -988,7 +1120,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>DRY &amp; WHITE – Roll-On Naturel Éclaircissant 50 ml</t>
+          <t>Dry &amp; White – Roll-On Naturel Éclaircissant</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1008,30 +1140,37 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Déodorant roll-on naturel qui offre une protection efficace jusqu’à 48 heures contre les odeurs et l’humidité, tout en respectant le processus naturel de transpiration. Sa formule est enrichie en Alpha-Arbutine, Niacinamide (Vitamine B3) et Vitamine C, des actifs reconnus pour aider à éclaircir et uniformiser la peau des aisselles, en réduisant progressivement les taches foncées. Sans alcool ni sels d’aluminium, il convient aux peaux sensibles et laisse une sensation de fraîcheur et de confort durable.</t>
+          <t>Déodorant roll-on naturel qui offre une protection efficace jusqu’à 48 heures contre les odeurs et l’humidité, tout en respectant le processus naturel de transpiration. Sa formule est enrichie en Alpha-Arbutine, Niacinamide (Vitamine B3) et Vitamine C , des actifs reconnus pour aider à éclaircir et uniformiser la peau des aisselles , en réduisant progressivement les taches foncées. Sans alcool ni sels d’aluminium, il convient aux peaux sensibles et laisse une sensation de fraîcheur et de confort durable.
+Formule : respectueux des animaux, sans colorant, testé dermatologiquement, sans gluten, sans huile minérale, sans pétrolatum, sans silicone, vegan, d’origine naturelle.</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
+          <t>Agiter avant emploi pour activer la formule. Appliquer sur des aisselles propres et sèches.</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Aqua, Butylene Glycol, Pentylene Glycol, Glycerin, Propanediol, Potassium Alum, Triethyl Citrate, Alpha-Arbutin, Niacinamide, 3-O-Ethyl Ascorbic Acid, Tetrasodium Glutamate Diacetate, Hydroxyethylcellulose, Parfum, Hydroxyacetophenone. ALCOHOL FREE ALUMINUM CHLOROHYDRATE FREE</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr">
+        <is>
           <t>images/8697711740411.jpg</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="M10" t="inlineStr">
         <is>
           <t>https://biobalance.tn/soins-personnels/67-customizable-mug.html</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
+      <c r="N10" t="inlineStr">
         <is>
           <t>https://biobalance.tn/soins-personnels/67-customizable-mug.html</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1051,7 +1190,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>DERMASEBUM PURIFYING FACIAL CLEANSING GEL</t>
+          <t>Dermasebum Purifying Facial Cleansing Gel</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1071,30 +1210,37 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Un soin quotidien contre les problèmes de peau grasse Effet « Soft Peeling » La formule sans savon et sans huile nettoie en douceur et en profondeur les pores en éliminant saletés, impuretés et maquillage. La mousse légère se rince facilement, sans laisser de résidus pouvant obstruer les pores. Gluconate de Zinc et AHA naturels (Myrtille, canne à sucre, érable à sucre, citron et extrait d’orange) réduisent la production excessive de sébum, la taille des pores, la brillance et les points noirs. Glycérine, Allantoïne, Bétaïne naturelle et Vitamine E Améliorent la barrière naturelle de la peau, préviennent la perte d’hydratation et aident à maintenir une peau bien hydratée. Mode d’emploi Utiliser quotidiennement. Masser délicatement sur le visage et le cou humides, deux fois par jour. Rincer abondamment à l’eau tiède puis sécher en tamponnant avec une serviette douce.</t>
+          <t>Un soin quotidien contre les problèmes de peau grasse Effet « Soft Peeling » La formule sans savon et sans huile nettoie en douceur et en profondeur les pores en éliminant saletés, impuretés et maquillage. La mousse légère se rince facilement, sans laisser de résidus pouvant obstruer les pores. Personnalisation N'oubliez pas de sauvegarder votre personnalisation pour pouvoir l'ajouter au panier Insérer votre texte ici 250 caractères max Enregistrer la personnalisation
+Formule : respectueux des animaux, sans colorant, testé dermatologiquement, sans gluten, sans pétrolatum, sans silicone.</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
+          <t>Utiliser quotidiennement. Masser délicatement sur le visage et le cou humides, deux fois par jour. Rincer abondamment à l’eau tiède puis sécher en tamponnant avec une serviette douce.</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Aqua, Sodium C14-16 Olefin Sulfonate, Niacinamide, Cocamidopropyl Betaine, Glycerin, Cocamidopropyl Hydroxysultaine, PEG-4 Rapeseedamide, Decyl Glucoside, PEG-120 Methyl Glucose Dioleate, Zinc Gluconate, Zinc Chloride, Centella Asiatica Extract, Vaccinium Myrtillus Fruit Extract, Saccharum Officinarum Extract, Acer Saccharum Extract, Citrus Aurantium Dulcis Fruit Extract, Citrus Limon Fruit Extract, Lactic Acid, Citric Acid, Tartaric Acid, Glycolic Acid, Malic Acid, Panthenol, Allantoin, Tocopheryl Acetate, Hexamidine Diisethionate, C12-15 Alkyl Lactate, Sodium Gluconate, Sorbitan Caprylate, Propanediol, Polysorbate 20, Parfum, Benzoic Acid. ALCOHOL FREE</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr">
+        <is>
           <t>images/8697711701009.jpg</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="M11" t="inlineStr">
         <is>
           <t>https://biobalance.tn/nettoyants-visage/28-customizable-mug.html</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
+      <c r="N11" t="inlineStr">
         <is>
           <t>https://biobalance.tn/nettoyants-visage/28-customizable-mug.html</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="M11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1114,7 +1260,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>DERMASOOTHE SOOTHING FACIAL CLEANSING GEL</t>
+          <t>Dermasoothe Soothing Facial Cleansing Gel</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1134,30 +1280,39 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Un soin apaisant qui respecte les peaux sensibles. Effet « Soft Peeling » La formule sans savon et sans huile nettoie la peau en douceur et élimine saletés, impuretés et maquillage.La mousse légère se rince facilement, sans laisser de résidus pouvant obstruer les pores. Avantages : Améliore la fonction naturelle de la barrière cutanée et réduit les rougeurs, les picotements et la sensibilité. INGRÉDIENTS : Bisabolol Complexe d’Acides AminésRenforce la résistance et la tolérance de la peau face aux agressions extérieures irritantes responsables de rougeurs, tiraillements et sensations de picotement.Glycérine, Aloe Vera, Allantoïne, Panthénol et Vitamine E Améliorent la barrière naturelle de la peau, préviennent la perte d’hydratation et aident à maintenir une peau bien hydratée. Mode d’emploi : Utiliser quotidiennement. Masser délicatement sur le visage et le cou humides, deux fois par jour. Rincer abondamment à l’eau tiède puis sécher en tamponnant avec une serviette douce.</t>
+          <t>Un soin apaisant qui respecte les peaux sensibles. Effet « Soft Peeling » La formule sans savon et sans huile nettoie la peau en douceur et élimine saletés, impuretés et maquillage. La mousse légère se rince facilement, sans laisser de résidus pouvant obstruer les pores.
+Avantages :
+• Améliore la fonction naturelle de la barrière cutanée et réduit les rougeurs, les picotements et la sensibilité. INGRÉDIENTS : Bisabolol Complexe d’Acides Aminés Renforce la résistance et la tolérance de la peau face aux agressions extérieures irritantes responsables de rougeurs, tiraillements et sensations de picotement. Glycérine, Aloe Vera, Allantoïne, Panthénol et Vitamine E Améliorent la barrière naturelle de la peau, préviennent la perte d’hydratation et aident à maintenir une peau bien hydratée.
+Formule : respectueux des animaux, sans colorant, testé dermatologiquement, sans gluten, sans pétrolatum, sans silicone.</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
+          <t>Utiliser quotidiennement. Masser délicatement sur le visage et le cou humides, deux fois par jour. Rincer abondamment à l’eau tiède puis sécher en tamponnant avec une serviette douce.</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Aqua, Glycerin, Sodium Laureth-5 Carboxylate, Sodium C14-16 Olefin Sulfonate, Cocamidopropyl Hydroxysultaine, Niacinamide, PEG-4 Rapeseedamide, Decyl Glucoside, PEG-120 Methyl Glucose Dioleate, Bisabolol, Aloe Barbadensis Leaf Juice, Sodium PCA, Sodium Lactate, Arginine, Aspartic Acid, PCA, Glycine, Alanine, Serine, Valine, Proline, Threonine, Isoleucine, Histidine, Phenylalanine, Panthenol, Allantoin, Tocopheryl Acetate, C12-15 Alkyl Lactate, Cocamidopropyl Betaine, Sodium Gluconate, Sorbitan Caprylate, Propanediol, Polysorbate 20, Parfum, Benzoic Acid, Citric Acid, Potassium Sorbate, Sodium Benzoate. ALCOHOL FREE</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr">
+        <is>
           <t>images/8697711701016.jpg</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="M12" t="inlineStr">
         <is>
           <t>https://biobalance.tn/nettoyants-visage/23-customizable-mug.html</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr">
+      <c r="N12" t="inlineStr">
         <is>
           <t>https://biobalance.tn/nettoyants-visage/23-customizable-mug.html</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="M12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1177,7 +1332,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>HELLO CLEAN CERAMIDE BOOSTER BI-PHASE MICELLAR WATER</t>
+          <t>Hello Clean Ceramide Booster Bi-Phase Micellar Water</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1197,30 +1352,43 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Eau micellaire biphasée démaquillante hydratante 500 ml Démaquillant micellaire biphasé spécialement formulé pour les peaux sèches, normales et sensibles. Sa formule à deux phases élimine efficacement le maquillage waterproof, les impuretés et l’excès de sébum, tout en renforçant la barrière cutanée, apportant une hydratation profonde et en calmant les sensations d’inconfort. Enrichie en céramide, vitamine C, camomille et squalane, elle nourrit et apaise la peau sans laisser de résidu gras ni collant. Avantages : • Élimine facilement le maquillage, même waterproof • Renforce la barrière cutanée pour protéger contre la perte d’hydratation • Hydrate profondément et nourrit la peau • Apaise la sensibilité et réduit les rougeurs • Laisse la peau douce, propre et confortable sans sensation grasse ou collante Conseil d’utilisation : Agiter avant utilisation pour mélanger les deux phases. Appliquer sur le visage, les yeux et les lèvres à l’aide d’un coton, sans frotter. Aucun rinçage nécessaire.</t>
+          <t>Eau micellaire biphasée démaquillante hydratante. Démaquillant micellaire biphasé spécialement formulé pour les peaux sèches, normales et sensibles. Sa formule à deux phases élimine efficacement le maquillage waterproof, les impuretés et l’excès de sébum, tout en renforçant la barrière cutanée, apportant une hydratation profonde et en calmant les sensations d’inconfort. Enrichie en céramide, vitamine C, camomille et squalane, elle nourrit et apaise la peau sans laisser de résidu gras ni collant.
+Avantages :
+• Élimine facilement le maquillage, même waterproof
+• Renforce la barrière cutanée pour protéger contre la perte d’hydratation
+• Hydrate profondément et nourrit la peau
+• Apaise la sensibilité et réduit les rougeurs
+• Laisse la peau douce, propre et confortable sans sensation grasse ou collante
+Formule : respectueux des animaux, sans colorant, testé dermatologiquement, sans gluten, sans huile minérale, sans parfum, sans pétrolatum, sans silicone, vegan, d’origine naturelle.</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
+          <t>Agiter avant utilisation pour mélanger les deux phases. Appliquer sur le visage, les yeux et les lèvres à l’aide d’un coton, sans frotter. Aucun rinçage nécessaire.</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Aqua, Coco-Caprylate, Butylene Glycol, Glycerin, Pentylene Glycol, Propanediol, Squalane, Polyglyceryl-4 Laurate/Sebacate, Polyglyceryl-6 Caprylate/Caprate, Ceramide NP, Sodium Hyaluronate, Ascorbyl Tetraisopalmitate, Tocopherol, Chamomilla Recutita Flower Extract, Sodium Gluconate, Sodium Levulinate, Potassium Sorbate. ALCOHOL FREE</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr">
+        <is>
           <t>images/8697711621833.jpg</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="M13" t="inlineStr">
         <is>
           <t>https://biobalance.tn/nettoyants-visage/34-customizable-mug.html</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>https://biobalance.tn/nettoyants-visage/34-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>https://biobalance.tn/nettoyants-visage/34-customizable-mug.html | https://www.barcodelookup.com/8697711621833</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1240,7 +1408,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>HELLO CLEAN HYALURONIC HYDRATION MICELLAR WATER</t>
+          <t>Hello Clean Hyaluronic Hydration Micellar Water</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1260,30 +1428,43 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Eau micellaire démaquillante hydratante 500 ml Démaquillant micellaire hydratant spécialement formulé pour nettoyer en profondeur tout en apportant une hydratation intense, même aux peaux sèches et sensibles. Grâce à un complexe d’acide hyaluronique, d’acides aminés, de Pentavitin et d’extrait de Centella Asiatica, cette eau micellaire élimine efficacement le maquillage, les impuretés et l’excès de sébum, tout en nourrissant, repulpant et sublimant l’éclat naturel de la peau. Avantages : • Nettoie en profondeur – élimine maquillage, impuretés et excès de sébum • Hydratation intense – l’acide hyaluronique et le Pentavitin boostent l’hydratation • Renforce la barrière cutanée – grâce au complexe d’acides aminés et à la Centella Asiatica • Repulpe et illumine la peau pour une apparence plus lisse et radieuse • Douce pour les yeux – ne pique pas et ne trouble pas la vision Conseil d’utilisation : Appliquer sur le visage, les yeux et les lèvres à l’aide d’un coton. Inutile de rincer.</t>
+          <t>Eau micellaire démaquillante hydratante. Démaquillant micellaire hydratant spécialement formulé pour nettoyer en profondeur tout en apportant une hydratation intense, même aux peaux sèches et sensibles. Grâce à un complexe d’acide hyaluronique, d’acides aminés, de Pentavitin et d’extrait de Centella Asiatica, cette eau micellaire élimine efficacement le maquillage, les impuretés et l’excès de sébum, tout en nourrissant, repulpant et sublimant l’éclat naturel de la peau.
+Avantages :
+• Nettoie en profondeur – élimine maquillage, impuretés et excès de sébum
+• Hydratation intense – l’acide hyaluronique et le Pentavitin boostent l’hydratation
+• Renforce la barrière cutanée – grâce au complexe d’acides aminés et à la Centella Asiatica
+• Repulpe et illumine la peau pour une apparence plus lisse et radieuse
+• Douce pour les yeux – ne pique pas et ne trouble pas la vision
+Formule : respectueux des animaux, sans colorant, testé dermatologiquement, sans gluten, sans huile minérale, sans parfum, sans pétrolatum, sans silicone, vegan, d’origine naturelle.</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
+          <t>Appliquer sur le visage, les yeux et les lèvres à l’aide d’un coton. Inutile de rincer.</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Aqua, Butylene Glycol, Glycerin, Pentylene Glycol, Propanediol, Polyglyceryl-4 Laurate/Sebacate, Polyglyceryl-6 Caprylate/Caprate, Betaine, Sodium Hyaluronate, Saccharide Isomerate, Inulin, Centella Asiatica Leaf Extract, Sodium PCA, Arginine, Sodium Gluconate, Sodium Lactate, Aspartic Acid, PCA, Glycine, Alanine, Serine, Valine, Proline, Threonine, Isoleucine, Histidine, Phenylalanine, Sodium Levulinate, Citric Acid, Sodium Citrate, Potassium Sorbate. ALCOHOL FREE</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr">
+        <is>
           <t>images/8697711621819.jpg</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="M14" t="inlineStr">
         <is>
           <t>https://biobalance.tn/nettoyants-visage/27-customizable-mug.html</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>https://biobalance.tn/nettoyants-visage/27-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>https://biobalance.tn/nettoyants-visage/27-customizable-mug.html | https://www.barcodelookup.com/8697711621819</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1303,7 +1484,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>HELLO CLEAN NIACINAMIDE CLARITY MICELLAR WATER</t>
+          <t>Hello Clean Niacinamide Clarity Micellar Water</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1323,30 +1504,43 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Eau micellaire démaquillante clarifiante 500 ml Démaquillant micellaire spécialement formulé pour les peaux grasses et mixtes. Sa formule enrichie en niacinamide, extrait de thé vert et extrait de concombre aide à réguler la production de sébum, nettoyer les pores en profondeur et prévenir l’apparition d’acné et de points noirs, tout en éliminant le maquillage, l’excès d’huile et les impuretés sans dessécher la peau. Avantages : • Aide à contrôler l’excès de sébum et la brillance • Nettoie efficacement le maquillage et les impuretés • Aide à réduire l’apparence des pores dilatés • Rafraîchit, apaise et hydrate grâce aux extraits naturels • Préserve l’équilibre naturel de la peau sans dessécher Conseil d’utilisation : Appliquer sur le visage, les yeux et les lèvres à l’aide d’un coton, sans frotter. Aucun rinçage nécessaire.</t>
+          <t>Eau micellaire démaquillante clarifiante. Démaquillant micellaire spécialement formulé pour les peaux grasses et mixtes. Sa formule enrichie en niacinamide, extrait de thé vert et extrait de concombre aide à réguler la production de sébum, nettoyer les pores en profondeur et prévenir l’apparition d’acné et de points noirs, tout en éliminant le maquillage, l’excès d’huile et les impuretés sans dessécher la peau.
+Avantages :
+• Aide à contrôler l’excès de sébum et la brillance
+• Nettoie efficacement le maquillage et les impuretés
+• Aide à réduire l’apparence des pores dilatés
+• Rafraîchit, apaise et hydrate grâce aux extraits naturels
+• Préserve l’équilibre naturel de la peau sans dessécher
+Formule : respectueux des animaux, sans colorant, testé dermatologiquement, sans gluten, sans huile minérale, sans parfum, sans pétrolatum, sans silicone, vegan, d’origine naturelle.</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
+          <t>Appliquer sur le visage, les yeux et les lèvres à l’aide d’un coton, sans frotter. Aucun rinçage nécessaire.</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Aqua, Glycerin, Butylene Glycol, Pentylene Glycol, Propanediol, Polyglyceryl-4 Laurate/Sebacate, Polyglyceryl-6 Caprylate/Caprate, Niacinamide, Camellia Sinensis Leaf Extract, Sodium Hyaluronate, Inulin, Cucumis Sativus Fruit Extract, Sodium Gluconate, Sodium Levulinate, Potassium Sorbate. ALCOHOL FREE</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr">
+        <is>
           <t>images/8697711621826.jpg</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr">
+      <c r="M15" t="inlineStr">
         <is>
           <t>https://biobalance.tn/nettoyants-visage/35-customizable-mug.html</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>https://biobalance.tn/nettoyants-visage/35-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>https://biobalance.tn/nettoyants-visage/35-customizable-mug.html | https://www.barcodelookup.com/8697711621826</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1366,7 +1560,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Eye Lash — sérum cils et sourcils 6 ml</t>
+          <t>Eyelash Growth Serum</t>
         </is>
       </c>
       <c r="E16" t="inlineStr"/>
@@ -1382,30 +1576,40 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Sérum pour cils et sourcils aux peptides (Biotinoyl Tripeptide-1), à la biotine et à l’acide hyaluronique. Appliquer une fine ligne à la base des cils ou sur les sourcils, de préférence le soir, pendant au moins 30 jours.</t>
+          <t>Sérum pour cils et sourcils aux peptides (Biotinoyl Tripeptide-1), à la biotine et à l’acide hyaluronique.
+Avantages :
+• Soutient la pousse et le volume des cils et des sourcils
+• Hydrate et nourrit grâce à l’acide hyaluronique et au panthénol
+Formule : respectueux des animaux, sans colorant, testé dermatologiquement, sans gluten, sans huile minérale, sans parfum, sans pétrolatum, sans conservateur, sans silicone.</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
+          <t>Retirer le maquillage et les résidus. Appliquer une fine ligne à la base des cils ou sur les sourcils, de préférence le soir (ou deux fois par jour). Utiliser chaque jour pendant au moins 30 jours. Éliminer les résidus d’huile démaquillante avant application.</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Aqua, Glycerin, Propanediol, Hydroxyethylcellulose, Biotinoyl Tripeptide-1, Serenoa Serrulata Fruit Extract, Maltodextrin, Biotin, Sodium Hyaluronate, Sodium PCA, Sodium Lactate, Arginine, Aspartic Acid, PCA, Glycine, Alanine, Serine, Valine, Proline, Threonine, Isoleucine, Histidine, Phenylalanine, Hydroxyacetophenone, Panthenol, Allantoin. ALCOHOL FREE</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr">
+        <is>
           <t>images/8697711722011.jpg</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr">
+      <c r="M16" t="inlineStr">
         <is>
           <t>https://www.barcodelookup.com/8697711722011</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr">
+      <c r="N16" t="inlineStr">
         <is>
           <t>https://www.barcodelookup.com/8697711722011</t>
         </is>
       </c>
-      <c r="L16" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="M16" t="inlineStr"/>
+      <c r="O16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1425,7 +1629,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Hello Clean — baume nettoyant 3 en 1 Vitamine C pure 100 ml</t>
+          <t>Hello Clean 3-in-1 Cleansing Balm Pure Vitamin C</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1445,30 +1649,45 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Baume nettoyant visage 3 en 1 à la vitamine C pure, pour peau terne. Sa texture sorbet se transforme en huile soyeuse au contact de la peau : il démaquille, nettoie et illumine. Spatule fournie.</t>
+          <t>Baume nettoyant visage 3 en 1 à la vitamine C pure, pour peau terne. Sa texture sorbet se transforme en huile soyeuse au contact de la peau : il démaquille le maquillage waterproof, enlève la crème solaire et les impuretés.
+Avantages :
+• Illumine le teint (vitamine C pure, antioxydant)
+• Réduit les rougeurs
+• Laisse la peau douce et hydratée
+Formule : respectueux des animaux, sans colorant, testé dermatologiquement, sans gluten, sans huile minérale, sans parfum, sans pétrolatum, sans conservateur, sans silicone, vegan, d’origine naturelle.</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
+          <t>Prélever la quantité voulue avec la spatule fournie. Masser sur peau sèche en mouvements circulaires jusqu’à dissolution du maquillage et des impuretés, ajouter de l’eau tiède, masser à nouveau puis rincer. Yeux : garder la paupière fermée.</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Caprylic/Capric Triglyceride, Dicaprylyl Carbonate, Euphorbia Cerifera Cera, Polyglyceryl-2 Caprate, Ascorbic Acid, Butylene Glycol, Hoya Lacunosa Flower Extract, Polysorbate 20, Tocopherol</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Usage externe uniquement. Tenir hors de portée des enfants. Conserver au frais, au sec, à l’abri du soleil.</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
           <t>images/8697711601514.jpg</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr">
+      <c r="M17" t="inlineStr">
         <is>
           <t>https://www.barcodelookup.com/8697711601514</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr">
+      <c r="N17" t="inlineStr">
         <is>
           <t>https://www.barcodelookup.com/8697711601514</t>
         </is>
       </c>
-      <c r="L17" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="M17" t="inlineStr"/>
+      <c r="O17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1488,7 +1707,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Hello Clean — baume nettoyant 3 en 1 Acide hyaluronique 100 ml</t>
+          <t>Hello Clean 3-in-1 Cleansing Balm Hyaluronic Acid</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1508,30 +1727,45 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Baume nettoyant visage 3 en 1 à l’acide hyaluronique, pour peau normale à sèche. Sa texture sorbet se transforme en huile soyeuse au contact de la peau : il démaquille, nettoie et hydrate. Spatule fournie.</t>
+          <t>Baume nettoyant visage 3 en 1 à l’acide hyaluronique (hyaluronate de sodium), pour peau normale à sèche. Sa texture sorbet se transforme en huile soyeuse au contact de la peau : il démaquille et nettoie en douceur.
+Avantages :
+• Hydrate intensément (acide hyaluronique)
+• Apaise grâce à l’extrait de fleur de Hoya Lacunosa
+• Laisse la peau douce et veloutée
+Formule : respectueux des animaux, sans colorant, testé dermatologiquement, sans gluten, sans huile minérale, sans parfum, sans pétrolatum, sans silicone, vegan, d’origine naturelle.</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
+          <t>Prélever la quantité voulue avec la spatule fournie. Masser sur peau sèche en mouvements circulaires jusqu’à dissolution du maquillage et des impuretés, ajouter de l’eau tiède, masser à nouveau puis rincer. Yeux : garder la paupière fermée.</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Caprylic/Capric Triglyceride, Dicaprylyl Carbonate, Euphorbia Cerifera Cera, Polyglyceryl-2 Caprate, Aqua, Butylene Glycol, Sodium Hyaluronate, Hoya Lacunosa Flower Extract, Sorbitan Caprylate, Propanediol, Benzoic Acid, Polysorbate 20, Tocopherol</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Usage externe uniquement. Tenir hors de portée des enfants. Conserver au frais, au sec, à l’abri du soleil.</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
           <t>images/8697711601538.jpg</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr">
+      <c r="M18" t="inlineStr">
         <is>
           <t>https://www.barcodelookup.com/8697711601538</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr">
+      <c r="N18" t="inlineStr">
         <is>
           <t>https://www.barcodelookup.com/8697711601538</t>
         </is>
       </c>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="M18" t="inlineStr"/>
+      <c r="O18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1551,7 +1785,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Hello Clean — baume nettoyant 3 en 1 Squalane 100 ml</t>
+          <t>Hello Clean 3-in-1 Cleansing Balm Squalane</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1571,30 +1805,45 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Baume nettoyant visage 3 en 1 au squalane et au bisabolol, pour peau sensible ou à rougeurs. Sa texture sorbet se transforme en huile soyeuse au contact de la peau : il démaquille, nettoie et apaise. Spatule fournie.</t>
+          <t>Baume nettoyant visage 3 en 1 au squalane et au bisabolol, pour peau sensible ou à rougeurs. Sa texture sorbet se transforme en huile soyeuse au contact de la peau : il démaquille et nettoie sans agresser.
+Avantages :
+• Nourrit et protège (squalane, antioxydant naturel)
+• Répare et calme la peau sensible ou irritée (bisabolol)
+• Laisse la peau douce et hydratée
+Formule : respectueux des animaux, sans colorant, testé dermatologiquement, sans gluten, sans huile minérale, sans parfum, sans pétrolatum, sans conservateur, sans silicone, vegan, d’origine naturelle.</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
+          <t>Prélever la quantité voulue avec la spatule fournie. Masser sur peau sèche en mouvements circulaires jusqu’à dissolution du maquillage et des impuretés, ajouter de l’eau tiède, masser à nouveau puis rincer. Yeux : garder la paupière fermée.</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Caprylic/Capric Triglyceride, Dicaprylyl Carbonate, Euphorbia Cerifera Cera, Squalane, Polyglyceryl-2 Caprate, Hoya Lacunosa Flower Extract, Bisabolol, Polysorbate 20, Tocopherol</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Usage externe uniquement. Tenir hors de portée des enfants. Conserver au frais, au sec, à l’abri du soleil.</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
           <t>images/8697711601521.jpg</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr">
+      <c r="M19" t="inlineStr">
         <is>
           <t>https://www.barcodelookup.com/8697711601521</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr">
+      <c r="N19" t="inlineStr">
         <is>
           <t>https://www.barcodelookup.com/8697711601521</t>
         </is>
       </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="M19" t="inlineStr"/>
+      <c r="O19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1614,7 +1863,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Hello Clean — baume nettoyant 3 en 1 Acide oléanolique 100 ml</t>
+          <t>Hello Clean 3-in-1 Cleansing Balm Oleanolic Acid</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1634,30 +1883,45 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Baume nettoyant visage 3 en 1 à l’acide oléanolique, pour peau grasse ou mixte : il contrôle l’excès de sébum et minimise les pores. Sa texture sorbet se transforme en huile soyeuse au contact de la peau. Spatule fournie.</t>
+          <t>Baume nettoyant visage 3 en 1 à l’acide oléanolique, pour peau grasse ou mixte. Sa texture sorbet se transforme en huile soyeuse au contact de la peau : il démaquille, nettoie et matifie.
+Avantages :
+• Contrôle l’excès de sébum
+• Minimise l’apparence des pores
+• Matifie et hydrate
+Formule : respectueux des animaux, sans colorant, testé dermatologiquement, sans gluten, sans huile minérale, sans parfum, sans pétrolatum, sans conservateur, sans silicone, vegan, d’origine naturelle.</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
+          <t>Prélever la quantité voulue avec la spatule fournie. Masser sur peau sèche en mouvements circulaires jusqu’à dissolution du maquillage et des impuretés, ajouter de l’eau tiède, masser à nouveau puis rincer. Yeux : garder la paupière fermée.</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Caprylic/Capric Triglyceride, Dicaprylyl Carbonate, Euphorbia Cerifera Cera, Polyglyceryl-2 Caprate, Butylene Glycol, Oleanolic Acid, Enantia Chlorantha Bark Extract, Hoya Lacunosa Flower Extract, Polysorbate 20, Tocopherol</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>Usage externe uniquement. Tenir hors de portée des enfants. Conserver au frais, au sec, à l’abri du soleil.</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
           <t>images/8697711601545.jpg</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr">
+      <c r="M20" t="inlineStr">
         <is>
           <t>https://www.barcodelookup.com/8697711601545</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr">
+      <c r="N20" t="inlineStr">
         <is>
           <t>https://www.barcodelookup.com/8697711601545</t>
         </is>
       </c>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="M20" t="inlineStr"/>
+      <c r="O20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1677,7 +1941,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>BETA SOLUTION PURE SALICYLIC ACID 2% SUPER SERUM</t>
+          <t>Beta Solution Pure Salicylic Acid 2% Super Serum</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1690,33 +1954,50 @@
           <t>Sérums</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr"/>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>30 ml</t>
+        </is>
+      </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>30 ml Testé dermatologiquement Exfoliation chimique ciblée contre les points noirs et blancs Ce sérum concentré contient 2 % d’acide salicylique, un acide bêta-hydroxy (BHA) reconnu pour ses propriétés lipolytiques (dissolution du sébum), kératolytiques (exfoliation des cellules mortes) et comédolytiques (désincrustation des pores). Grâce à sa capacité à pénétrer profondément dans les pores, il aide à éliminer les cellules mortes et l’excès de sébum, favorisant ainsi une peau plus nette et plus claire, notamment en ciblant les points noirs et points blancs. Avantages : • Élimine les cellules mortes et le sébum à l’intérieur des pores • Réduit visiblement les points noirs et les points blancs • Régule la production excessive de sébum • Améliore la texture et l’apparence globale de la peau • Aide à prévenir l’apparition de nouvelles imperfections Conseil d’utilisation : Utiliser une petite quantité sur une peau propre après le nettoyage, en évitant le contour des yeux. Appliquer matin et soir. Laisser le sérum être absorbé avant d’appliquer votre crème hydratante. Pour optimiser les résultats et protéger la peau, appliquer toujours une protection solaire pendant la journée lorsque vous utilisez ce produit et pendant une semaine après la fin de son utilisation.</t>
+          <t>Exfoliation chimique ciblée contre les points noirs et blancs Ce sérum concentré contient 2 % d’acide salicylique, un acide bêta-hydroxy (BHA) reconnu pour ses propriétés lipolytiques (dissolution du sébum), kératolytiques (exfoliation des cellules mortes) et comédolytiques (désincrustation des pores). Grâce à sa capacité à pénétrer profondément dans les pores, il aide à éliminer les cellules mortes et l’excès de sébum, favorisant ainsi une peau plus nette et plus claire, notamment en ciblant les points noirs et points blancs.
+Avantages :
+• Élimine les cellules mortes et le sébum à l’intérieur des pores
+• Réduit visiblement les points noirs et les points blancs
+• Régule la production excessive de sébum
+• Améliore la texture et l’apparence globale de la peau
+• Aide à prévenir l’apparition de nouvelles imperfections
+Formule : respectueux des animaux, sans colorant, testé dermatologiquement, sans gluten, sans huile minérale, sans parfum, sans pétrolatum, sans conservateur, sans silicone, vegan, d’origine naturelle.</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
+          <t>Utiliser une petite quantité sur une peau propre après le nettoyage, en évitant le contour des yeux. Appliquer matin et soir. Laisser le sérum être absorbé avant d’appliquer votre crème hydratante. Pour optimiser les résultats et protéger la peau, appliquer toujours une protection solaire pendant la journée lorsque vous utilisez ce produit et pendant une semaine après la fin de son utilisation.</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Aqua, Propanediol, Glycerin, Salicylic Acid, Polysorbate 20, Xanthan Gum, Hydroxyacetophenone, Tetrasodium Glutamate Diacetate</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr">
+        <is>
           <t>images/8697711600845.jpg</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr">
+      <c r="M21" t="inlineStr">
         <is>
           <t>https://biobalance.tn/serum/40-customizable-mug.html</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>https://biobalance.tn/serum/40-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>https://biobalance.tn/serum/40-customizable-mug.html | https://www.barcodelookup.com/8697711600845</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1736,7 +2017,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>DEEP PEELING SUPER SERUM</t>
+          <t>Deep Peeling Super Serum</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1749,33 +2030,50 @@
           <t>Sérums</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr"/>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>30 ml</t>
+        </is>
+      </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>AHA 10% + BHA 2% + RED ALGAE 30 ml TESTÉ DERMATOLOGIQUEMENT Peeling visage illuminateur &amp; unifiant le teint Le sérum Deep Peeling exfolie à la fois la surface de la peau et l’intérieur des pores grâce à une combinaison de 10 % d’AHAs (acides alpha-hydroxy : glycolique, lactique, mandélique) et 2 % de BHA (acide salicylique) dans une seule formule. Les AHAs agissent en éliminant les cellules mortes à la surface, tandis que le BHA pénètre profondément pour déboucher les pores et aider à prévenir les points noirs et boutons. Les algues rouges hydratent la peau et aident à accroître sa tolérance au traitement acide, pour un teint plus lisse, net et éclatant. Avantages : • Exfolie les couches externes de la peau pour un teint plus lumineux (AHAs) • Nettoie en profondeur l’intérieur des pores (BHA) • Aide à prévenir la formation de points noirs et de boutons • Redonne de l’éclat et unifie le teint • Hydrate et renforce la résistance de la peau au peeling Conseil d’utilisation : Utiliser uniquement le soir sur une peau propre et sèche, en évitant le contour des yeux. Laisser agir 10 minutes, puis rincer abondamment à l’eau. À appliquer deux fois par semaine, en laissant au moins 3 jours de pause entre chaque usage. Pour des résultats durables, utilisez régulièrement.</t>
+          <t>AHA 10% + BHA 2% + red algae. Peeling visage illuminateur &amp; unifiant le teint Le sérum Deep Peeling exfolie à la fois la surface de la peau et l’intérieur des pores grâce à une combinaison de 10 % d’AHAs (acides alpha-hydroxy : glycolique, lactique, mandélique) et 2 % de BHA (acide salicylique) dans une seule formule. Les AHAs agissent en éliminant les cellules mortes à la surface, tandis que le BHA pénètre profondément pour déboucher les pores et aider à prévenir les points noirs et boutons. Les algues rouges hydratent la peau et aident à accroître sa tolérance au traitement acide, pour un teint plus lisse, net et éclatant.
+Avantages :
+• Exfolie les couches externes de la peau pour un teint plus lumineux (AHAs)
+• Nettoie en profondeur l’intérieur des pores (BHA)
+• Aide à prévenir la formation de points noirs et de boutons
+• Redonne de l’éclat et unifie le teint
+• Hydrate et renforce la résistance de la peau au peeling
+Formule : respectueux des animaux, sans colorant, testé dermatologiquement, sans gluten, sans huile minérale, sans parfum, sans pétrolatum, sans conservateur, sans silicone, vegan, d’origine naturelle.</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
+          <t>Utiliser uniquement le soir sur une peau propre et sèche, en évitant le contour des yeux. Laisser agir 10 minutes, puis rincer abondamment à l’eau. À appliquer deux fois par semaine, en laissant au moins 3 jours de pause entre chaque usage. Pour des résultats durables, utilisez régulièrement.</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Aqua, Pentylene Glycol, Glycerin, Propanediol, Butylene Glycol, Lactic Acid, Gracilaria Verrucosa Extract, Salicylic Acid, Glycolic Acid, Mandelic Acid, Hydroxymethoxyphenyl Decanone, Xanthan Gum, Dipropylene Glycol, Hydroxyacetophenone, Tetrasodium Glutamate Diacetate</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="inlineStr">
+        <is>
           <t>images/8697711602122.jpg</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr">
+      <c r="M22" t="inlineStr">
         <is>
           <t>https://biobalance.tn/serum/42-customizable-mug.html</t>
         </is>
       </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>https://biobalance.tn/serum/42-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="L22" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="M22" t="inlineStr"/>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>https://biobalance.tn/serum/42-customizable-mug.html | https://www.barcodelookup.com/8697711602122</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1795,10 +2093,14 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>ORGANIC ALOE VERA SHAMPOO</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr"/>
+          <t>Organic Aloe Vera Shampoo</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Organic</t>
+        </is>
+      </c>
       <c r="F23" t="inlineStr">
         <is>
           <t>Soins capillaires</t>
@@ -1811,30 +2113,43 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>EXTRAITS D’ALOE VERA BIO &amp; PROVITAMINE B5 330 ml TESTÉ DERMATOLOGIQUEMENT Hydratation intense &amp; soin réparateur pour cheveux secs, cassants et abîmés Ce shampoing à l’aloe vera biologique est spécialement formulé pour hydrater profondément les cheveux et le cuir chevelu, nourrir en douceur, réduire la casse, renforcer la fibre capillaire et apaiser les sensations de sécheresse. Enrichi en provitamine B5, protéines végétales et minéraux bio- fermentés, il aide à restaurer la douceur, la brillance et la résistance des cheveux fragilisés tout en nettoyant sans agresser. Avantages : • Hydrate profondément le cuir chevelu et les cheveux secs • Aide à prévenir la sécheresse, la casse et la fragilité des cheveux • Renforce la fibre capillaire de la racine aux pointes • Scelle l’humidité pour une douceur durable et une brillance naturelle • Aide à réduire les pellicules et apaise le cuir chevelu Conseil d’utilisation : Appliquer sur cheveux mouillés, masser doucement du cuir chevelu jusqu’aux pointes, puis rincer abondamment. Pour de meilleurs résultats, utiliser ensuite avec l’après-shampoing à l’huile d’argan biologique.</t>
+          <t>Extraits d’aloe vera bio &amp; provitamine B5. Hydratation intense &amp; soin réparateur pour cheveux secs, cassants et abîmés Ce shampoing à l’aloe vera biologique est spécialement formulé pour hydrater profondément les cheveux et le cuir chevelu, nourrir en douceur, réduire la casse, renforcer la fibre capillaire et apaiser les sensations de sécheresse. Enrichi en provitamine B5, protéines végétales et minéraux bio- fermentés, il aide à restaurer la douceur, la brillance et la résistance des cheveux fragilisés tout en nettoyant sans agresser.
+Avantages :
+• Hydrate profondément le cuir chevelu et les cheveux secs
+• Aide à prévenir la sécheresse, la casse et la fragilité des cheveux
+• Renforce la fibre capillaire de la racine aux pointes
+• Scelle l’humidité pour une douceur durable et une brillance naturelle
+• Aide à réduire les pellicules et apaise le cuir chevelu
+Formule : respectueux des animaux, sans colorant, testé dermatologiquement, sans gluten, sans huile minérale, sans pétrolatum, sans silicone.</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
+          <t>Appliquer sur cheveux mouillés, masser doucement du cuir chevelu jusqu’aux pointes, puis rincer abondamment. Pour de meilleurs résultats, utiliser ensuite avec l’après-shampoing à l’huile d’argan biologique.</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Aqua, Cocamidopropyl Betaine, Sodium C14-16 Olefin Sulfonate, Sodium Laureth-5 Carboxylate, Coco-Glucoside, Glyceryl Oleate, Decyl Glucoside, Betaine, Aloe Barbadensis Leaf Juice Powder, Glycerin, Hydrolyzed Corn Protein, Hydrolyzed Wheat Protein, Panthenol, Hydrogenated Palm Glycerides Citrate, Tocopherol, Hydrolyzed Soy Protein, Saccharomyces/Zinc Ferment, Saccharomyces/Copper Ferment, Saccharomyces/Magnesium Ferment, Saccharomyces/iron Ferment, Saccharomyces/Silicon Ferment, Leuconostoc/Radish Root Ferment Filtrate, Hexylene Glycol, Saccharum Officinarum Extract, Citrus Limon Fruit Extract, Pyrus Malus Fruit Extract, Camellia Sinensis Leaf Extract, Hexapeptide-11, Allantoin, Centella Asiatica Extract, Hydroxypropyl Guar Hydroxypropyltrimonium Chloride, Polysorbate 20, Tetrasodium Glutamate Diacetate, Sorbitan Caprylate, Propanediol, Parfum, Sodium Benzoate, Potassium Sorbate, Citric Acid, Benzoic Acid. ALCOHOL FREE</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr">
+        <is>
           <t>images/8697711700187.jpg</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr">
+      <c r="M23" t="inlineStr">
         <is>
           <t>https://biobalance.tn/soins-capillaires/50-customizable-mug.html</t>
         </is>
       </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>https://biobalance.tn/soins-capillaires/50-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="L23" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>https://biobalance.tn/soins-capillaires/50-customizable-mug.html | https://www.barcodelookup.com/8697711700187</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1854,10 +2169,14 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>ORGANIC CITRUS SHAMPOO</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr"/>
+          <t>Organic Citrus Shampoo</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Organic</t>
+        </is>
+      </c>
       <c r="F24" t="inlineStr">
         <is>
           <t>Soins capillaires</t>
@@ -1870,30 +2189,44 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>300EXTRAITS D’AGRUMES BIO &amp; COMPLEXE NATUREL MULTI-ACTIF 330 ml TESTÉ DERMATOLOGIQUEMENT Shampoing purifiant pour cuir chevelu gras et cheveux propres plus longtemps Ce shampoing aux extraits d’agrumes biologiques est spécialement formulé pour réguler l’excès de sébum, purifier le cuir chevelu et les cheveux, éliminer les pellicules et apaiser les démangeaisons du cuir chevelu. Grâce à un complexe d’ingrédients naturels, il aide aussi à renforcer les racines, hydrater la fibre capillaire, améliorer l’élasticité, tout en redonnant aux cheveux leur éclat et leur fraîcheur naturelle. Avantages : • Régule l’excès de sébum pour garder les cheveux propres plus longtemps • Purifie le cuir chevelu et les cheveux • Élimine les pellicules et les impuretés • Apaise les démangeaisons du cuir chevelu • Renforce les racines et améliore la résistance des cheveux • Améliore l’éclat, la brillance et la texture générale des cheveux Conseil d’utilisation : Appliquer sur cheveux mouillés, masser doucement jusqu’aux pointes puis rincer abondamment. Pour de meilleurs résultats, utiliser ensuite avec un après-shampoing à l’huile d’argan biologique.</t>
+          <t>Extraits d’agrumes bio &amp; complexe naturel multi-actif. Shampoing purifiant pour cuir chevelu gras et cheveux propres plus longtemps Ce shampoing aux extraits d’agrumes biologiques est spécialement formulé pour réguler l’excès de sébum, purifier le cuir chevelu et les cheveux, éliminer les pellicules et apaiser les démangeaisons du cuir chevelu. Grâce à un complexe d’ingrédients naturels, il aide aussi à renforcer les racines, hydrater la fibre capillaire, améliorer l’élasticité, tout en redonnant aux cheveux leur éclat et leur fraîcheur naturelle.
+Avantages :
+• Régule l’excès de sébum pour garder les cheveux propres plus longtemps
+• Purifie le cuir chevelu et les cheveux
+• Élimine les pellicules et les impuretés
+• Apaise les démangeaisons du cuir chevelu
+• Renforce les racines et améliore la résistance des cheveux
+• Améliore l’éclat, la brillance et la texture générale des cheveux
+Formule : respectueux des animaux, sans colorant, testé dermatologiquement, sans gluten, sans huile minérale, sans pétrolatum, sans silicone.</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
+          <t>Appliquer sur cheveux mouillés, masser doucement jusqu’aux pointes puis rincer abondamment. Pour de meilleurs résultats, utiliser ensuite avec un après-shampoing à l’huile d’argan biologique.</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Aqua, Cocamidopropyl Betaine, Sodium C14-16 Olefin Sulfonate, Sodium Laureth-5 Carboxylate, Decyl Glucoside, Betaine, Citrus Limon Juice, Rosmarinus Officinalis Leaf Extract, Coco-Glucoside, Glyceryl Oleate, Hydrolyzed Corn Protein, Hydrolyzed Wheat Protein, Hydrogenated Palm Glycerides Citrate, Tocopherol, Hexylene Glycol, Saccharum Officinarum Extract, Citrus Limon Fruit Extract, Pyrus Malus Fruit Extract, Camellia Sinensis Leaf Extract, Hexapeptide-11, Glycerin, Panthenol, Allantoin, Centella Asiatica Extract, Hydrolyzed Soy Protein, Saccharomyces/Zinc Ferment, Saccharomyces/Copper Ferment, Saccharomyces/Magnesium Ferment, Saccharomyces/iron Ferment, Saccharomyces/Silicon Ferment, Leuconostoc/Radish Root Ferment Filtrate, Hydroxypropyl Guar Hydroxypropyltrimonium Chloride, Polysorbate 20, Tetrasodium Glutamate Diacetate, Sorbitan Caprylate, Propanediol, Parfum, Sodium Benzoate, Potassium Sorbate, Citric Acid, Benzoic Acid. ALCOHOL FREE</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr">
+        <is>
           <t>images/8697711700170.jpg</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr">
+      <c r="M24" t="inlineStr">
         <is>
           <t>https://biobalance.tn/soins-capillaires/49-customizable-mug.html</t>
         </is>
       </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>https://biobalance.tn/soins-capillaires/49-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="L24" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>https://biobalance.tn/soins-capillaires/49-customizable-mug.html | https://www.barcodelookup.com/8697711700170</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1913,10 +2246,14 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>ORGANIC LAVENDER SHAMPOO</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr"/>
+          <t>Organic Lavender Shampoo</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Organic</t>
+        </is>
+      </c>
       <c r="F25" t="inlineStr">
         <is>
           <t>Soins capillaires</t>
@@ -1929,30 +2266,43 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>EXTRAIT DE LAVANDE BIO, NIACINAMIDE &amp; MINÉRAUX BIO-FERMENTÉS 330 ml TESTÉ DERMATOLOGIQUEMENT Shampoing fortifiant pour cheveux longs, forts et en bonne santé Ce shampoing à la lavande biologique est spécialement formulé pour soutenir une croissance capillaire plus longue, plus forte et plus saine. Il nourrit les cheveux de la racine jusqu’aux pointes, aide à réparer les dommages, améliore la brillance et la flexibilité des fibres capillaires, et réduit les pellicules pour une chevelure éclatante de vitalité et de santé. Avantages : • Favorise une croissance capillaire plus longue et plus forte • Nourrit et renforce les cheveux de la racine aux pointes • Répare les dommages et illumine les cheveux ternes • Améliore la souplesse, la force et la brillance des cheveux • Aide à éliminer les pellicules et purifie le cuir chevelu Conseil d’utilisation : Appliquer sur cheveux mouillés, masser doucement jusqu’aux pointes et rincer abondamment. Pour de meilleurs résultats, utiliser ensuite avec le conditioner à l’huile d’argan biologique Bio Balance.</t>
+          <t>Extrait de lavande bio, niacinamide &amp; minéraux bio-fermentés. Shampoing fortifiant pour cheveux longs, forts et en bonne santé Ce shampoing à la lavande biologique est spécialement formulé pour soutenir une croissance capillaire plus longue, plus forte et plus saine. Il nourrit les cheveux de la racine jusqu’aux pointes, aide à réparer les dommages, améliore la brillance et la flexibilité des fibres capillaires, et réduit les pellicules pour une chevelure éclatante de vitalité et de santé.
+Avantages :
+• Favorise une croissance capillaire plus longue et plus forte
+• Nourrit et renforce les cheveux de la racine aux pointes
+• Répare les dommages et illumine les cheveux ternes
+• Améliore la souplesse, la force et la brillance des cheveux
+• Aide à éliminer les pellicules et purifie le cuir chevelu
+Formule : respectueux des animaux, sans colorant, testé dermatologiquement, sans gluten, sans huile minérale, sans pétrolatum, sans silicone.</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
+          <t>Appliquer sur cheveux mouillés, masser doucement jusqu’aux pointes et rincer abondamment. Pour de meilleurs résultats, utiliser ensuite avec le conditioner à l’huile d’argan biologique Bio Balance.</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Aqua, Cocamidopropyl Betaine, Sodium C14-16 Olefin Sulfonate, Sodium Laureth-5 Carboxylate, Decyl Glucoside, Betaine, Lavandula Angustifolia Flower Extract, Coco-Glucoside, Glyceryl Oleate, Hydrolyzed Corn Protein, Hydrolyzed Wheat Protein, Niacinamide, Hydrolyzed Soy Protein, Saccharomyces/Zinc Ferment, Saccharomyces/Copper Ferment, Saccharomyces/Magnesium Ferment, Saccharomyces/iron Ferment, Saccharomyces/Silicon Ferment, Leuconostoc/Radish Root Ferment Filtrate, Hydrogenated Palm Glycerides Citrate, Tocopherol, Hexylene Glycol, Saccharum Officinarum Extract, Citrus Limon Fruit Extract, Pyrus Malus Fruit Extract, Camellia Sinensis Leaf Extract, Hexapeptide-11, Glycerin, Panthenol, Allantoin, Centella Asiatica Extract, Hydroxypropyl Guar Hydroxypropyltrimonium Chloride, Polysorbate 20, Tetrasodium Glutamate Diacetate, Sorbitan Caprylate, Propanediol, Parfum, Sodium Benzoate, Potassium Sorbate, Citric Acid, Benzoic Acid. ALCOHOL FREE</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr">
+        <is>
           <t>images/8697711700156.jpg</t>
         </is>
       </c>
-      <c r="J25" t="inlineStr">
+      <c r="M25" t="inlineStr">
         <is>
           <t>https://biobalance.tn/soins-capillaires/48-customizable-mug.html</t>
         </is>
       </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>https://biobalance.tn/soins-capillaires/48-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="L25" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>https://biobalance.tn/soins-capillaires/48-customizable-mug.html | https://www.barcodelookup.com/8697711700156</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1972,10 +2322,14 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>ORGANIC POMEGRANATE SHAMPOO</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr"/>
+          <t>Organic Pomegranate Shampoo</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Organic</t>
+        </is>
+      </c>
       <c r="F26" t="inlineStr">
         <is>
           <t>Soins capillaires</t>
@@ -1988,30 +2342,43 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>EXTRAIT DE GRENADE BIO &amp; KÉRATINE VÉGÉTALE 330 ml TESTÉ DERMATOLOGIQUEMENT Soin protecteur pour cheveux colorés, abîmés &amp; fragilisés Ce shampoing à la grenade bio est spécialement formulé pour protéger, réparer et renforcer les cheveux fragilisés, abîmés ou colorés. Sa formule riche en antioxydants aide à préserver la couleur, sceller la brillance et détoxifier le cuir chevelu, tout en renforçant la fibre capillaire contre les agressions du soleil, de la chaleur, des produits chimiques et du coiffage quotidien. Avantages : • Protège et prolonge l’éclat de la couleur des cheveux • Renforce les cheveux fragilisés et abîmés • Répare la fibre capillaire et améliore la résistance • Aide à éliminer les pellicules et purifie le cuir chevelu • Laisse les cheveux plus lisses, brillants et faciles à coiffer Conseil d’utilisation : Appliquer sur cheveux mouillés, masser doucement jusqu’aux pointes et rincer abondamment. Pour de meilleurs résultats, utiliser ensuite avec le conditioner à l’huile d’argan biologique Bio Balance.</t>
+          <t>Extrait de grenade bio &amp; kératine végétale. Soin protecteur pour cheveux colorés, abîmés &amp; fragilisés Ce shampoing à la grenade bio est spécialement formulé pour protéger, réparer et renforcer les cheveux fragilisés, abîmés ou colorés. Sa formule riche en antioxydants aide à préserver la couleur, sceller la brillance et détoxifier le cuir chevelu, tout en renforçant la fibre capillaire contre les agressions du soleil, de la chaleur, des produits chimiques et du coiffage quotidien.
+Avantages :
+• Protège et prolonge l’éclat de la couleur des cheveux
+• Renforce les cheveux fragilisés et abîmés
+• Répare la fibre capillaire et améliore la résistance
+• Aide à éliminer les pellicules et purifie le cuir chevelu
+• Laisse les cheveux plus lisses, brillants et faciles à coiffer
+Formule : respectueux des animaux, sans colorant, testé dermatologiquement, sans gluten, sans huile minérale, sans pétrolatum, sans silicone.</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
+          <t>Appliquer sur cheveux mouillés, masser doucement jusqu’aux pointes et rincer abondamment. Pour de meilleurs résultats, utiliser ensuite avec le conditioner à l’huile d’argan biologique Bio Balance.</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Aqua, Cocamidopropyl Betaine, Sodium C14-16 Olefin Sulfonate, Sodium Laureth-5 Carboxylate, Decyl Glucoside, Betaine, Punica Granatum Fruit Extract, Coco-Glucoside, Glyceryl Oleate, Hydrolyzed Corn Protein, Hydrolyzed Wheat Protein, Hydrolyzed Soy Protein, Saccharomyces/Zinc Ferment, Saccharomyces/Copper Ferment, Saccharomyces/Magnesium Ferment, Saccharomyces/iron Ferment, Saccharomyces/Silicon Ferment, Leuconostoc/Radish Root Ferment Filtrate, Hydrogenated Palm Glycerides Citrate, Tocopherol, Hexylene Glycol, Saccharum Officinarum Extract, Citrus Limon Fruit Extract, Pyrus Malus Fruit Extract, Camellia Sinensis Leaf Extract, Hexapeptide-11, Glycerin, Centella Asiatica Extract, Panthenol, Allantoin, Hydroxypropyl Guar Hydroxypropyltrimonium Chloride, Polysorbate 20, Tetrasodium Glutamate Diacetate, Ethylhexyl Salicylate, Sorbitan Caprylate, Propanediol, Parfum, Citric Acid, Benzoic Acid, Sodium Benzoate, Potassium Sorbate. ALCOHOL FREE</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr">
+        <is>
           <t>images/8697711700163.jpg</t>
         </is>
       </c>
-      <c r="J26" t="inlineStr">
+      <c r="M26" t="inlineStr">
         <is>
           <t>https://biobalance.tn/soins-capillaires/47-customizable-mug.html</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t>https://biobalance.tn/soins-capillaires/47-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="L26" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>https://biobalance.tn/soins-capillaires/47-customizable-mug.html | https://www.barcodelookup.com/8697711700163</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2031,11 +2398,19 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Biobalance Sérum Collagène Marin + Vitamine C 30ml</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr"/>
+          <t>Marine Collagen + Vitamin C Super Serum</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Super Serum</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Sérums</t>
+        </is>
+      </c>
       <c r="G27" t="inlineStr">
         <is>
           <t>30 ml</t>
@@ -2043,30 +2418,37 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Ce sérum à 4,5 % de collagène marin et à 0,5 % de vitamine C agit pour uniformiser le teint et la texture de la peau, augmenter l'élasticité pour une peau plus ferme, laisse le teint doux, lisse et éclatant.</t>
+          <t>Ce sérum à 4,5 % de collagène marin et à 0,5 % de vitamine C agit pour uniformiser le teint et la texture de la peau, augmenter l'élasticité pour une peau plus ferme, laisse le teint doux, lisse et éclatant.
+Formule : respectueux des animaux, sans colorant, testé dermatologiquement, sans gluten, sans huile minérale, sans parfum, sans pétrolatum, sans conservateur, sans silicone.</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
+          <t>Appliquer directement sur le visage nettoyé, matin et soir. Laisser le sérum pénétrer avant d’appliquer la crème hydratante.</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Aqua, Glycerin, Propanediol, Hydrolyzed Collagen, Xanthan Gum, 3-O-Ethyl Ascorbic Acid, Hydroxyacetophenone, Sodium Phytate</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr">
+        <is>
           <t>images/8697711600838.jpg</t>
         </is>
       </c>
-      <c r="J27" t="inlineStr">
+      <c r="M27" t="inlineStr">
         <is>
           <t>https://www.maparatunisie.tn/produit/biobalance-serum-collagene-marin-vitamine-c-30ml/</t>
         </is>
       </c>
-      <c r="K27" t="inlineStr">
-        <is>
-          <t>https://www.maparatunisie.tn/produit/biobalance-serum-collagene-marin-vitamine-c-30ml/</t>
-        </is>
-      </c>
-      <c r="L27" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="M27" t="inlineStr"/>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>https://www.maparatunisie.tn/produit/biobalance-serum-collagene-marin-vitamine-c-30ml/ | https://www.barcodelookup.com/8697711600838</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2086,7 +2468,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>DISCOLORATION FREE LUMISKIN 4% SUPER SERUM</t>
+          <t>Discoloration Free Lumiskin 4% Super Serum</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -2106,30 +2488,43 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Sérum super-éclat anti-taches 30 ml Testé dermatologiquement Sérum avancé conçu pour réduire visiblement l’hyperpigmentation et unifier le teint. Ce traitement ciblé à base de Lumiskin® 4 %, une molécule performante, agit en régulant la production de mélanine pour aider à atténuer les taches brunes, les marques d’acné et les zones de pigmentation irrégulière, tout en restaurer l’éclat naturel et la clarté de la peau. Avantages : • Réduit la quantité de mélanine jusqu’à –70 % • Diminue visiblement l’apparence des taches brunes et empêche leur réapparition • Éclaircit et unifie le teint • Améliore l’éclat et la luminosité de la peau • Convient à tous les types de peau, même sensibles Conseil d’utilisation : Appliquer directement sur une peau propre, matin et soir. Laisser le sérum être absorbé avant d’appliquer votre crème hydratante ou soin quotidien. Il est recommandé d’utiliser une protection solaire haute (SPF 50+) pendant la journée pour optimiser les résultats et aider à prévenir la formation de nouvelles tâches pigmentaires.</t>
+          <t>Sérum super-éclat anti-taches. Sérum avancé conçu pour réduire visiblement l’hyperpigmentation et unifier le teint. Ce traitement ciblé à base de Lumiskin® 4 %, une molécule performante, agit en régulant la production de mélanine pour aider à atténuer les taches brunes, les marques d’acné et les zones de pigmentation irrégulière, tout en restaurer l’éclat naturel et la clarté de la peau.
+Avantages :
+• Réduit la quantité de mélanine jusqu’à –70 %
+• Diminue visiblement l’apparence des taches brunes et empêche leur réapparition
+• Éclaircit et unifie le teint
+• Améliore l’éclat et la luminosité de la peau
+• Convient à tous les types de peau, même sensibles
+Formule : respectueux des animaux, sans colorant, testé dermatologiquement, sans gluten, sans huile minérale, sans parfum, sans pétrolatum, sans conservateur, sans silicone, vegan, d’origine naturelle.</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
+          <t>Appliquer directement sur une peau propre, matin et soir. Laisser le sérum être absorbé avant d’appliquer votre crème hydratante ou soin quotidien. Il est recommandé d’utiliser une protection solaire haute (SPF 50+) pendant la journée pour optimiser les résultats et aider à prévenir la formation de nouvelles tâches pigmentaires.</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>Aqua, Coco-Caprylate/Caprate, Caprylic/Capric Triglyceride, Glyceryl Oleate Citrate, Propanediol, Xanthan Gum, Diacetyl Boldine, Hydroxyacetophenone, Sodium Phytate</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr">
+        <is>
           <t>images/8697711600814.jpg</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr">
+      <c r="M28" t="inlineStr">
         <is>
           <t>https://biobalance.tn/serum/36-customizable-mug.html</t>
         </is>
       </c>
-      <c r="K28" t="inlineStr">
-        <is>
-          <t>https://biobalance.tn/serum/36-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="L28" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="M28" t="inlineStr"/>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>https://biobalance.tn/serum/36-customizable-mug.html | https://www.barcodelookup.com/8697711600814</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2149,7 +2544,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>HYALURONIC 3D HYALURONIC ACID 1% SUPER SERUM</t>
+          <t>Hyaluronic 3D Hyaluronic Acid 1% Super Serum</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -2169,30 +2564,43 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>30 ml Testé dermatologiquement Ce sérum avancé est formulé avec un complexe d’acide hyaluronique multimoléculaire à 1 %, combinant des acides hyaluroniques de faible, moyen et haut poids moléculaire pour une hydratation multi-niveaux qui pénètre toutes les couches de la peau. Cette approche renforce l’hydratation, repulpe la peau et aide à améliorer son apparence générale en ciblant la sécheresse, les ridules et la perte d’élasticité. Avantages : • Hydrate intensément à plusieurs niveaux — de la surface aux couches profondes de la peau • Aide à réduire visiblement l’apparence des ridules et des rides • Améliore la texture, l’élasticité et la fermeté de la peau • Laisse la peau plus souple, rebondie et rafraîchie • Convient à tous les types de peau, y compris sensibles Conseil d’utilisation : Appliquer directement sur le visage propre, matin et soir. Laisser le sérum être absorbé avant d’appliquer votre crème hydratante ou soin quotidien.</t>
+          <t>Ce sérum avancé est formulé avec un complexe d’acide hyaluronique multimoléculaire à 1 %, combinant des acides hyaluroniques de faible, moyen et haut poids moléculaire pour une hydratation multi-niveaux qui pénètre toutes les couches de la peau. Cette approche renforce l’hydratation, repulpe la peau et aide à améliorer son apparence générale en ciblant la sécheresse, les ridules et la perte d’élasticité.
+Avantages :
+• Hydrate intensément à plusieurs niveaux — de la surface aux couches profondes de la peau
+• Aide à réduire visiblement l’apparence des ridules et des rides
+• Améliore la texture, l’élasticité et la fermeté de la peau
+• Laisse la peau plus souple, rebondie et rafraîchie
+• Convient à tous les types de peau, y compris sensibles
+Formule : respectueux des animaux, sans colorant, testé dermatologiquement, sans gluten, sans huile minérale, sans parfum, sans pétrolatum, sans conservateur, sans silicone, vegan, d’origine naturelle.</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
+          <t>Appliquer directement sur le visage propre, matin et soir. Laisser le sérum être absorbé avant d’appliquer votre crème hydratante ou soin quotidien.</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>Aqua, Propanediol, Sodium Hyaluronate, Xanthan Gum, Hydroxyacetophenone, Sodium Phytate</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="inlineStr">
+        <is>
           <t>images/8697711600777.jpg</t>
         </is>
       </c>
-      <c r="J29" t="inlineStr">
+      <c r="M29" t="inlineStr">
         <is>
           <t>https://biobalance.tn/serum/38-customizable-mug.html</t>
         </is>
       </c>
-      <c r="K29" t="inlineStr">
-        <is>
-          <t>https://biobalance.tn/serum/38-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="L29" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="M29" t="inlineStr"/>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>https://biobalance.tn/serum/38-customizable-mug.html | https://www.barcodelookup.com/8697711600777</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2212,7 +2620,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>NIACINAMIDE-G SUPER SERUM</t>
+          <t>Niacinamide-G Super Serum</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -2232,30 +2640,44 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>30 ml Testé dermatologiquement Anti-taches, Anti-rides &amp; Éclaircissant Ce sérum révolutionnaire combine 15 % de niacinamide (vitamine B3) et 5 % d’acide glycolique dans une seule formule pour offrir une solution complète aux problèmes de vieillissement cutané, d’excès de sébum et d’imperfections. Avantages : • Réduit l’apparence des taches brunes et de l’hyperpigmentation • Diminue l’apparence des rides et des ridules • Régule la sécrétion de sébum pour une peau plus équilibrée • Cible les imperfections, les points noirs et les éruptions • Effet exfoliant doux : affine la texture de la peau et resserre l’apparence des pores • Aide à révéler une peau plus claire, lisse et lumineuse Conseil d’utilisation : Utiliser une seule fois par jour, le soir seulement, sur une peau propre. Ne pas rincer. Laisser le sérum être absorbé par la peau avant d’appliquer votre crème hydratante. Si vous avez la peau sensible, utilisez-le 2 à 3 fois par semaine.</t>
+          <t>Anti-taches, Anti-rides &amp; Éclaircissant Ce sérum révolutionnaire combine 15 % de niacinamide (vitamine B3) et 5 % d’acide glycolique dans une seule formule pour offrir une solution complète aux problèmes de vieillissement cutané, d’excès de sébum et d’imperfections.
+Avantages :
+• Réduit l’apparence des taches brunes et de l’hyperpigmentation
+• Diminue l’apparence des rides et des ridules
+• Régule la sécrétion de sébum pour une peau plus équilibrée
+• Cible les imperfections, les points noirs et les éruptions
+• Effet exfoliant doux : affine la texture de la peau et resserre l’apparence des pores
+• Aide à révéler une peau plus claire, lisse et lumineuse
+Formule : respectueux des animaux, sans colorant, testé dermatologiquement, sans gluten, sans huile minérale, sans parfum, sans pétrolatum, sans conservateur, sans silicone, vegan, d’origine naturelle.</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
+          <t>Utiliser une seule fois par jour, le soir seulement, sur une peau propre. Ne pas rincer. Laisser le sérum être absorbé par la peau avant d’appliquer votre crème hydratante. Si vous avez la peau sensible, utilisez-le 2 à 3 fois par semaine.</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Aqua, Niacinamide, Butylene Glycol, Glycerin, Pentylene Glycol, Propanediol, Glycolic Acid, Panthenol, Hydroxyacetophenone, Xanthan Gum, Tetrasodium Glutamate Diacetate</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr"/>
+      <c r="L30" t="inlineStr">
+        <is>
           <t>images/8697711600876.jpg</t>
         </is>
       </c>
-      <c r="J30" t="inlineStr">
+      <c r="M30" t="inlineStr">
         <is>
           <t>https://biobalance.tn/serum/39-customizable-mug.html</t>
         </is>
       </c>
-      <c r="K30" t="inlineStr">
-        <is>
-          <t>https://biobalance.tn/serum/39-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="L30" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="M30" t="inlineStr"/>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>https://biobalance.tn/serum/39-customizable-mug.html | https://www.barcodelookup.com/8697711600876</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2275,7 +2697,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Biobalance Super Serum Advanced Night Recovery 30ml</t>
+          <t>Advanced Night Recovery Super Serum</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -2283,7 +2705,11 @@
           <t>Super Serum</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr"/>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Sérums</t>
+        </is>
+      </c>
       <c r="G31" t="inlineStr">
         <is>
           <t>30 ml</t>
@@ -2296,25 +2722,31 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
+          <t>Appliquer une petite quantité de sérum sur le visage propre et sec, matin et soir, et masser par mouvements circulaires doux jusqu’à absorption.</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>Aqua, Glycerin, Pentylene Glycol, Propanediol, Butylene Glycol, Squalane, Methyl Gluceth-20, Centella Asiatica Extract, Resveratrol, Ceramide NP, 3-O-Ethyl Ascorbic Acid, Sodium Hyaluronate, Inositol, Tocopherol, Beetroot Red, Maltodextrin, Xantha Gum, Hydroxyacetophenone, Tetrasodium Glutamate Diacetate, Citric Acid</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr"/>
+      <c r="L31" t="inlineStr">
+        <is>
           <t>images/8697711602115.jpg</t>
         </is>
       </c>
-      <c r="J31" t="inlineStr">
+      <c r="M31" t="inlineStr">
         <is>
           <t>https://www.maparatunisie.tn/produit/biobalance-super-serum-advanced-night-recovery-30ml/</t>
         </is>
       </c>
-      <c r="K31" t="inlineStr">
-        <is>
-          <t>https://www.maparatunisie.tn/produit/biobalance-super-serum-advanced-night-recovery-30ml/</t>
-        </is>
-      </c>
-      <c r="L31" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="M31" t="inlineStr"/>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>https://www.maparatunisie.tn/produit/biobalance-super-serum-advanced-night-recovery-30ml/ | https://www.barcodelookup.com/8697711602115</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2334,7 +2766,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Super Serum — contour des yeux nuit 20 ml</t>
+          <t>Night Recovery Super Serum Eye Contour</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -2354,30 +2786,40 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Super sérum contour des yeux au phyto-rétinol (bakuchiol), aux céramides et à l’acide hyaluronique, anti-rides et réparateur intense. Appliquer une petite quantité sur peau propre et sèche, autour des yeux, par mouvements circulaires.</t>
+          <t>Super sérum contour des yeux au phyto-rétinol (bakuchiol), aux céramides et à l’acide hyaluronique : anti-rides et réparateur intense.
+Avantages :
+• Réduit les ridules et raffermit le contour des yeux (phyto-rétinol)
+• Renforce la barrière cutanée (céramide NP)
+• Hydrate et revitalise (acide hyaluronique)</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
+          <t>Appliquer une petite quantité sur peau propre et sèche et masser doucement autour des yeux, par mouvements circulaires, jusqu’à absorption, matin et soir.</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>Aqua, Glycerin, Coco-Caprylate/Caprate, Butylene Glycol, Pentylene Glycol, Propanediol, Glyceryl Oleate Citrate, Bakuchiol, Caprylic/Capric Triglyceride, Ceramide NP, Sodium Hyaluronate, Tocopherol, Xanthan Gum, Hydroxyacetophenone, Tetrasodium Glutamate Diacetate</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr"/>
+      <c r="L32" t="inlineStr">
+        <is>
           <t>images/8697711602139.jpg</t>
         </is>
       </c>
-      <c r="J32" t="inlineStr">
+      <c r="M32" t="inlineStr">
         <is>
           <t>https://www.barcodelookup.com/8697711602139</t>
         </is>
       </c>
-      <c r="K32" t="inlineStr">
+      <c r="N32" t="inlineStr">
         <is>
           <t>https://www.barcodelookup.com/8697711602139</t>
         </is>
       </c>
-      <c r="L32" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="M32" t="inlineStr"/>
+      <c r="O32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2397,7 +2839,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>PURE VITAMIN C L-ASCORBIC ACID 10% SUPER SERUM</t>
+          <t>Pure Vitamin C L-Ascorbic Acid 10% Super Serum</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -2417,30 +2859,43 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>30 ml Testé dermatologiquement Sérum concentré à base de 10 % d’acide L-ascorbique (vitamine C pure) formulé sans eau pour une stabilité maximale et une efficacité renforcée. Cette forme stabilisée de vitamine C est un antioxydant puissant qui aide à protéger la peau contre les radicaux libres, stimuler la synthèse du collagène et améliorer l’éclat du teint, tout en contribuant à réduire l’apparence des taches pigmentaires, des rides et des ridules. Avantages : • Protège la peau des dommages causés par les radicaux libres grâce à son action antioxydante • Stimule la synthèse du collagène pour une peau visiblement plus ferme et rebondie • Améliore la clarté du teint et réduit l’apparence des rides • Aide à atténuer les taches brunes et les irrégularités du teint • Formule sans eau, stable et adaptée à tous les types de peau Conseil d’utilisation : Appliquer directement sur le visage propre, matin et soir. Laisser le sérum être absorbé avant d’appliquer votre soin hydratant. Pour de meilleurs résultats, utiliser une protection solaire le matin.</t>
+          <t>Sérum concentré à base de 10 % d’acide L-ascorbique (vitamine C pure) formulé sans eau pour une stabilité maximale et une efficacité renforcée. Cette forme stabilisée de vitamine C est un antioxydant puissant qui aide à protéger la peau contre les radicaux libres, stimuler la synthèse du collagène et améliorer l’éclat du teint, tout en contribuant à réduire l’apparence des taches pigmentaires, des rides et des ridules.
+Avantages :
+• Protège la peau des dommages causés par les radicaux libres grâce à son action antioxydante
+• Stimule la synthèse du collagène pour une peau visiblement plus ferme et rebondie
+• Améliore la clarté du teint et réduit l’apparence des rides
+• Aide à atténuer les taches brunes et les irrégularités du teint
+• Formule sans eau, stable et adaptée à tous les types de peau
+Formule : respectueux des animaux, sans colorant, testé dermatologiquement, sans gluten, sans huile minérale, sans parfum, sans pétrolatum, sans conservateur, sans silicone, vegan, d’origine naturelle.</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
+          <t>Appliquer directement sur le visage propre, matin et soir. Laisser le sérum être absorbé avant d’appliquer votre soin hydratant. Pour de meilleurs résultats, utiliser une protection solaire le matin.</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>Propanediol, Ascorbic Acid</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr"/>
+      <c r="L33" t="inlineStr">
+        <is>
           <t>images/8697711600760.jpg</t>
         </is>
       </c>
-      <c r="J33" t="inlineStr">
+      <c r="M33" t="inlineStr">
         <is>
           <t>https://biobalance.tn/serum/37-customizable-mug.html</t>
         </is>
       </c>
-      <c r="K33" t="inlineStr">
-        <is>
-          <t>https://biobalance.tn/serum/37-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="L33" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="M33" t="inlineStr"/>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>https://biobalance.tn/serum/37-customizable-mug.html | https://www.barcodelookup.com/8697711600760</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2460,7 +2915,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>NATURAL RETINOL’E SUPER SERUM</t>
+          <t>Natural Retinol’e Super Serum</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -2480,30 +2935,44 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>30 ml Testé dermatologiquement Ce sérum avancé associe 0,3 % de rétinol pur et 2 % de vitamine E pour améliorer visiblement la qualité de la peau. Sa formule aide à lisser la surface cutanée, favoriser le renouvellement de la peau et améliorer l’uniformité du teint, tout en apportant nutrition et protection grâce à la vitamine E. Cette combinaison agit efficacement sur les signes de l’âge, la texture irrégulière et le manque d’éclat. Avantages : • Aide à réduire visiblement l’apparence des rides et ridules • Améliore la texture et la fermeté de la peau • Favorise un teint plus uniforme et lumineux • Aide à soutenir le renouvellement cutané • Contribue à nourrir et protéger la peau grâce à la vitamine E • Convient à la plupart des types de peau Conseil d’utilisation : Appliquer le soir sur une peau propre et sèche. Laisser le sérum être absorbé avant d’appliquer votre crème hydratante. Utiliser une protection solaire durant la journée. Commencer par 2 à 3 applications par semaine, puis augmenter progressivement selon la tolérance de la peau.</t>
+          <t>Ce sérum avancé associe 0,3 % de rétinol pur et 2 % de vitamine E pour améliorer visiblement la qualité de la peau. Sa formule aide à lisser la surface cutanée, favoriser le renouvellement de la peau et améliorer l’uniformité du teint, tout en apportant nutrition et protection grâce à la vitamine E. Cette combinaison agit efficacement sur les signes de l’âge, la texture irrégulière et le manque d’éclat.
+Avantages :
+• Aide à réduire visiblement l’apparence des rides et ridules
+• Améliore la texture et la fermeté de la peau
+• Favorise un teint plus uniforme et lumineux
+• Aide à soutenir le renouvellement cutané
+• Contribue à nourrir et protéger la peau grâce à la vitamine E
+• Convient à la plupart des types de peau
+Formule : respectueux des animaux, sans colorant, testé dermatologiquement, sans gluten, sans huile minérale, sans parfum, sans pétrolatum, sans conservateur, sans silicone, vegan, d’origine naturelle.</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
+          <t>Appliquer le soir sur une peau propre et sèche. Laisser le sérum être absorbé avant d’appliquer votre crème hydratante. Utiliser une protection solaire durant la journée. Commencer par 2 à 3 applications par semaine, puis augmenter progressivement selon la tolérance de la peau.</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Coco-Caprylate/Caprate, Squalane, Tocopheryl Acetate, Tocopherol, Helianthus Annuus Seed Oil, Retinol, Bisabolol, Polysorbate 20, BHA, BHT</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr"/>
+      <c r="L34" t="inlineStr">
+        <is>
           <t>images/8697711600852.jpg</t>
         </is>
       </c>
-      <c r="J34" t="inlineStr">
+      <c r="M34" t="inlineStr">
         <is>
           <t>https://biobalance.tn/serum/64-customizable-mug.html</t>
         </is>
       </c>
-      <c r="K34" t="inlineStr">
-        <is>
-          <t>https://biobalance.tn/serum/64-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="L34" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="M34" t="inlineStr"/>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>https://biobalance.tn/serum/64-customizable-mug.html | https://www.barcodelookup.com/8697711600852</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2523,7 +2992,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>CAFFEINE SOLUTION 5% + EGCG + HYALURONIC ACID SUPER SERUM</t>
+          <t>Caffeine Solution 5% + EGCG + Hyaluronic Acid Super Serum</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -2543,30 +3012,43 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>30 ml Testé dermatologiquement Anti-cernes, Anti-poches &amp; Fermeté du contour de l’œil Ce sérum yeux léger est formulé avec 5 % de caféine, EGCG dérivé du thé vert et acide hyaluronique pour revitaliser et éclaircir le contour délicat des yeux. Il aide à réduire l’apparence des cernes, atténuer les poches, hydrater intensément et améliorer l’élasticité de la peau autour du regard. Avantages : • Éclaircit visiblement le contour des yeux • Hydrate intensément et repulpe la peau • Contribue à raffermir la zone fragile du regard • Réduit l’apparence des poches et signes de fatigue • Améliore l’élasticité et l’apparence générale de la peau autour des yeux Conseil d’utilisation : Appliquer matin et soir sur le contour des yeux propre et sec en mouvements circulaires doux. Laisser le sérum être absorbé avant d’appliquer votre soin hydratant.</t>
+          <t>Anti-cernes, Anti-poches &amp; Fermeté du contour de l’œil Ce sérum yeux léger est formulé avec 5 % de caféine, EGCG dérivé du thé vert et acide hyaluronique pour revitaliser et éclaircir le contour délicat des yeux. Il aide à réduire l’apparence des cernes, atténuer les poches, hydrater intensément et améliorer l’élasticité de la peau autour du regard.
+Avantages :
+• Éclaircit visiblement le contour des yeux
+• Hydrate intensément et repulpe la peau
+• Contribue à raffermir la zone fragile du regard
+• Réduit l’apparence des poches et signes de fatigue
+• Améliore l’élasticité et l’apparence générale de la peau autour des yeux
+Formule : respectueux des animaux, sans colorant, testé dermatologiquement, sans gluten, sans huile minérale, sans parfum, sans pétrolatum, sans conservateur, sans silicone, vegan, d’origine naturelle.</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
+          <t>Appliquer matin et soir sur le contour des yeux propre et sec en mouvements circulaires doux. Laisser le sérum être absorbé avant d’appliquer votre soin hydratant.</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Aqua, Caffeine, Glycerin, Propanediol, Butylene Glycol, Pentylene Glycol, Epigallocatechin Gallatyl Glucoside, Hydroxyacetophenone, Sodium Hyaluronate, Xanthan Gum, Hydroxyethylcellulose, Tetrasodium Glutamate Diacetate</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr"/>
+      <c r="L35" t="inlineStr">
+        <is>
           <t>images/8697711600890.jpg</t>
         </is>
       </c>
-      <c r="J35" t="inlineStr">
+      <c r="M35" t="inlineStr">
         <is>
           <t>https://biobalance.tn/serum/41-customizable-mug.html</t>
         </is>
       </c>
-      <c r="K35" t="inlineStr">
-        <is>
-          <t>https://biobalance.tn/serum/41-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="L35" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="M35" t="inlineStr"/>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>https://biobalance.tn/serum/41-customizable-mug.html | https://www.barcodelookup.com/8697711600890</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2589,39 +3071,60 @@
           <t>Super Glow Gel Cream Moisturizer</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr"/>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Super Cream</t>
+        </is>
+      </c>
       <c r="F36" t="inlineStr">
         <is>
           <t>Crèmes visage</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr"/>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>50 ml</t>
+        </is>
+      </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Enrichie en vitamine C stabilisée (3-O-Ethyl Ascorbic Acid) et en acide férulique, cette gel-crème illumine le teint, unifie la peau et aide à lutter contre les signes visibles du vieillissement, tout en protégeant la peau des agressions extérieures. Avantages : • Illumine et ravive l’éclat du teint • Aide à atténuer l’apparence des taches pigmentaires • Unifie le teint et améliore la luminosité • Protège la peau grâce à une action antioxydante • Texture légère, rapidement absorbée Conseil d’utilisation : Appliquer deux fois par jour, matin et soir, sur le visage et le cou, sur une peau propre.</t>
+          <t>Enrichie en vitamine C stabilisée (3-O-Ethyl Ascorbic Acid) et en acide férulique, cette gel-crème illumine le teint, unifie la peau et aide à lutter contre les signes visibles du vieillissement, tout en protégeant la peau des agressions extérieures.
+Avantages :
+• Illumine et ravive l’éclat du teint
+• Aide à atténuer l’apparence des taches pigmentaires
+• Unifie le teint et améliore la luminosité
+• Protège la peau grâce à une action antioxydante
+• Texture légère, rapidement absorbée
+Formule : respectueux des animaux, sans colorant, testé dermatologiquement, sans gluten, sans huile minérale, sans parfum, sans pétrolatum, sans silicone, vegan, d’origine naturelle.</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
+          <t>Appliquer deux fois par jour, matin et soir, sur le visage et le cou, sur une peau propre.</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>Aqua, Glycerin, Caprylic/Capric Triglyceride, Coco-Caprylate/Caprate, Glyceryl Stearate, 3-O-Ethyl Ascorbic Acid, Butylene Glycol, Cetearyl Alcohol, Polyglyceryl-6 Palmitate/Succinate, Ferulic Acid, Acacia Senegal Gum, Xanthan Gum, Tocopherol, Tetrasodium Glutamate Diacetate, Sorbitan Caprylate, Propanediol, Benzoic Acid. ALCOHOL FREE</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr"/>
+      <c r="L36" t="inlineStr">
+        <is>
           <t>images/8697711602023.jpg</t>
         </is>
       </c>
-      <c r="J36" t="inlineStr">
+      <c r="M36" t="inlineStr">
         <is>
           <t>https://biobalance.tn/supercreams-/29-customizable-mug.html</t>
         </is>
       </c>
-      <c r="K36" t="inlineStr">
-        <is>
-          <t>https://biobalance.tn/supercreams-/29-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="L36" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="M36" t="inlineStr"/>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>https://biobalance.tn/supercreams-/29-customizable-mug.html | https://www.barcodelookup.com/8697711602023</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2641,42 +3144,63 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>SUPER HYDRATOR CREAM MOISTURIZER</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr"/>
+          <t>Super Hydrator Cream Moisturizer</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Super Cream</t>
+        </is>
+      </c>
       <c r="F37" t="inlineStr">
         <is>
           <t>Crèmes visage</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr"/>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>50 ml</t>
+        </is>
+      </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Testé dermatologiquement Cette crème hydratante avancée est formulée avec Céramide NP et Vitamine F, une combinaison essentielle qui aide à renforcer la barrière naturelle d’hydratation de la peau et à prévenir la perte d’eau. Sa texture légère pénètre rapidement pour offrir une hydratation profonde, apaiser la peau et améliorer son équilibre naturel. Avantages : • Hydrate intensément et durablement la peau • Renforce la barrière cutanée et limite la déshydratation • Apaise et améliore l’élasticité de la peau • Laisse la peau douce, lisse et équilibrée • Idéale pour les peaux sèches, très sèches et sensibles Conseil d’utilisation : Appliquer sur le visage propre, matin et soir. Masser doucement jusqu’à absorption complète avant d’appliquer votre routine quotidienne..</t>
+          <t>Cette crème hydratante avancée est formulée avec Céramide NP et Vitamine F, une combinaison essentielle qui aide à renforcer la barrière naturelle d’hydratation de la peau et à prévenir la perte d’eau. Sa texture légère pénètre rapidement pour offrir une hydratation profonde, apaiser la peau et améliorer son équilibre naturel.
+Avantages :
+• Hydrate intensément et durablement la peau
+• Renforce la barrière cutanée et limite la déshydratation
+• Apaise et améliore l’élasticité de la peau
+• Laisse la peau douce, lisse et équilibrée
+• Idéale pour les peaux sèches, très sèches et sensibles
+Formule : respectueux des animaux, sans colorant, testé dermatologiquement, sans gluten, sans huile minérale, sans parfum, sans pétrolatum, sans silicone, vegan, d’origine naturelle.</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
+          <t>Appliquer sur le visage propre, matin et soir. Masser doucement jusqu’à absorption complète avant d’appliquer votre routine quotidienne..</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>Aqua, Glycerin, Caprylic/Capric Triglyceride, Coco-Caprylate/Caprate, Glyceryl Stearate, Butylene Glycol, Cetearyl Alcohol, Polyglyceryl-6 Palmitate/Succinate, Ceramide NP, Linoleic Acid, Linolenic Acid, Acacia Senegal Gum, Xanthan Gum, Tocopherol, Tetrasodium Glutamate Diacetate, Sorbitan Caprylate, Propanediol, Benzoic Acid. ALCOHOL FREE</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr"/>
+      <c r="L37" t="inlineStr">
+        <is>
           <t>images/8697711602054.jpg</t>
         </is>
       </c>
-      <c r="J37" t="inlineStr">
+      <c r="M37" t="inlineStr">
         <is>
           <t>https://biobalance.tn/supercreams-/65-customizable-mug.html</t>
         </is>
       </c>
-      <c r="K37" t="inlineStr">
-        <is>
-          <t>https://biobalance.tn/supercreams-/65-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="L37" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="M37" t="inlineStr"/>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>https://biobalance.tn/supercreams-/65-customizable-mug.html | https://www.barcodelookup.com/8697711602054</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2699,39 +3223,60 @@
           <t>Super Lift Cream Moisturizer</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr"/>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Super Cream</t>
+        </is>
+      </c>
       <c r="F38" t="inlineStr">
         <is>
           <t>Crèmes visage</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr"/>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>50 ml</t>
+        </is>
+      </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Le Phyto-Retinol (Bakuchiol) associé à la L-Carnosine agit de manière multifonctionnelle pour cibler les signes visibles du vieillissement cutané, améliorer la fermeté de la peau et renforcer sa structure. Avantages : • Raffermit la peau et améliore l’élasticité • Réduit l’apparence des rides et ridules • Stimule la production de collagène • Protège contre le vieillissement induit par la lumière bleue • Aide à uniformiser le teint et à atténuer les taches pigmentaires Conseil d’utilisation : Appliquer deux fois par jour, matin et soir, sur le visage et le cou.</t>
+          <t>Le Phyto-Retinol (Bakuchiol) associé à la L-Carnosine agit de manière multifonctionnelle pour cibler les signes visibles du vieillissement cutané, améliorer la fermeté de la peau et renforcer sa structure.
+Avantages :
+• Raffermit la peau et améliore l’élasticité
+• Réduit l’apparence des rides et ridules
+• Stimule la production de collagène
+• Protège contre le vieillissement induit par la lumière bleue
+• Aide à uniformiser le teint et à atténuer les taches pigmentaires
+Formule : respectueux des animaux, sans colorant, testé dermatologiquement, sans gluten, sans huile minérale, sans parfum, sans pétrolatum, sans silicone, vegan, d’origine naturelle.</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
+          <t>Appliquer deux fois par jour, matin et soir, sur le visage et le cou.</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>Aqua, Glycerin, Caprylic/Capric Triglyceride, Coco-Caprylate/Caprate, Glyceryl Stearate, Butylene Glycol, Cetearyl Alcohol, Polyglyceryl-6 Palmitate/Succinate, Bakuchiol, Carnosine, Tocopherol, Xanthan Gum, Tetrasodium Glutamate Diacetate, Sorbitan Caprylate, Propanediol, Benzoic Acid. ALCOHOL FREE</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr"/>
+      <c r="L38" t="inlineStr">
+        <is>
           <t>images/8697711602047.jpg</t>
         </is>
       </c>
-      <c r="J38" t="inlineStr">
+      <c r="M38" t="inlineStr">
         <is>
           <t>https://biobalance.tn/super-lift/30-customizable-mug.html</t>
         </is>
       </c>
-      <c r="K38" t="inlineStr">
-        <is>
-          <t>https://biobalance.tn/super-lift/30-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="L38" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="M38" t="inlineStr"/>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>https://biobalance.tn/super-lift/30-customizable-mug.html | https://www.barcodelookup.com/8697711602047</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2751,7 +3296,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>GLOW SKIN C SUPER TONER</t>
+          <t>Glow Skin C Super Toner</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -2764,33 +3309,48 @@
           <t>Nettoyants visage</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr"/>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>250 ml</t>
+        </is>
+      </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>ETHYL ASCORBIC ACID – EXTRAit DE RACINE DE RÉGLISSE – ACIDE HYALURONIQUE 96 % d’origine naturelle 250 ml TESTÉ DERMATOLOGIQUEMENT Éclaircissant parfait – Anti-taches – Anti-rides Les lotions toniques éliminent visiblement les dernières traces de maquillage, laissant la peau exceptionnellement propre, fraîche et adoucie. Avantages : • Lisse, adoucit et revitalise instantanément la peau • llumine et restaure l’éclat pour un teint radieux • Hydrate et équilibre la peau Conseil d’utilisation : Appliquer à l’aide d’un coton après avoir nettoyé la peau. Essuyer avec des mouvements du centre du visage vers l’extérieur jusqu’à ce que le coton soit propre.</t>
+          <t>Ethyl ascorbic acid – extrait de racine de réglisse – acide hyaluronique 96 % d’origine naturelle. Éclaircissant parfait – Anti-taches – Anti-rides Les lotions toniques éliminent visiblement les dernières traces de maquillage, laissant la peau exceptionnellement propre, fraîche et adoucie.
+Avantages :
+• Lisse, adoucit et revitalise instantanément la peau
+• llumine et restaure l’éclat pour un teint radieux
+• Hydrate et équilibre la peau
+Formule : respectueux des animaux, sans colorant, testé dermatologiquement, sans gluten, sans huile minérale, sans parfum, sans pétrolatum, sans conservateur, sans silicone, vegan, d’origine naturelle.</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
+          <t>Appliquer à l’aide d’un coton après avoir nettoyé la peau. Essuyer avec des mouvements du centre du visage vers l’extérieur jusqu’à ce que le coton soit propre.</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>Aqua, Butylene Glycol, Glycerin, Propanediol, Pentylene Glycol, Polyglyceryl-4 Laurate/Sebacate, Polyglyceryl-6 Caprylate/Caprate, 3-O-Ethyl Ascorbic Acid, Glycyrrhiza Glabra Root Extract, Sodium Hyaluronate, Xanthan Gum, Tetrasodium Glutamate Diacetate, Hydroxyacetophenone. ALCOHOL FREE</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr"/>
+      <c r="L39" t="inlineStr">
+        <is>
           <t>images/8697711602313.jpg</t>
         </is>
       </c>
-      <c r="J39" t="inlineStr">
+      <c r="M39" t="inlineStr">
         <is>
           <t>https://biobalance.tn/nettoyants-visage/43-customizable-mug.html</t>
         </is>
       </c>
-      <c r="K39" t="inlineStr">
-        <is>
-          <t>https://biobalance.tn/nettoyants-visage/43-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="L39" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="M39" t="inlineStr"/>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>https://biobalance.tn/nettoyants-visage/43-customizable-mug.html | https://www.barcodelookup.com/8697711602313</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2810,7 +3370,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>PORE TIGHT SUPER TONER</t>
+          <t>Pore Tight Super Toner</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -2830,30 +3390,43 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>LACTIC ACID 7% – AHA + BHA + PHA – TEA TREE OIL 88 % d’origine naturelle 250 ml TESTÉ DERMATOLOGIQUEMENT Anti-acné, Anti-points noirs – Uniformise le teint – Minimise les pores Ce tonique à action multiple est formulé pour cibler les imperfections, les points noirs, les pores dilatés et le teint irrégulier en une seule étape. Enrichi en acide lactique (7 %), un AHA doux mais efficace, et combiné à un complexe d’exfoliation AHA + BHA + PHA, il aide à éliminer les cellules mortes, nettoyer les pores en profondeur et stimuler le renouvellement cellulaire. L’huile d’arbre à thé purifiante contribue à réduire l’excès de sébum et à calmer les zones sujettes aux imperfections, laissant la peau propre, rafraîchie et lisse. Avantages : • Élimine les dernières traces de maquillage et l’excès de sébum • Exfolie en douceur la peau pour un teint plus net • Aide à prévenir les points noirs et boutons • Minimise visiblement l’apparence des pores dilatés • Laisse la peau rafraîchie, plus lisse et équilibrée Conseil d’utilisation : Appliquer le soir à l’aide d’un coton après avoir nettoyé la peau. Essuyer délicatement le visage du centre vers l’extérieur jusqu’à ce que le coton soit propre. Ne pas rincer.</t>
+          <t>Lactic acid 7% – AHA + BHA + PHA – tea tree oil 88 % d’origine naturelle. Anti-acné, Anti-points noirs – Uniformise le teint – Minimise les pores Ce tonique à action multiple est formulé pour cibler les imperfections, les points noirs, les pores dilatés et le teint irrégulier en une seule étape. Enrichi en acide lactique (7 %), un AHA doux mais efficace, et combiné à un complexe d’exfoliation AHA + BHA + PHA, il aide à éliminer les cellules mortes, nettoyer les pores en profondeur et stimuler le renouvellement cellulaire. L’huile d’arbre à thé purifiante contribue à réduire l’excès de sébum et à calmer les zones sujettes aux imperfections, laissant la peau propre, rafraîchie et lisse.
+Avantages :
+• Élimine les dernières traces de maquillage et l’excès de sébum
+• Exfolie en douceur la peau pour un teint plus net
+• Aide à prévenir les points noirs et boutons
+• Minimise visiblement l’apparence des pores dilatés
+• Laisse la peau rafraîchie, plus lisse et équilibrée
+Formule : respectueux des animaux, sans colorant, testé dermatologiquement, sans gluten, sans huile minérale, sans parfum, sans pétrolatum, sans conservateur, sans silicone, vegan, d’origine naturelle.</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
+          <t>Appliquer le soir à l’aide d’un coton après avoir nettoyé la peau. Essuyer délicatement le visage du centre vers l’extérieur jusqu’à ce que le coton soit propre. Ne pas rincer.</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>Aqua, Butylene Glycol, Glycerin, Lactic Acid, Pentylene Glycol, Propanediol, Glycolic Acid, Salicylic Acid, Polyglyceryl-4 Laurate/Sebacate, Polyglyceryl-6 Caprylate/Caprate, Melaleuca Alternifolia Leaf Oil, Gluconolactone, Mandelic Acid, Vaccinium Myrtillus Fruit/Leaf Extract, Saccharum Officinarum Extract, Citrus Aurantium Dulcis Fruit Extract, Citrus Limon Fruit Extract, Acer Saccharum Extract, Sodium Hyaluronate, Xanthan Gum, Tetrasodium Glutamate Diacetate, Hydroxyacetophenone. ALCOHOL FREE</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr"/>
+      <c r="L40" t="inlineStr">
+        <is>
           <t>images/8697711602337.jpg</t>
         </is>
       </c>
-      <c r="J40" t="inlineStr">
+      <c r="M40" t="inlineStr">
         <is>
           <t>https://biobalance.tn/nettoyants-visage/44-customizable-mug.html</t>
         </is>
       </c>
-      <c r="K40" t="inlineStr">
-        <is>
-          <t>https://biobalance.tn/nettoyants-visage/44-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="L40" t="inlineStr">
-        <is>
-          <t>complet</t>
-        </is>
-      </c>
-      <c r="M40" t="inlineStr"/>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>https://biobalance.tn/nettoyants-visage/44-customizable-mug.html | https://www.barcodelookup.com/8697711602337</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
12 biobalance.tn products back in the catalog with their barcodes; test data purged
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/initial-catalog/produits.xlsx
+++ b/data/initial-catalog/produits.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O40"/>
+  <dimension ref="A1:O52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1210,7 +1210,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Un soin quotidien contre les problèmes de peau grasse Effet « Soft Peeling » La formule sans savon et sans huile nettoie en douceur et en profondeur les pores en éliminant saletés, impuretés et maquillage. La mousse légère se rince facilement, sans laisser de résidus pouvant obstruer les pores. Personnalisation N'oubliez pas de sauvegarder votre personnalisation pour pouvoir l'ajouter au panier Insérer votre texte ici 250 caractères max Enregistrer la personnalisation
+          <t>Un soin quotidien contre les problèmes de peau grasse Effet « Soft Peeling » La formule sans savon et sans huile nettoie en douceur et en profondeur les pores en éliminant saletés, impuretés et maquillage. La mousse légère se rince facilement, sans laisser de résidus pouvant obstruer les pores. Personnalisation N'oubliez pas de sauvegarder votre personnalisation pour pouvoir l'ajouter au panier Insérer votre texte ici 250 caractères max Enregistrer la personnalisation.
 Formule : respectueux des animaux, sans colorant, testé dermatologiquement, sans gluten, sans pétrolatum, sans silicone.</t>
         </is>
       </c>
@@ -1281,8 +1281,7 @@
       <c r="H12" t="inlineStr">
         <is>
           <t>Un soin apaisant qui respecte les peaux sensibles. Effet « Soft Peeling » La formule sans savon et sans huile nettoie la peau en douceur et élimine saletés, impuretés et maquillage. La mousse légère se rince facilement, sans laisser de résidus pouvant obstruer les pores.
-Avantages :
-• Améliore la fonction naturelle de la barrière cutanée et réduit les rougeurs, les picotements et la sensibilité. INGRÉDIENTS : Bisabolol Complexe d’Acides Aminés Renforce la résistance et la tolérance de la peau face aux agressions extérieures irritantes responsables de rougeurs, tiraillements et sensations de picotement. Glycérine, Aloe Vera, Allantoïne, Panthénol et Vitamine E Améliorent la barrière naturelle de la peau, préviennent la perte d’hydratation et aident à maintenir une peau bien hydratée.
+Améliore la fonction naturelle de la barrière cutanée et réduit les rougeurs, les picotements et la sensibilité. INGRÉDIENTS : Bisabolol Complexe d’Acides Aminés Renforce la résistance et la tolérance de la peau face aux agressions extérieures irritantes responsables de rougeurs, tiraillements et sensations de picotement. Glycérine, Aloe Vera, Allantoïne, Panthénol et Vitamine E Améliorent la barrière naturelle de la peau, préviennent la perte d’hydratation et aident à maintenir une peau bien hydratée.
 Formule : respectueux des animaux, sans colorant, testé dermatologiquement, sans gluten, sans pétrolatum, sans silicone.</t>
         </is>
       </c>
@@ -3428,6 +3427,850 @@
       </c>
       <c r="O40" t="inlineStr"/>
     </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>8697711011122</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>BB-WEB-52</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Repulpeur Lèvres Hot Chocolate N°03</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Repulpeur Lèvres Hot Chocolate N°03</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>LipojeN</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Maquillage</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>5 ml</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Le Repulpeur lèvres Hot Chocolate est le secret des lèvres pulpeuses, lisses et parfaitement hydratées.
+Grâce à sa formule exclusive combinant des tripeptides repulpants, de l’acide hyaluronique et un extrait de gingembre, il repulpe intensément, lisse les ridules et hydrate en profondeur, tout en offrant une couleur intense et brillante qui révèle toute votre féminité et votre sensualité dès le premier passage. Une alternative naturelle et douce aux injections d’acide hyaluronique, à utiliser quotidiennement comme un rouge à lèvres, avec une protection solaire contre les rayons UVA et UVB.</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Pour profiter pleinement des bienfaits des repulpeurs lèvres LipojeN, voici quelques conseils d’utilisation bien utiles : Assurez-vous que vos lèvres soient propres et sèches avant l’application. Appliquez le rouge à lèvres LipojeN au moins 3 fois par jour pendant 30 jours pour obtenir de bons résultats . Les jours où vous ne souhaitez pas vous maquiller, il est possible d’appliquer le Glossy crystal clear numéro 01 pour ne pas interrompre le traitement. N’hésitez pas à renouveler l’application aussi souvent que souhaité pour maintenir l’hydratation et l’apparence pulpeuse de vos lèvres. Nous recommandons d’effectuer un léger gommage des lèvres 1 à 2 fois par semaine. Cela permet d’éliminer les peaux mortes et favorise une meilleure absorption du produit. Une réelle alternative, douce et naturelle, aux injections d’acide hyaluronique !</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>DIMETHICONE, DICAPRYLYL CARBONATE, QUATERIUM-90 SEPIOLITE, ISONONYL ISONONANOATE, TRIMETHYLSILOXYSILICATE, QUATERIUM-90 MONTMORILLONITE, ISOPROPYL MYRISTATE, ETHYLHEXYL PALMITATE, TRIBEHENIN, SORBITAN ISOSTEARATE, PALMITOYL TRIPEPTIDE-1, LACTIC ACID, BHT, ETHYLHEXYL METHOXYCINNAMATE, CAPRYLYL GLYCOL, BUTYROSPERMUM PARKII BUTTER, CAMELLIA JAPONICA SEED OIL, TOCOPHERYL ACETATE, TOCOPHEROL, ISOPROPYL TITANIUM TRIISOSTEARATE, POLYHYDROXYSTEARIC ACID, STEARALKONIUM HECTORITE, PROPYLENE CARBONATE, AROMA, [ +/- MAY CONTAIN CI 77891 /TITANIUM DIOXIDE, CI 15880 /RED 63: 1, CI 17200 /RED 33, CI 15850 /RED 57, CI 15850 /RED 57: 1, CI 77491, CI 77492, CI 77499 /IRON OXIDES]</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr"/>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>images/8697711011122.jpg</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>https://biobalance.tn/maquillage/52-customizable-mug.html</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>https://biobalance.tn/maquillage/52-customizable-mug.html | https://www.barcodelookup.com/8697711011122</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>8697711011139</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>BB-WEB-54</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Repulpeur Lèvres Rose Venus N°04</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Repulpeur Lèvres Rose Venus N°04</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>LipojeN</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Maquillage</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>5 ml</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Le Repulpeur lèvres Rose Venus est le secret des lèvres pulpeuses, lisses et parfaitement hydratées.
+Grâce à sa formule exclusive combinant des tripeptides repulpants, de l’acide hyaluronique et un extrait de gingembre, il repulpe intensément, lisse les ridules et hydrate en profondeur, tout en offrant une couleur intense et brillante qui révèle toute votre féminité et votre sensualité dès le premier passage. Une alternative naturelle et douce aux injections d’acide hyaluronique, à utiliser quotidiennement comme un rouge à lèvres, avec une protection solaire contre les rayons UVA et UVB.</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Pour profiter pleinement des bienfaits des repulpeurs lèvres LipojeN, voici quelques conseils d’utilisation bien utiles : Assurez-vous que vos lèvres soient propres et sèches avant l’application. Appliquez le rouge à lèvres LipojeN au moins 3 fois par jour pendant 30 jours pour obtenir de bons résultats . Les jours où vous ne souhaitez pas vous maquiller, il est possible d’appliquer le Glossy crystal clear numéro 01 pour ne pas interrompre le traitement. N’hésitez pas à renouveler l’application aussi souvent que souhaité pour maintenir l’hydratation et l’apparence pulpeuse de vos lèvres. Nous recommandons d’effectuer un léger gommage des lèvres 1 à 2 fois par semaine. Cela permet d’éliminer les peaux mortes et favorise une meilleure absorption du produit. Une réelle alternative, douce et naturelle, aux injections d’acide hyaluronique !</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>DIMETHICONE, DICAPRYLYL CARBONATE, QUATERIUM-90 SEPIOLITE, ISONONYL ISONONANOATE, TRIMETHYLSILOXYSILICATE, QUATERIUM-90 MONTMORILLONITE, ISOPROPYL MYRISTATE, ETHYLHEXYL PALMITATE, TRIBEHENIN, SORBITAN ISOSTEARATE, PALMITOYL TRIPEPTIDE-1, LACTIC ACID, BHT, ETHYLHEXYL METHOXYCINNAMATE, CAPRYLYL GLYCOL, BUTYROSPERMUM PARKII BUTTER, CAMELLIA JAPONICA SEED OIL, TOCOPHERYL ACETATE, TOCOPHEROL, ISOPROPYL TITANIUM TRIISOSTEARATE, POLYHYDROXYSTEARIC ACID, STEARALKONIUM HECTORITE, PROPYLENE CARBONATE, AROMA, [ +/- MAY CONTAIN CI 77891 /TITANIUM DIOXIDE, CI 15880 /RED 63: 1, CI 17200 /RED 33, CI 15850 /RED 57, CI 15850 /RED 57: 1, CI 77491, CI 77492, CI 77499 /IRON OXIDES]</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr"/>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>images/8697711011139.jpg</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>https://biobalance.tn/maquillage/54-customizable-mug.html</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>https://biobalance.tn/maquillage/54-customizable-mug.html | https://www.barcodelookup.com/8697711011139</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>8697711011146</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>BB-WEB-55</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Repulpeur Lèvres Rosy Petal N°05</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Repulpeur Lèvres Rosy Petal N°05</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>LipojeN</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Maquillage</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>5 ml</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Le Repulpeur lèvres Rosy Petal est le secret des lèvres pulpeuses, lisses et parfaitement hydratées.
+Grâce à sa formule exclusive combinant des tripeptides repulpants, de l’acide hyaluronique et un extrait de gingembre, il repulpe intensément, lisse les ridules et hydrate en profondeur, tout en offrant une couleur intense et brillante qui révèle toute votre féminité et votre sensualité dès le premier passage. Une alternative naturelle et douce aux injections d’acide hyaluronique, à utiliser quotidiennement comme un rouge à lèvres, avec une protection solaire contre les rayons UVA et UVB.</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Pour profiter pleinement des bienfaits des repulpeurs lèvres LipojeN, voici quelques conseils d’utilisation bien utiles : Assurez-vous que vos lèvres soient propres et sèches avant l’application. Appliquez le rouge à lèvres LipojeN au moins 3 fois par jour pendant 30 jours pour obtenir de bons résultats . Les jours où vous ne souhaitez pas vous maquiller, il est possible d’appliquer le Glossy crystal clear numéro 01 pour ne pas interrompre le traitement. N’hésitez pas à renouveler l’application aussi souvent que souhaité pour maintenir l’hydratation et l’apparence pulpeuse de vos lèvres. Nous recommandons d’effectuer un léger gommage des lèvres 1 à 2 fois par semaine. Cela permet d’éliminer les peaux mortes et favorise une meilleure absorption du produit. Une réelle alternative, douce et naturelle, aux injections d’acide hyaluronique !</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>DIMETHICONE, DICAPRYLYL CARBONATE, QUATERIUM-90 SEPIOLITE, ISONONYL ISONONANOATE, TRIMETHYLSILOXYSILICATE, QUATERIUM-90 MONTMORILLONITE, ISOPROPYL MYRISTATE, ETHYLHEXYL PALMITATE, TRIBEHENIN, SORBITAN ISOSTEARATE, PALMITOYL TRIPEPTIDE-1, LACTIC ACID, BHT, ETHYLHEXYL METHOXYCINNAMATE, CAPRYLYL GLYCOL, BUTYROSPERMUM PARKII BUTTER, CAMELLIA JAPONICA SEED OIL, TOCOPHERYL ACETATE, TOCOPHEROL, ISOPROPYL TITANIUM TRIISOSTEARATE, POLYHYDROXYSTEARIC ACID, STEARALKONIUM HECTORITE, PROPYLENE CARBONATE, AROMA, [ +/- MAY CONTAIN CI 77891 /TITANIUM DIOXIDE, CI 15880 /RED 63: 1, CI 17200 /RED 33, CI 15850 /RED 57, CI 15850 /RED 57: 1, CI 77491, CI 77492, CI 77499 /IRON OXIDES]</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr"/>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>images/8697711011146.jpg</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>https://biobalance.tn/maquillage/55-customizable-mug.html</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>https://biobalance.tn/maquillage/55-customizable-mug.html | https://www.barcodelookup.com/8697711011146</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>8697711011160</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>BB-WEB-56</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Repulpeur Lèvres High Society N°07</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Repulpeur Lèvres High Society N°07</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>LipojeN</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Maquillage</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>5 ml</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Le Repulpeur lèvres High Society est le secret des lèvres pulpeuses, lisses et parfaitement hydratées.
+Grâce à sa formule exclusive combinant des tripeptides repulpants, de l’acide hyaluronique et un extrait de gingembre, il repulpe intensément, lisse les ridules et hydrate en profondeur, tout en offrant une couleur intense et brillante qui révèle toute votre féminité et votre sensualité dès le premier passage. Une alternative naturelle et douce aux injections d’acide hyaluronique, à utiliser quotidiennement comme un rouge à lèvres, avec une protection solaire contre les rayons UVA et UVB.</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Pour profiter pleinement des bienfaits des repulpeurs lèvres LipojeN, voici quelques conseils d’utilisation bien utiles : Assurez-vous que vos lèvres soient propres et sèches avant l’application. Appliquez le rouge à lèvres LipojeN au moins 3 fois par jour pendant 30 jours pour obtenir de bons résultats . Les jours où vous ne souhaitez pas vous maquiller, il est possible d’appliquer le Glossy crystal clear numéro 01 pour ne pas interrompre le traitement. N’hésitez pas à renouveler l’application aussi souvent que souhaité pour maintenir l’hydratation et l’apparence pulpeuse de vos lèvres. Nous recommandons d’effectuer un léger gommage des lèvres 1 à 2 fois par semaine. Cela permet d’éliminer les peaux mortes et favorise une meilleure absorption du produit. Une réelle alternative, douce et naturelle, aux injections d’acide hyaluronique !</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>DIMETHICONE, DICAPRYLYL CARBONATE, QUATERIUM-90 SEPIOLITE, ISONONYL ISONONANOATE, TRIMETHYLSILOXYSILICATE, QUATERIUM-90 MONTMORILLONITE, ISOPROPYL MYRISTATE, ETHYLHEXYL PALMITATE, TRIBEHENIN, SORBITAN ISOSTEARATE, PALMITOYL TRIPEPTIDE-1, LACTIC ACID, BHT, ETHYLHEXYL METHOXYCINNAMATE, CAPRYLYL GLYCOL, BUTYROSPERMUM PARKII BUTTER, CAMELLIA JAPONICA SEED OIL, TOCOPHERYL ACETATE, TOCOPHEROL, ISOPROPYL TITANIUM TRIISOSTEARATE, POLYHYDROXYSTEARIC ACID, STEARALKONIUM HECTORITE, PROPYLENE CARBONATE, AROMA, [ +/- MAY CONTAIN CI 77891 /TITANIUM DIOXIDE, CI 15880 /RED 63: 1, CI 17200 /RED 33, CI 15850 /RED 57, CI 15850 /RED 57: 1, CI 77491, CI 77492, CI 77499 /IRON OXIDES]</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr"/>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>images/8697711011160.jpg</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>https://biobalance.tn/maquillage/56-customizable-mug.html</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>https://biobalance.tn/maquillage/56-customizable-mug.html | https://www.barcodelookup.com/8697711011160</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>8697711011191</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>BB-WEB-57</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Repulpeur Lèvres Hot Red N°10</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Repulpeur Lèvres Hot Red N°10</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>LipojeN</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Maquillage</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>5 ml</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Soin Repulpeur Semi Mat Lipojen Hot Red, le secret des lèvres pulpeuses, lisses et parfaitement hydratées.
+Grâce à sa formule exclusive combinant des tripeptides repulpants, de l’acide hyaluronique et un extrait de gingembre, il repulpe intensément, lisse les ridules et hydrate en profondeur, tout en offrant une couleur intense et brillante qui révèle toute votre féminité et votre sensualité dès le premier passage. Une alternative naturelle et douce aux injections d’acide hyaluronique, à utiliser quotidiennement comme un rouge à lèvres, avec une protection solaire contre les rayons UVA et UVB.</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Pour profiter pleinement des bienfaits des repulpeurs lèvres LipojeN, voici quelques conseils d’utilisation bien utiles : Assurez-vous que vos lèvres soient propres et sèches avant l’application. Appliquez le rouge à lèvres LipojeN au moins 3 fois par jour pendant 30 jours pour obtenir de bons résultats . Les jours où vous ne souhaitez pas vous maquiller, il est possible d’appliquer le Glossy crystal clear numéro 01 pour ne pas interrompre le traitement. N’hésitez pas à renouveler l’application aussi souvent que souhaité pour maintenir l’hydratation et l’apparence pulpeuse de vos lèvres. Nous recommandons d’effectuer un léger gommage des lèvres 1 à 2 fois par semaine. Cela permet d’éliminer les peaux mortes et favorise une meilleure absorption du produit. Une réelle alternative, douce et naturelle, aux injections d’acide hyaluronique !</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>DIMETHICONE, DICAPRYLYL CARBONATE, QUATERIUM-90 SEPIOLITE, ISONONYL ISONONANOATE, TRIMETHYLSILOXYSILICATE, QUATERIUM-90 MONTMORILLONITE, ISOPROPYL MYRISTATE, ETHYLHEXYL PALMITATE, TRIBEHENIN, SORBITAN ISOSTEARATE, PALMITOYL TRIPEPTIDE-1, LACTIC ACID, BHT, ETHYLHEXYL METHOXYCINNAMATE, CAPRYLYL GLYCOL, BUTYROSPERMUM PARKII BUTTER, CAMELLIA JAPONICA SEED OIL, TOCOPHERYL ACETATE, TOCOPHEROL, ISOPROPYL TITANIUM TRIISOSTEARATE, POLYHYDROXYSTEARIC ACID, STEARALKONIUM HECTORITE, PROPYLENE CARBONATE, AROMA, [ +/- MAY CONTAIN CI 77891 /TITANIUM DIOXIDE, CI 15880 /RED 63: 1, CI 17200 /RED 33, CI 15850 /RED 57, CI 15850 /RED 57: 1, CI 77491, CI 77492, CI 77499 /IRON OXIDES]</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr"/>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>images/8697711011191.jpg</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>https://biobalance.tn/maquillage/57-customizable-mug.html</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>https://biobalance.tn/maquillage/57-customizable-mug.html | https://www.barcodelookup.com/8697711011191</t>
+        </is>
+      </c>
+      <c r="O45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>8697711011221</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>BB-WEB-58</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Repulpeur Lèvres Flamingo Love N°31</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Repulpeur Lèvres Flamingo Love N°31</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>LipojeN</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Maquillage</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>5 ml</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Soin Repulpeur Flamingo Love, le secret des lèvres pulpeuses, lisses et parfaitement hydratées.
+Grâce à sa formule exclusive combinant des tripeptides repulpants, de l’acide hyaluronique et un extrait de gingembre, il repulpe intensément, lisse les ridules et hydrate en profondeur, tout en offrant une couleur intense et brillante qui révèle toute votre féminité et votre sensualité dès le premier passage. Une alternative naturelle et douce aux injections d’acide hyaluronique, à utiliser quotidiennement comme un rouge à lèvres, avec une protection solaire contre les rayons UVA et UVB.</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Pour profiter pleinement des bienfaits des repulpeurs lèvres LipojeN, voici quelques conseils d’utilisation bien utiles : Assurez-vous que vos lèvres soient propres et sèches avant l’application. Appliquez le rouge à lèvres LipojeN au moins 3 fois par jour pendant 30 jours pour obtenir de bons résultats . Les jours où vous ne souhaitez pas vous maquiller, il est possible d’appliquer le Glossy crystal clear numéro 01 pour ne pas interrompre le traitement. N’hésitez pas à renouveler l’application aussi souvent que souhaité pour maintenir l’hydratation et l’apparence pulpeuse de vos lèvres. Nous recommandons d’effectuer un léger gommage des lèvres 1 à 2 fois par semaine. Cela permet d’éliminer les peaux mortes et favorise une meilleure absorption du produit. Une réelle alternative, douce et naturelle, aux injections d’acide hyaluronique !</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>HYDROGENATED POLYISOBUTENE, CAPRYLIC/CAPRIC TRIGLYCERIDE, BUTYROSPERMUM PARKII BUTTER, CERA ALBA, AQUA, ETHYLHEXYL METHOXYCINNAMATE, SODIUM HYALURONATE, BHT, TOCOPHERYL ACETATE, PALMITOYL TRIPEPTIDE-1, CAMELLIA JAPONICA SEED OIL, AROMA, ETHYLHEXYL PALMITATE, TRIBEHENIN, SORBITAN ISOSTEARATE, LACTIC ACID, SORBITAN CAPRYLATE, PROPANEDIOL, BENZOIC ACID, ISONONYL ISONONANOATE, ISOPROPYL MYRISTATE, ISOPROPYL TITANIUM TRIISOSTEARATE, STEARALKONIUM HECTORITE, POLYHYDROXYSTEARIC ACID, PROPYLENE CARBONATE, [ +/- MAY CONTAIN MICA, CI 77891 CI 77491, CI 77492, CI 15850, CI75470</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr"/>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>images/8697711011221.jpg</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>https://biobalance.tn/maquillage/58-customizable-mug.html</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>https://biobalance.tn/maquillage/58-customizable-mug.html | https://www.barcodelookup.com/8697711011221</t>
+        </is>
+      </c>
+      <c r="O46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>8697711011238</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>BB-WEB-59</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Repulpeur Lèvres Coral Dream N°32</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Repulpeur Lèvres Coral Dream N°32</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>LipojeN</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Maquillage</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>5 ml</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Le Repulpeur lèvres Coral Dream est le secret des lèvres pulpeuses, lisses et parfaitement hydratées.
+Grâce à sa formule exclusive combinant des tripeptides repulpants, de l’acide hyaluronique et un extrait de gingembre, il repulpe intensément, lisse les ridules et hydrate en profondeur, tout en offrant une couleur intense et brillante qui révèle toute votre féminité et votre sensualité dès le premier passage. Une alternative naturelle et douce aux injections d’acide hyaluronique, à utiliser quotidiennement comme un rouge à lèvres, avec une protection solaire contre les rayons UVA et UVB.</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Pour profiter pleinement des bienfaits des repulpeurs lèvres LipojeN, voici quelques conseils d’utilisation bien utiles : Assurez-vous que vos lèvres soient propres et sèches avant l’application. Appliquez le rouge à lèvres LipojeN au moins 3 fois par jour pendant 30 jours pour obtenir de bons résultats . Les jours où vous ne souhaitez pas vous maquiller, il est possible d’appliquer le Glossy crystal clear numéro 01 pour ne pas interrompre le traitement. N’hésitez pas à renouveler l’application aussi souvent que souhaité pour maintenir l’hydratation et l’apparence pulpeuse de vos lèvres. Nous recommandons d’effectuer un léger gommage des lèvres 1 à 2 fois par semaine. Cela permet d’éliminer les peaux mortes et favorise une meilleure absorption du produit. Une réelle alternative, douce et naturelle, aux injections d’acide hyaluronique !</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>HYDROGENATED POLYISOBUTENE, CAPRYLIC/CAPRIC TRIGLYCERIDE, BUTYROSPERMUM PARKII BUTTER, CERA ALBA, AQUA, ETHYLHEXYL METHOXYCINNAMATE, SODIUM HYALURONATE, BHT, TOCOPHERYL ACETATE, PALMITOYL TRIPEPTIDE-1, CAMELLIA JAPONICA SEED OIL, AROMA, ETHYLHEXYL PALMITATE, TRIBEHENIN, SORBITAN ISOSTEARATE, LACTIC ACID, SORBITAN CAPRYLATE, PROPANEDIOL, BENZOIC ACID, ISONONYL ISONONANOATE, ISOPROPYL MYRISTATE, ISOPROPYL TITANIUM TRIISOSTEARATE, STEARALKONIUM HECTORITE, POLYHYDROXYSTEARIC ACID, PROPYLENE CARBONATE, [ +/- MAY CONTAIN MICA, CI 77891, CI 77491, CI 77492, CI 15850, CI75470]</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr"/>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>images/8697711011238.jpg</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>https://biobalance.tn/maquillage/59-customizable-mug.html</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>https://biobalance.tn/maquillage/59-customizable-mug.html | https://www.barcodelookup.com/8697711011238</t>
+        </is>
+      </c>
+      <c r="O47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>8697711011252</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>BB-WEB-60</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Repulpeur Lèvres Fuchsia Vibes N°34</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Repulpeur Lèvres Fuchsia Vibes N°34</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>LipojeN</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Maquillage</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>5 ml</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Le Repulpeur lèvres Fuchsia Vibes est le secret des lèvres pulpeuses, lisses et parfaitement hydratées.
+Grâce à sa formule exclusive combinant des tripeptides repulpants, de l’acide hyaluronique et un extrait de gingembre, il repulpe intensément, lisse les ridules et hydrate en profondeur, tout en offrant une couleur intense et brillante qui révèle toute votre féminité et votre sensualité dès le premier passage. Une alternative naturelle et douce aux injections d’acide hyaluronique, à utiliser quotidiennement comme un rouge à lèvres, avec une protection solaire contre les rayons UVA et UVB.</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Pour profiter pleinement des bienfaits des repulpeurs lèvres LipojeN, voici quelques conseils d’utilisation bien utiles : Assurez-vous que vos lèvres soient propres et sèches avant l’application. Appliquez le rouge à lèvres LipojeN au moins 3 fois par jour pendant 30 jours pour obtenir de bons résultats . Les jours où vous ne souhaitez pas vous maquiller, il est possible d’appliquer le Glossy crystal clear numéro 01 pour ne pas interrompre le traitement. N’hésitez pas à renouveler l’application aussi souvent que souhaité pour maintenir l’hydratation et l’apparence pulpeuse de vos lèvres. Nous recommandons d’effectuer un léger gommage des lèvres 1 à 2 fois par semaine. Cela permet d’éliminer les peaux mortes et favorise une meilleure absorption du produit. Une réelle alternative, douce et naturelle, aux injections d’acide hyaluronique !</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>HYDROGENATED POLYISOBUTENE, CAPRYLIC/CAPRIC TRIGLYCERIDE, BUTYROSPERMUM PARKII BUTTER, CERA ALBA, AQUA, ETHYLHEXYL METHOXYCINNAMATE, SODIUM HYALURONATE, BHT, TOCOPHERYL ACETATE, PALMITOYL TRIPEPTIDE-1, CAMELLIA JAPONICA SEED OIL, AROMA, ETHYLHEXYL PALMITATE, TRIBEHENIN, SORBITAN ISOSTEARATE, LACTIC ACID, SORBITAN CAPRYLATE, PROPANEDIOL, BENZOIC ACID, ISONONYL ISONONANOATE, ISOPROPYL MYRISTATE, ISOPROPYL TITANIUM TRIISOSTEARATE, STEARALKONIUM HECTORITE, POLYHYDROXYSTEARIC ACID, PROPYLENE CARBONATE, [ +/- MAY CONTAIN MICA, CI 77891, CI 77491, CI 77492, CI 15850, CI75470]</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr"/>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>images/8697711011252.jpg</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>https://biobalance.tn/maquillage/60-customizable-mug.html</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>https://biobalance.tn/maquillage/60-customizable-mug.html | https://www.barcodelookup.com/8697711011252</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>8697711011269</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>BB-WEB-61</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Repulpeur Lèvres Candy Crush N°35</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Repulpeur Lèvres Candy Crush N°35</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>LipojeN</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Maquillage</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>5 ml</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>20Le Repulpeur lèvres Candy Crush est le secret des lèvres pulpeuses, lisses et parfaitement hydratées.
+Grâce à sa formule exclusive combinant des tripeptides repulpants, de l’acide hyaluronique et un extrait de gingembre, il repulpe intensément, lisse les ridules et hydrate en profondeur, tout en offrant une couleur intense et brillante qui révèle toute votre féminité et votre sensualité dès le premier passage. Une alternative naturelle et douce aux injections d’acide hyaluronique, à utiliser quotidiennement comme un rouge à lèvres, avec une protection solaire contre les rayons UVA et UVB.</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Pour profiter pleinement des bienfaits des repulpeurs lèvres LipojeN, voici quelques conseils d’utilisation bien utiles : Assurez-vous que vos lèvres soient propres et sèches avant l’application. Appliquez le rouge à lèvres LipojeN au moins 3 fois par jour pendant 30 jours pour obtenir de bons résultats . Les jours où vous ne souhaitez pas vous maquiller, il est possible d’appliquer le Glossy crystal clear numéro 01 pour ne pas interrompre le traitement. N’hésitez pas à renouveler l’application aussi souvent que souhaité pour maintenir l’hydratation et l’apparence pulpeuse de vos lèvres. Nous recommandons d’effectuer un léger gommage des lèvres 1 à 2 fois par semaine. Cela permet d’éliminer les peaux mortes et favorise une meilleure absorption du produit. Une réelle alternative, douce et naturelle, aux injections d’acide hyaluronique !</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr"/>
+      <c r="K49" t="inlineStr"/>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>images/8697711011269.jpg</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>https://biobalance.tn/maquillage/61-customizable-mug.html</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>https://biobalance.tn/maquillage/61-customizable-mug.html</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>ingrédients</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>8697711011283</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>BB-WEB-62</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Repulpeur Lèvres Cinnamon Roll N°37</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Repulpeur Lèvres Cinnamon Roll N°37</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>LipojeN</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Maquillage</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>5 ml</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>20Le Repulpeur lèvres Cinnamon Roll est le secret des lèvres pulpeuses, lisses et parfaitement hydratées.
+Grâce à sa formule exclusive combinant des tripeptides repulpants, de l’acide hyaluronique et un extrait de gingembre, il repulpe intensément, lisse les ridules et hydrate en profondeur, tout en offrant une couleur intense et brillante qui révèle toute votre féminité et votre sensualité dès le premier passage. Une alternative naturelle et douce aux injections d’acide hyaluronique, à utiliser quotidiennement comme un rouge à lèvres, avec une protection solaire contre les rayons UVA et UVB.</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Pour profiter pleinement des bienfaits des repulpeurs lèvres LipojeN, voici quelques conseils d’utilisation bien utiles : Assurez-vous que vos lèvres soient propres et sèches avant l’application. Appliquez le rouge à lèvres LipojeN au moins 3 fois par jour pendant 30 jours pour obtenir de bons résultats . Les jours où vous ne souhaitez pas vous maquiller, il est possible d’appliquer le Glossy crystal clear numéro 01 pour ne pas interrompre le traitement. N’hésitez pas à renouveler l’application aussi souvent que souhaité pour maintenir l’hydratation et l’apparence pulpeuse de vos lèvres. Nous recommandons d’effectuer un léger gommage des lèvres 1 à 2 fois par semaine. Cela permet d’éliminer les peaux mortes et favorise une meilleure absorption du produit. Une réelle alternative, douce et naturelle, aux injections d’acide hyaluronique !</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr"/>
+      <c r="K50" t="inlineStr"/>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>images/8697711011283.jpg</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>https://biobalance.tn/maquillage/62-customizable-mug.html</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>https://biobalance.tn/maquillage/62-customizable-mug.html</t>
+        </is>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>ingrédients</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>8697711721014</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>BB-WEB-53</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Acnevit Anti-Acne Serum</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Acnevit Anti-Acne Serum</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Acnevit</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Sérums</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>30 ml</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Le sérum Acnevit Anti-Acne traite l’acné, prévient l’apparition de nouveaux boutons et atténue la couleur des marques d’acné pour un teint uniforme et visiblement plus net. Il n’est pas nécessaire d’utiliser une crème de jour, une crème de nuit, un tonique ou un masque. Le sérum Acnevit remplace tous ces produits, éliminant ainsi les applications multiples, longues et coûteuses. Il suffit d’appliquer le sérum Acnevit Anti-Acne uniquement, deux fois par jour pendant les dix premiers jours, puis une fois par jour pour obtenir un résultat optimal. / Sans huile / Non comédogène / Sans colorant / Sans savon.</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Appliquer le sérum deux fois par jour pendant les dix premiers jours, puis une fois par jour pour obtenir les résultats.</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr"/>
+      <c r="K51" t="inlineStr"/>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>images/8697711721014.jpg</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>https://biobalance.tn/serum/53-customizable-mug.html</t>
+        </is>
+      </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>https://biobalance.tn/serum/53-customizable-mug.html</t>
+        </is>
+      </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>ingrédients</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>8697711721021</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>BB-WEB-63</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Acnevit Anti-Acne Cleansing Gel</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Acnevit Anti-Acne Cleansing Gel</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Acnevit</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Nettoyants visage</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>200 ml</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Acnevit Gel Nettoyant Anti-Acné nettoie la peau en douceur et en profondeur jusque dans les pores, pour une peau nette et purifiée. Grâce à l’association efficace de Niacinamide, Extrait de feuille de Romarin, Extrait de Centella Asiatica, Extrait de pépins de raisin et Allantoïne, ses agents apaisants aident à prévenir les irritations, évitent le dessèchement excessif tout en hydratant et protégeant la peau.
+Avantages :
+• Nettoie la peau en douceur et en profondeur jusque dans les pores, pour une peau nette.
+• Réduit la production excessive de sébum.
+• Réduit la taille des pores.
+• Diminue la brillance et les points noirs.
+• La mousse légère se rince facilement, sans laisser de résidus pouvant obstruer les pores.</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Appliquer sur le visage humide en évitant le contour des yeux, masser puis rincer à l’eau tiède. Utiliser deux fois par jour.</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr"/>
+      <c r="K52" t="inlineStr"/>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>images/8697711721021.jpg</t>
+        </is>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>https://biobalance.tn/nettoyants-visage/63-customizable-mug.html</t>
+        </is>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>https://biobalance.tn/nettoyants-visage/63-customizable-mug.html</t>
+        </is>
+      </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>ingrédients</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Ingredient lists for the last four products (Acnevit serum and gel, LipojeN N°35 and N°37)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/initial-catalog/produits.xlsx
+++ b/data/initial-catalog/produits.xlsx
@@ -3476,7 +3476,7 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>DIMETHICONE, DICAPRYLYL CARBONATE, QUATERIUM-90 SEPIOLITE, ISONONYL ISONONANOATE, TRIMETHYLSILOXYSILICATE, QUATERIUM-90 MONTMORILLONITE, ISOPROPYL MYRISTATE, ETHYLHEXYL PALMITATE, TRIBEHENIN, SORBITAN ISOSTEARATE, PALMITOYL TRIPEPTIDE-1, LACTIC ACID, BHT, ETHYLHEXYL METHOXYCINNAMATE, CAPRYLYL GLYCOL, BUTYROSPERMUM PARKII BUTTER, CAMELLIA JAPONICA SEED OIL, TOCOPHERYL ACETATE, TOCOPHEROL, ISOPROPYL TITANIUM TRIISOSTEARATE, POLYHYDROXYSTEARIC ACID, STEARALKONIUM HECTORITE, PROPYLENE CARBONATE, AROMA, [ +/- MAY CONTAIN CI 77891 /TITANIUM DIOXIDE, CI 15880 /RED 63: 1, CI 17200 /RED 33, CI 15850 /RED 57, CI 15850 /RED 57: 1, CI 77491, CI 77492, CI 77499 /IRON OXIDES]</t>
+          <t>DIMETHICONE, DICAPRYLYL CARBONATE, QUATERIUM-90 SEPIOLITE, ISONONYL ISONONANOATE, TRIMETHYLSILOXYSILICATE, QUATERIUM-90 MONTMORILLONITE, ISOPROPYL MYRISTATE, ETHYLHEXYL PALMITATE, TRIBEHENIN, SORBITAN ISOSTEARATE, PALMITOYL TRIPEPTIDE-1, LACTIC ACID, BHT, ETHYLHEXYL METHOXYCINNAMATE, CAPRYLYL GLYCOL, BUTYROSPERMUM PARKII BUTTER, CAMELLIA JAPONICA SEED OIL, TOCOPHERYL ACETATE, TOCOPHEROL, ISOPROPYL TITANIUM TRIISOSTEARATE, POLYHYDROXYSTEARIC ACID, STEARALKONIUM HECTORITE, PROPYLENE CARBONATE, AROMA, [+/- MAY CONTAIN CI 77891 /TITANIUM DIOXIDE, CI 15880 /RED 63: 1, CI 17200 /RED 33, CI 15850 /RED 57, CI 15850 /RED 57: 1, CI 77491, CI 77492, CI 77499 /IRON OXIDES]</t>
         </is>
       </c>
       <c r="K41" t="inlineStr"/>
@@ -3546,7 +3546,7 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>DIMETHICONE, DICAPRYLYL CARBONATE, QUATERIUM-90 SEPIOLITE, ISONONYL ISONONANOATE, TRIMETHYLSILOXYSILICATE, QUATERIUM-90 MONTMORILLONITE, ISOPROPYL MYRISTATE, ETHYLHEXYL PALMITATE, TRIBEHENIN, SORBITAN ISOSTEARATE, PALMITOYL TRIPEPTIDE-1, LACTIC ACID, BHT, ETHYLHEXYL METHOXYCINNAMATE, CAPRYLYL GLYCOL, BUTYROSPERMUM PARKII BUTTER, CAMELLIA JAPONICA SEED OIL, TOCOPHERYL ACETATE, TOCOPHEROL, ISOPROPYL TITANIUM TRIISOSTEARATE, POLYHYDROXYSTEARIC ACID, STEARALKONIUM HECTORITE, PROPYLENE CARBONATE, AROMA, [ +/- MAY CONTAIN CI 77891 /TITANIUM DIOXIDE, CI 15880 /RED 63: 1, CI 17200 /RED 33, CI 15850 /RED 57, CI 15850 /RED 57: 1, CI 77491, CI 77492, CI 77499 /IRON OXIDES]</t>
+          <t>DIMETHICONE, DICAPRYLYL CARBONATE, QUATERIUM-90 SEPIOLITE, ISONONYL ISONONANOATE, TRIMETHYLSILOXYSILICATE, QUATERIUM-90 MONTMORILLONITE, ISOPROPYL MYRISTATE, ETHYLHEXYL PALMITATE, TRIBEHENIN, SORBITAN ISOSTEARATE, PALMITOYL TRIPEPTIDE-1, LACTIC ACID, BHT, ETHYLHEXYL METHOXYCINNAMATE, CAPRYLYL GLYCOL, BUTYROSPERMUM PARKII BUTTER, CAMELLIA JAPONICA SEED OIL, TOCOPHERYL ACETATE, TOCOPHEROL, ISOPROPYL TITANIUM TRIISOSTEARATE, POLYHYDROXYSTEARIC ACID, STEARALKONIUM HECTORITE, PROPYLENE CARBONATE, AROMA, [+/- MAY CONTAIN CI 77891 /TITANIUM DIOXIDE, CI 15880 /RED 63: 1, CI 17200 /RED 33, CI 15850 /RED 57, CI 15850 /RED 57: 1, CI 77491, CI 77492, CI 77499 /IRON OXIDES]</t>
         </is>
       </c>
       <c r="K42" t="inlineStr"/>
@@ -3616,7 +3616,7 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>DIMETHICONE, DICAPRYLYL CARBONATE, QUATERIUM-90 SEPIOLITE, ISONONYL ISONONANOATE, TRIMETHYLSILOXYSILICATE, QUATERIUM-90 MONTMORILLONITE, ISOPROPYL MYRISTATE, ETHYLHEXYL PALMITATE, TRIBEHENIN, SORBITAN ISOSTEARATE, PALMITOYL TRIPEPTIDE-1, LACTIC ACID, BHT, ETHYLHEXYL METHOXYCINNAMATE, CAPRYLYL GLYCOL, BUTYROSPERMUM PARKII BUTTER, CAMELLIA JAPONICA SEED OIL, TOCOPHERYL ACETATE, TOCOPHEROL, ISOPROPYL TITANIUM TRIISOSTEARATE, POLYHYDROXYSTEARIC ACID, STEARALKONIUM HECTORITE, PROPYLENE CARBONATE, AROMA, [ +/- MAY CONTAIN CI 77891 /TITANIUM DIOXIDE, CI 15880 /RED 63: 1, CI 17200 /RED 33, CI 15850 /RED 57, CI 15850 /RED 57: 1, CI 77491, CI 77492, CI 77499 /IRON OXIDES]</t>
+          <t>DIMETHICONE, DICAPRYLYL CARBONATE, QUATERIUM-90 SEPIOLITE, ISONONYL ISONONANOATE, TRIMETHYLSILOXYSILICATE, QUATERIUM-90 MONTMORILLONITE, ISOPROPYL MYRISTATE, ETHYLHEXYL PALMITATE, TRIBEHENIN, SORBITAN ISOSTEARATE, PALMITOYL TRIPEPTIDE-1, LACTIC ACID, BHT, ETHYLHEXYL METHOXYCINNAMATE, CAPRYLYL GLYCOL, BUTYROSPERMUM PARKII BUTTER, CAMELLIA JAPONICA SEED OIL, TOCOPHERYL ACETATE, TOCOPHEROL, ISOPROPYL TITANIUM TRIISOSTEARATE, POLYHYDROXYSTEARIC ACID, STEARALKONIUM HECTORITE, PROPYLENE CARBONATE, AROMA, [+/- MAY CONTAIN CI 77891 /TITANIUM DIOXIDE, CI 15880 /RED 63: 1, CI 17200 /RED 33, CI 15850 /RED 57, CI 15850 /RED 57: 1, CI 77491, CI 77492, CI 77499 /IRON OXIDES]</t>
         </is>
       </c>
       <c r="K43" t="inlineStr"/>
@@ -3686,7 +3686,7 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>DIMETHICONE, DICAPRYLYL CARBONATE, QUATERIUM-90 SEPIOLITE, ISONONYL ISONONANOATE, TRIMETHYLSILOXYSILICATE, QUATERIUM-90 MONTMORILLONITE, ISOPROPYL MYRISTATE, ETHYLHEXYL PALMITATE, TRIBEHENIN, SORBITAN ISOSTEARATE, PALMITOYL TRIPEPTIDE-1, LACTIC ACID, BHT, ETHYLHEXYL METHOXYCINNAMATE, CAPRYLYL GLYCOL, BUTYROSPERMUM PARKII BUTTER, CAMELLIA JAPONICA SEED OIL, TOCOPHERYL ACETATE, TOCOPHEROL, ISOPROPYL TITANIUM TRIISOSTEARATE, POLYHYDROXYSTEARIC ACID, STEARALKONIUM HECTORITE, PROPYLENE CARBONATE, AROMA, [ +/- MAY CONTAIN CI 77891 /TITANIUM DIOXIDE, CI 15880 /RED 63: 1, CI 17200 /RED 33, CI 15850 /RED 57, CI 15850 /RED 57: 1, CI 77491, CI 77492, CI 77499 /IRON OXIDES]</t>
+          <t>DIMETHICONE, DICAPRYLYL CARBONATE, QUATERIUM-90 SEPIOLITE, ISONONYL ISONONANOATE, TRIMETHYLSILOXYSILICATE, QUATERIUM-90 MONTMORILLONITE, ISOPROPYL MYRISTATE, ETHYLHEXYL PALMITATE, TRIBEHENIN, SORBITAN ISOSTEARATE, PALMITOYL TRIPEPTIDE-1, LACTIC ACID, BHT, ETHYLHEXYL METHOXYCINNAMATE, CAPRYLYL GLYCOL, BUTYROSPERMUM PARKII BUTTER, CAMELLIA JAPONICA SEED OIL, TOCOPHERYL ACETATE, TOCOPHEROL, ISOPROPYL TITANIUM TRIISOSTEARATE, POLYHYDROXYSTEARIC ACID, STEARALKONIUM HECTORITE, PROPYLENE CARBONATE, AROMA, [+/- MAY CONTAIN CI 77891 /TITANIUM DIOXIDE, CI 15880 /RED 63: 1, CI 17200 /RED 33, CI 15850 /RED 57, CI 15850 /RED 57: 1, CI 77491, CI 77492, CI 77499 /IRON OXIDES]</t>
         </is>
       </c>
       <c r="K44" t="inlineStr"/>
@@ -3756,7 +3756,7 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>DIMETHICONE, DICAPRYLYL CARBONATE, QUATERIUM-90 SEPIOLITE, ISONONYL ISONONANOATE, TRIMETHYLSILOXYSILICATE, QUATERIUM-90 MONTMORILLONITE, ISOPROPYL MYRISTATE, ETHYLHEXYL PALMITATE, TRIBEHENIN, SORBITAN ISOSTEARATE, PALMITOYL TRIPEPTIDE-1, LACTIC ACID, BHT, ETHYLHEXYL METHOXYCINNAMATE, CAPRYLYL GLYCOL, BUTYROSPERMUM PARKII BUTTER, CAMELLIA JAPONICA SEED OIL, TOCOPHERYL ACETATE, TOCOPHEROL, ISOPROPYL TITANIUM TRIISOSTEARATE, POLYHYDROXYSTEARIC ACID, STEARALKONIUM HECTORITE, PROPYLENE CARBONATE, AROMA, [ +/- MAY CONTAIN CI 77891 /TITANIUM DIOXIDE, CI 15880 /RED 63: 1, CI 17200 /RED 33, CI 15850 /RED 57, CI 15850 /RED 57: 1, CI 77491, CI 77492, CI 77499 /IRON OXIDES]</t>
+          <t>DIMETHICONE, DICAPRYLYL CARBONATE, QUATERIUM-90 SEPIOLITE, ISONONYL ISONONANOATE, TRIMETHYLSILOXYSILICATE, QUATERIUM-90 MONTMORILLONITE, ISOPROPYL MYRISTATE, ETHYLHEXYL PALMITATE, TRIBEHENIN, SORBITAN ISOSTEARATE, PALMITOYL TRIPEPTIDE-1, LACTIC ACID, BHT, ETHYLHEXYL METHOXYCINNAMATE, CAPRYLYL GLYCOL, BUTYROSPERMUM PARKII BUTTER, CAMELLIA JAPONICA SEED OIL, TOCOPHERYL ACETATE, TOCOPHEROL, ISOPROPYL TITANIUM TRIISOSTEARATE, POLYHYDROXYSTEARIC ACID, STEARALKONIUM HECTORITE, PROPYLENE CARBONATE, AROMA, [+/- MAY CONTAIN CI 77891 /TITANIUM DIOXIDE, CI 15880 /RED 63: 1, CI 17200 /RED 33, CI 15850 /RED 57, CI 15850 /RED 57: 1, CI 77491, CI 77492, CI 77499 /IRON OXIDES]</t>
         </is>
       </c>
       <c r="K45" t="inlineStr"/>
@@ -3826,7 +3826,7 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>HYDROGENATED POLYISOBUTENE, CAPRYLIC/CAPRIC TRIGLYCERIDE, BUTYROSPERMUM PARKII BUTTER, CERA ALBA, AQUA, ETHYLHEXYL METHOXYCINNAMATE, SODIUM HYALURONATE, BHT, TOCOPHERYL ACETATE, PALMITOYL TRIPEPTIDE-1, CAMELLIA JAPONICA SEED OIL, AROMA, ETHYLHEXYL PALMITATE, TRIBEHENIN, SORBITAN ISOSTEARATE, LACTIC ACID, SORBITAN CAPRYLATE, PROPANEDIOL, BENZOIC ACID, ISONONYL ISONONANOATE, ISOPROPYL MYRISTATE, ISOPROPYL TITANIUM TRIISOSTEARATE, STEARALKONIUM HECTORITE, POLYHYDROXYSTEARIC ACID, PROPYLENE CARBONATE, [ +/- MAY CONTAIN MICA, CI 77891 CI 77491, CI 77492, CI 15850, CI75470</t>
+          <t>HYDROGENATED POLYISOBUTENE, CAPRYLIC/CAPRIC TRIGLYCERIDE, BUTYROSPERMUM PARKII BUTTER, CERA ALBA, AQUA, ETHYLHEXYL METHOXYCINNAMATE, SODIUM HYALURONATE, BHT, TOCOPHERYL ACETATE, PALMITOYL TRIPEPTIDE-1, CAMELLIA JAPONICA SEED OIL, AROMA, ETHYLHEXYL PALMITATE, TRIBEHENIN, SORBITAN ISOSTEARATE, LACTIC ACID, SORBITAN CAPRYLATE, PROPANEDIOL, BENZOIC ACID, ISONONYL ISONONANOATE, ISOPROPYL MYRISTATE, ISOPROPYL TITANIUM TRIISOSTEARATE, STEARALKONIUM HECTORITE, POLYHYDROXYSTEARIC ACID, PROPYLENE CARBONATE, [+/- MAY CONTAIN MICA, CI 77891, CI 77491, CI 77492, CI 15850, CI 75470]</t>
         </is>
       </c>
       <c r="K46" t="inlineStr"/>
@@ -3896,7 +3896,7 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>HYDROGENATED POLYISOBUTENE, CAPRYLIC/CAPRIC TRIGLYCERIDE, BUTYROSPERMUM PARKII BUTTER, CERA ALBA, AQUA, ETHYLHEXYL METHOXYCINNAMATE, SODIUM HYALURONATE, BHT, TOCOPHERYL ACETATE, PALMITOYL TRIPEPTIDE-1, CAMELLIA JAPONICA SEED OIL, AROMA, ETHYLHEXYL PALMITATE, TRIBEHENIN, SORBITAN ISOSTEARATE, LACTIC ACID, SORBITAN CAPRYLATE, PROPANEDIOL, BENZOIC ACID, ISONONYL ISONONANOATE, ISOPROPYL MYRISTATE, ISOPROPYL TITANIUM TRIISOSTEARATE, STEARALKONIUM HECTORITE, POLYHYDROXYSTEARIC ACID, PROPYLENE CARBONATE, [ +/- MAY CONTAIN MICA, CI 77891, CI 77491, CI 77492, CI 15850, CI75470]</t>
+          <t>HYDROGENATED POLYISOBUTENE, CAPRYLIC/CAPRIC TRIGLYCERIDE, BUTYROSPERMUM PARKII BUTTER, CERA ALBA, AQUA, ETHYLHEXYL METHOXYCINNAMATE, SODIUM HYALURONATE, BHT, TOCOPHERYL ACETATE, PALMITOYL TRIPEPTIDE-1, CAMELLIA JAPONICA SEED OIL, AROMA, ETHYLHEXYL PALMITATE, TRIBEHENIN, SORBITAN ISOSTEARATE, LACTIC ACID, SORBITAN CAPRYLATE, PROPANEDIOL, BENZOIC ACID, ISONONYL ISONONANOATE, ISOPROPYL MYRISTATE, ISOPROPYL TITANIUM TRIISOSTEARATE, STEARALKONIUM HECTORITE, POLYHYDROXYSTEARIC ACID, PROPYLENE CARBONATE, [+/- MAY CONTAIN MICA, CI 77891, CI 77491, CI 77492, CI 15850, CI 75470]</t>
         </is>
       </c>
       <c r="K47" t="inlineStr"/>
@@ -3966,7 +3966,7 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>HYDROGENATED POLYISOBUTENE, CAPRYLIC/CAPRIC TRIGLYCERIDE, BUTYROSPERMUM PARKII BUTTER, CERA ALBA, AQUA, ETHYLHEXYL METHOXYCINNAMATE, SODIUM HYALURONATE, BHT, TOCOPHERYL ACETATE, PALMITOYL TRIPEPTIDE-1, CAMELLIA JAPONICA SEED OIL, AROMA, ETHYLHEXYL PALMITATE, TRIBEHENIN, SORBITAN ISOSTEARATE, LACTIC ACID, SORBITAN CAPRYLATE, PROPANEDIOL, BENZOIC ACID, ISONONYL ISONONANOATE, ISOPROPYL MYRISTATE, ISOPROPYL TITANIUM TRIISOSTEARATE, STEARALKONIUM HECTORITE, POLYHYDROXYSTEARIC ACID, PROPYLENE CARBONATE, [ +/- MAY CONTAIN MICA, CI 77891, CI 77491, CI 77492, CI 15850, CI75470]</t>
+          <t>HYDROGENATED POLYISOBUTENE, CAPRYLIC/CAPRIC TRIGLYCERIDE, BUTYROSPERMUM PARKII BUTTER, CERA ALBA, AQUA, ETHYLHEXYL METHOXYCINNAMATE, SODIUM HYALURONATE, BHT, TOCOPHERYL ACETATE, PALMITOYL TRIPEPTIDE-1, CAMELLIA JAPONICA SEED OIL, AROMA, ETHYLHEXYL PALMITATE, TRIBEHENIN, SORBITAN ISOSTEARATE, LACTIC ACID, SORBITAN CAPRYLATE, PROPANEDIOL, BENZOIC ACID, ISONONYL ISONONANOATE, ISOPROPYL MYRISTATE, ISOPROPYL TITANIUM TRIISOSTEARATE, STEARALKONIUM HECTORITE, POLYHYDROXYSTEARIC ACID, PROPYLENE CARBONATE, [+/- MAY CONTAIN MICA, CI 77891, CI 77491, CI 77492, CI 15850, CI 75470]</t>
         </is>
       </c>
       <c r="K48" t="inlineStr"/>
@@ -4034,7 +4034,11 @@
           <t>Pour profiter pleinement des bienfaits des repulpeurs lèvres LipojeN, voici quelques conseils d’utilisation bien utiles : Assurez-vous que vos lèvres soient propres et sèches avant l’application. Appliquez le rouge à lèvres LipojeN au moins 3 fois par jour pendant 30 jours pour obtenir de bons résultats . Les jours où vous ne souhaitez pas vous maquiller, il est possible d’appliquer le Glossy crystal clear numéro 01 pour ne pas interrompre le traitement. N’hésitez pas à renouveler l’application aussi souvent que souhaité pour maintenir l’hydratation et l’apparence pulpeuse de vos lèvres. Nous recommandons d’effectuer un léger gommage des lèvres 1 à 2 fois par semaine. Cela permet d’éliminer les peaux mortes et favorise une meilleure absorption du produit. Une réelle alternative, douce et naturelle, aux injections d’acide hyaluronique !</t>
         </is>
       </c>
-      <c r="J49" t="inlineStr"/>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>HYDROGENATED POLYISOBUTENE, CAPRYLIC/CAPRIC TRIGLYCERIDE, BUTYROSPERMUM PARKII BUTTER, CERA ALBA, AQUA, ETHYLHEXYL METHOXYCINNAMATE, SODIUM HYALURONATE, BHT, TOCOPHERYL ACETATE, PALMITOYL TRIPEPTIDE-1, CAMELLIA JAPONICA SEED OIL, AROMA, ETHYLHEXYL PALMITATE, TRIBEHENIN, SORBITAN ISOSTEARATE, LACTIC ACID, SORBITAN CAPRYLATE, PROPANEDIOL, BENZOIC ACID, ISONONYL ISONONANOATE, ISOPROPYL MYRISTATE, ISOPROPYL TITANIUM TRIISOSTEARATE, STEARALKONIUM HECTORITE, POLYHYDROXYSTEARIC ACID, PROPYLENE CARBONATE, [+/- MAY CONTAIN MICA, CI 77891, CI 77491, CI 77492, CI 15850, CI 75470]</t>
+        </is>
+      </c>
       <c r="K49" t="inlineStr"/>
       <c r="L49" t="inlineStr">
         <is>
@@ -4051,11 +4055,7 @@
           <t>https://biobalance.tn/maquillage/61-customizable-mug.html</t>
         </is>
       </c>
-      <c r="O49" t="inlineStr">
-        <is>
-          <t>ingrédients</t>
-        </is>
-      </c>
+      <c r="O49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -4104,7 +4104,11 @@
           <t>Pour profiter pleinement des bienfaits des repulpeurs lèvres LipojeN, voici quelques conseils d’utilisation bien utiles : Assurez-vous que vos lèvres soient propres et sèches avant l’application. Appliquez le rouge à lèvres LipojeN au moins 3 fois par jour pendant 30 jours pour obtenir de bons résultats . Les jours où vous ne souhaitez pas vous maquiller, il est possible d’appliquer le Glossy crystal clear numéro 01 pour ne pas interrompre le traitement. N’hésitez pas à renouveler l’application aussi souvent que souhaité pour maintenir l’hydratation et l’apparence pulpeuse de vos lèvres. Nous recommandons d’effectuer un léger gommage des lèvres 1 à 2 fois par semaine. Cela permet d’éliminer les peaux mortes et favorise une meilleure absorption du produit. Une réelle alternative, douce et naturelle, aux injections d’acide hyaluronique !</t>
         </is>
       </c>
-      <c r="J50" t="inlineStr"/>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>HYDROGENATED POLYISOBUTENE, CAPRYLIC/CAPRIC TRIGLYCERIDE, BUTYROSPERMUM PARKII BUTTER, CERA ALBA, AQUA, ETHYLHEXYL METHOXYCINNAMATE, SODIUM HYALURONATE, BHT, TOCOPHERYL ACETATE, PALMITOYL TRIPEPTIDE-1, CAMELLIA JAPONICA SEED OIL, AROMA, ETHYLHEXYL PALMITATE, TRIBEHENIN, SORBITAN ISOSTEARATE, LACTIC ACID, SORBITAN CAPRYLATE, PROPANEDIOL, BENZOIC ACID, ISONONYL ISONONANOATE, ISOPROPYL MYRISTATE, ISOPROPYL TITANIUM TRIISOSTEARATE, STEARALKONIUM HECTORITE, POLYHYDROXYSTEARIC ACID, PROPYLENE CARBONATE, [+/- MAY CONTAIN MICA, CI 77891, CI 77491, CI 77492, CI 15850, CI 75470]</t>
+        </is>
+      </c>
       <c r="K50" t="inlineStr"/>
       <c r="L50" t="inlineStr">
         <is>
@@ -4121,11 +4125,7 @@
           <t>https://biobalance.tn/maquillage/62-customizable-mug.html</t>
         </is>
       </c>
-      <c r="O50" t="inlineStr">
-        <is>
-          <t>ingrédients</t>
-        </is>
-      </c>
+      <c r="O50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -4173,7 +4173,11 @@
           <t>Appliquer le sérum deux fois par jour pendant les dix premiers jours, puis une fois par jour pour obtenir les résultats.</t>
         </is>
       </c>
-      <c r="J51" t="inlineStr"/>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>Aqua, Glycerin, Propanediol, Betaine, Zinc Lactate, Niacinamide, Sodium Ascorbyl Phosphate, Xanthan Gum, Nordihydroguaiaretic Acid, Oleanolic Acid, Biotin, PEG-60 Almond Glycerides, Caprylyl Glycol, Carbomer, Sodium Metabisulfite, Centella Asiatica Extract, Butylene Glycol, Polysorbate 20, Hydroxyethylcellulose, Phenoxyethanol, Ethylhexylglycerin, Citric Acid, Sodium Citrate</t>
+        </is>
+      </c>
       <c r="K51" t="inlineStr"/>
       <c r="L51" t="inlineStr">
         <is>
@@ -4187,14 +4191,10 @@
       </c>
       <c r="N51" t="inlineStr">
         <is>
-          <t>https://biobalance.tn/serum/53-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="O51" t="inlineStr">
-        <is>
-          <t>ingrédients</t>
-        </is>
-      </c>
+          <t>https://biobalance.tn/serum/53-customizable-mug.html | https://gemerwholesale.com/en/a/bio-balance-acnevit-serum | https://myoras.com/products/acnevit-anti-acne-serum</t>
+        </is>
+      </c>
+      <c r="O51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -4248,7 +4248,11 @@
           <t>Appliquer sur le visage humide en évitant le contour des yeux, masser puis rincer à l’eau tiède. Utiliser deux fois par jour.</t>
         </is>
       </c>
-      <c r="J52" t="inlineStr"/>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>Aqua, Sodium C14-16 Olefin Sulfonate, Cocamidopropyl Betaine, Decyl Glucoside, PEG-120 Methyl Glucose Dioleate, Tocopherol, C12-15 Alkyl Lactate, Glycerin, Sodium Ascorbyl Phosphate, Centella Asiatica Extract, Vitis Vinifera Seed Extract, Rosmarinus Officinalis Leaf Extract, Propylene Glycol, Niacinamide, Panthenol, Zinc Gluconate, Allantoin, Parfum, Limonene, Disodium EDTA, Hexamidine Diisethionate, Phenoxyethanol, Benzoic Acid, Dehydroacetic Acid, Butylene Glycol</t>
+        </is>
+      </c>
       <c r="K52" t="inlineStr"/>
       <c r="L52" t="inlineStr">
         <is>
@@ -4262,14 +4266,10 @@
       </c>
       <c r="N52" t="inlineStr">
         <is>
-          <t>https://biobalance.tn/nettoyants-visage/63-customizable-mug.html</t>
-        </is>
-      </c>
-      <c r="O52" t="inlineStr">
-        <is>
-          <t>ingrédients</t>
-        </is>
-      </c>
+          <t>https://biobalance.tn/nettoyants-visage/63-customizable-mug.html | https://feel22.com/products/acnevit-anti-acne-cleansing-gel</t>
+        </is>
+      </c>
+      <c r="O52" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>